<commit_message>
Sale Grand Central del viernes: la tarde de Chelsea gana una hora [d9ec91]
Estaba a las 16:20 para que Thais lo viera — pero ella lo tiene en 0, y JP
ya lo hace el lunes 31 a la manana. Eran 40 minutos para alguien que no lo
quiere. Sin esa parada el traslado de las 15:50 tampoco hace falta: se sale
16:25 de Chelsea derecho a la Morgan, y galerias + almuerzo pasan de 1h20 a
casi 2h. Morgan 17:00, SUMMIT 18:10 y Vanguard 22:00 quedan intactos.

Los dias 5 y 6 se revisaron y no se tocaron: todo lo agendado esos dias lo
quieren los dos.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NYC_2026_Planificador.xlsx
+++ b/NYC_2026_Planificador.xlsx
@@ -18315,7 +18315,7 @@
       </c>
       <c r="S169" s="17" t="inlineStr">
         <is>
-          <t>Día 3 · lun 31/8, Día 7 · vie 4/9</t>
+          <t>Día 3 · lun 31/8</t>
         </is>
       </c>
       <c r="T169" s="18" t="inlineStr">
@@ -23035,7 +23035,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I181"/>
+  <dimension ref="A1:I180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26110,7 +26110,7 @@
     <row r="126" ht="32" customHeight="1">
       <c r="A126" s="34" t="inlineStr">
         <is>
-          <t>Salieron el West Village, Washington Square y el Whitney; entraron el High Line, THE VESSEL (al pie del arranque, $10 y 45 min), la Morgan (hoy GRATIS 17-20) y SUMMIT — que se movió AL ATARDECER por el pedido de ustedes: entrada 18:10, luz plena, la puesta ~19:21 multiplicada por los espejos de Kusama (es EL lugar de la ciudad para ese momento) y la noche encendida hasta las 20:15. EL PAGO, dicho honesto: la Morgan se hace en una hora entrando 17:00 en punto, y la cena de hoy es un bocado rápido — por eso el almuerzo en Chelsea Market es EL fuerte del día.</t>
+          <t>Salieron el West Village, Washington Square y el Whitney; entraron el High Line, THE VESSEL (al pie del arranque, $10 y 45 min), la Morgan (hoy GRATIS 17-20) y SUMMIT — que se movió AL ATARDECER por el pedido de ustedes: entrada 18:10, luz plena, la puesta ~19:21 multiplicada por los espejos de Kusama (es EL lugar de la ciudad para ese momento) y la noche encendida hasta las 20:15. EL PAGO, dicho honesto: la Morgan se hace en una hora entrando 17:00 en punto, y la cena de hoy es un bocado rápido — por eso el almuerzo en Chelsea Market es EL fuerte del día. SALIÓ GRAND CENTRAL: estaba a las 16:20 con el argumento de que JP ya lo vio el lunes y Thais no — pero ella lo tiene en 0, así que eran 40 minutos para alguien que no lo quiere. Sin esa parada tampoco hace falta cortar Chelsea a las 15:50: se sale 16:25 derecho a la Morgan y la tarde de galerías y almuerzo gana una hora larga.</t>
         </is>
       </c>
     </row>
@@ -26305,7 +26305,7 @@
       </c>
       <c r="C133" s="37" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="D133" s="38" t="inlineStr">
@@ -26315,7 +26315,7 @@
       </c>
       <c r="E133" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en Chelsea Market — COMER FUERTE: es la comida grande del día, la cena de hoy es un bocado rápido entre el SUMMIT y el Vanguard. Los Tacos No.1 o Very Fresh Noodles.</t>
+          <t>Almuerzo en Chelsea Market — COMER FUERTE: es la comida grande del día, la cena de hoy es un bocado rápido entre el SUMMIT y el Vanguard. Los Tacos No.1 o Very Fresh Noodles. Ahora hay casi DOS HORAS: sin apuro, y si quedaron galerías de Chelsea sin ver, se vuelve.</t>
         </is>
       </c>
       <c r="F133" s="37" t="inlineStr">
@@ -26335,12 +26335,12 @@
       <c r="A134" s="35" t="n"/>
       <c r="B134" s="36" t="inlineStr">
         <is>
-          <t>15:50</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C134" s="37" t="inlineStr">
         <is>
-          <t>16:20</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D134" s="38" t="inlineStr">
@@ -26350,7 +26350,7 @@
       </c>
       <c r="E134" s="39" t="inlineStr">
         <is>
-          <t>A Grand Central SIN desandar: L desde 14 St-8 Av hasta Union Sq y 4/5 exprés hasta Grand Central (~20 min puerta a puerta). Volver caminando a Hudson Yards sería 1,9 km al revés.</t>
+          <t>A la Morgan: L desde 14 St-8 Av hasta Union Sq y 6 hasta 33 St, o A/C/E hasta 34 St-Penn y siete cuadras a pie (~30 min). Salir 16:25 deja margen para entrar 17:00 EN PUNTO.</t>
         </is>
       </c>
       <c r="F134" s="37" t="inlineStr"/>
@@ -26360,124 +26360,116 @@
     </row>
     <row r="135" ht="30" customHeight="1">
       <c r="A135" s="35" t="n"/>
-      <c r="B135" s="36" t="inlineStr">
-        <is>
-          <t>16:20</t>
-        </is>
-      </c>
-      <c r="C135" s="37" t="inlineStr">
+      <c r="B135" s="42" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="D135" s="38" t="inlineStr">
+      <c r="C135" s="43" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D135" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E135" s="39" t="inlineStr">
-        <is>
-          <t>Grand Central PARA THAIS: el techo celeste, la Whispering Gallery y el mercado — JP ya lo vio el lunes, ella no, y está literalmente abajo del SUMMIT.</t>
-        </is>
-      </c>
-      <c r="F135" s="37" t="inlineStr">
-        <is>
-          <t>Grand Central Terminal</t>
+      <c r="E135" s="45" t="inlineStr">
+        <is>
+          <t>★ MORGAN LIBRARY — GRATIS los viernes 17-20h: entrar 17:00 EN PUNTO y hacerla en una hora — la biblioteca son tres salas gloriosas (estanterías de nogal, la Biblia de Gutenberg): alcanza. RESERVA OBLIGATORIA, se libera el viernes 28 de agosto. Está a 8 min a pie de One Vanderbilt.</t>
+        </is>
+      </c>
+      <c r="F135" s="43" t="inlineStr">
+        <is>
+          <t>The Morgan Library &amp; Museum</t>
         </is>
       </c>
       <c r="G135" s="40" t="inlineStr"/>
       <c r="H135" s="41" t="inlineStr"/>
       <c r="I135" s="41" t="inlineStr"/>
     </row>
-    <row r="136" ht="30" customHeight="1">
+    <row r="136" ht="16" customHeight="1">
       <c r="A136" s="35" t="n"/>
-      <c r="B136" s="42" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C136" s="43" t="inlineStr">
+      <c r="B136" s="36" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="D136" s="44" t="inlineStr">
+      <c r="C136" s="37" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="D136" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E136" s="45" t="inlineStr">
-        <is>
-          <t>★ MORGAN LIBRARY — GRATIS los viernes 17-20h: entrar 17:00 EN PUNTO y hacerla en una hora — la biblioteca son tres salas gloriosas (estanterías de nogal, la Biblia de Gutenberg): alcanza. RESERVA OBLIGATORIA, se libera el viernes 28 de agosto. Está a 8 min a pie de One Vanderbilt.</t>
-        </is>
-      </c>
-      <c r="F136" s="43" t="inlineStr">
-        <is>
-          <t>The Morgan Library &amp; Museum</t>
-        </is>
-      </c>
-      <c r="G136" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~9 min a pie · 0.7 km · estimado</t>
-        </is>
-      </c>
+      <c r="E136" s="39" t="inlineStr">
+        <is>
+          <t>Caminar las seis cuadras de la Morgan a One Vanderbilt (~8-10 min).</t>
+        </is>
+      </c>
+      <c r="F136" s="37" t="inlineStr"/>
+      <c r="G136" s="40" t="inlineStr"/>
       <c r="H136" s="41" t="inlineStr"/>
       <c r="I136" s="41" t="inlineStr"/>
     </row>
-    <row r="137" ht="16" customHeight="1">
+    <row r="137" ht="30" customHeight="1">
       <c r="A137" s="35" t="n"/>
-      <c r="B137" s="36" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="C137" s="37" t="inlineStr">
+      <c r="B137" s="42" t="inlineStr">
         <is>
           <t>18:10</t>
         </is>
       </c>
-      <c r="D137" s="38" t="inlineStr">
+      <c r="C137" s="43" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="D137" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E137" s="39" t="inlineStr">
-        <is>
-          <t>Caminar de vuelta las seis cuadras a One Vanderbilt (~8-10 min).</t>
-        </is>
-      </c>
-      <c r="F137" s="37" t="inlineStr"/>
+      <c r="E137" s="45" t="inlineStr">
+        <is>
+          <t>★★ SUMMIT ONE VANDERBILT — EL ARCO COMPLETO: entrada 18:10 con luz, el atardecer ~19:21 multiplicado por los espejos infinitos de Kusama, y la noche encendida hasta ~20:15. Ticket ATARDECER $57-63 — es la franja que primero se agota: reservar YA. NO está en ningún pase.</t>
+        </is>
+      </c>
+      <c r="F137" s="43" t="inlineStr">
+        <is>
+          <t>SUMMIT One Vanderbilt</t>
+        </is>
+      </c>
       <c r="G137" s="40" t="inlineStr"/>
       <c r="H137" s="41" t="inlineStr"/>
       <c r="I137" s="41" t="inlineStr"/>
     </row>
     <row r="138" ht="30" customHeight="1">
       <c r="A138" s="35" t="n"/>
-      <c r="B138" s="42" t="inlineStr">
-        <is>
-          <t>18:10</t>
-        </is>
-      </c>
-      <c r="C138" s="43" t="inlineStr">
+      <c r="B138" s="36" t="inlineStr">
         <is>
           <t>20:20</t>
         </is>
       </c>
-      <c r="D138" s="44" t="inlineStr">
+      <c r="C138" s="37" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="D138" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E138" s="45" t="inlineStr">
-        <is>
-          <t>★★ SUMMIT ONE VANDERBILT — EL ARCO COMPLETO: entrada 18:10 con luz, el atardecer ~19:21 multiplicado por los espejos infinitos de Kusama, y la noche encendida hasta ~20:15. Ticket ATARDECER $57-63 — es la franja que primero se agota: reservar YA. NO está en ningún pase.</t>
-        </is>
-      </c>
-      <c r="F138" s="43" t="inlineStr">
-        <is>
-          <t>SUMMIT One Vanderbilt</t>
-        </is>
-      </c>
+      <c r="E138" s="39" t="inlineStr">
+        <is>
+          <t>Bajar AL VILLAGE PRIMERO y cenar allá: 4/5/6 o 7 hasta 14 St-Union Sq y 1 hasta Christopher St (~25 min). Cenar cerca de Grand Central y bajar después llega justo; hacerlo al revés deja margen.</t>
+        </is>
+      </c>
+      <c r="F138" s="37" t="inlineStr"/>
       <c r="G138" s="40" t="inlineStr"/>
       <c r="H138" s="41" t="inlineStr"/>
       <c r="I138" s="41" t="inlineStr"/>
@@ -26486,12 +26478,12 @@
       <c r="A139" s="35" t="n"/>
       <c r="B139" s="36" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C139" s="37" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D139" s="38" t="inlineStr">
@@ -26501,7 +26493,7 @@
       </c>
       <c r="E139" s="39" t="inlineStr">
         <is>
-          <t>Bajar AL VILLAGE PRIMERO y cenar allá: 4/5/6 o 7 hasta 14 St-Union Sq y 1 hasta Christopher St (~25 min). Cenar cerca de Grand Central y bajar después llega justo; hacerlo al revés deja margen.</t>
+          <t>Cena en el West Village, a cinco minutos del club. El Vanguard NO sirve NADA de comida (lo dicen así: 'ni un maní') y no se permite entrar comida: lo que no cenen ahora, no se cena. 40 minutos alcanzan.</t>
         </is>
       </c>
       <c r="F139" s="37" t="inlineStr"/>
@@ -26513,12 +26505,12 @@
       <c r="A140" s="35" t="n"/>
       <c r="B140" s="36" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C140" s="37" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D140" s="38" t="inlineStr">
@@ -26528,7 +26520,7 @@
       </c>
       <c r="E140" s="39" t="inlineStr">
         <is>
-          <t>Cena en el West Village, a cinco minutos del club. El Vanguard NO sirve NADA de comida (lo dicen así: 'ni un maní') y no se permite entrar comida: lo que no cenen ahora, no se cena. 40 minutos alcanzan.</t>
+          <t>EN LA PUERTA DEL VANGUARD a las 21:30 EN PUNTO: el acomodo del segundo set arranca a esa hora y los asientos son POR ORDEN DE LLEGADA — la entrada es General Admission, no numerada. Con 123 asientos, los diez minutos de diferencia son estar frente al piano o contra la columna. El ticket lo dice: el acomodo tardío, con entrada o sin ella, queda a criterio del encargado.</t>
         </is>
       </c>
       <c r="F140" s="37" t="inlineStr"/>
@@ -26538,199 +26530,199 @@
     </row>
     <row r="141" ht="30" customHeight="1">
       <c r="A141" s="35" t="n"/>
-      <c r="B141" s="36" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C141" s="37" t="inlineStr">
+      <c r="B141" s="42" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D141" s="38" t="inlineStr">
+      <c r="C141" s="43" t="inlineStr"/>
+      <c r="D141" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E141" s="39" t="inlineStr">
-        <is>
-          <t>EN LA PUERTA DEL VANGUARD a las 21:30 EN PUNTO: el acomodo del segundo set arranca a esa hora y los asientos son POR ORDEN DE LLEGADA — la entrada es General Admission, no numerada. Con 123 asientos, los diez minutos de diferencia son estar frente al piano o contra la columna. El ticket lo dice: el acomodo tardío, con entrada o sin ella, queda a criterio del encargado.</t>
-        </is>
-      </c>
-      <c r="F141" s="37" t="inlineStr"/>
+      <c r="E141" s="45" t="inlineStr">
+        <is>
+          <t>★★ VILLAGE VANGUARD — JOHN PATITUCCI TRIO con Chris Potter y Brian Blade, SET DE LAS 22:00. Movido acá desde el martes para que vayan LOS DOS (pedido de Juan). El sótano triangular de 1935, 123 asientos, la acústica que grabó a Coltrane. ✔ ENTRADAS COMPRADAS el 26/8: 2 × General Admission $45 (#18741454 y #18741456), a nombre de Juan Pablo Garicoïts. Falta solo el mínimo de UNA CONSUMICIÓN por cabeza en la mesa (vale gaseosa, jugo o agua) — se paga ahí, aceptan tarjeta.</t>
+        </is>
+      </c>
+      <c r="F141" s="43" t="inlineStr">
+        <is>
+          <t>Village Vanguard</t>
+        </is>
+      </c>
       <c r="G141" s="40" t="inlineStr"/>
       <c r="H141" s="41" t="inlineStr"/>
       <c r="I141" s="41" t="inlineStr"/>
     </row>
-    <row r="142" ht="30" customHeight="1">
-      <c r="A142" s="35" t="n"/>
-      <c r="B142" s="42" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C142" s="43" t="inlineStr"/>
-      <c r="D142" s="44" t="inlineStr">
+    <row r="142" ht="32" customHeight="1">
+      <c r="A142" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  EL CANJE DE ESTA NOCHE: para meter el Vanguard con Thais, SALIÓ BILL'S PLACE. No hay otra noche donde entre (Bill Saxton toca solo viernes y sábado, y el sábado está tomado por Peter Luger + el play + el Café Wha). Con las entradas ya compradas y sin cambios ni transferencias, el canje quedó CERRADO: Bill's Place sale del viaje. // El Whitney es gratis hoy de 17 a 22h, pero choca con la Morgan y ustedes lo bajaron a 'quizás' mientras que la Morgan quedó en 2. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y el Whitney ahora cierra los martes. SI ALGO SALIERA MAL con el acomodo (llegar tarde y que no haya lugar): Mezzrow o Smalls quedan a cuatro cuadras ($25 con bebida, Smalls tiene jam de madrugada los viernes desde la 1:00), o el Blue Note — el 4 y 5 de septiembre toca Chief Adjuah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 8 · Sábado 05/09 · Brooklyn, Peter Luger, un PLAY y Café Wha hasta la madrugada  —  base: The Beacon  ·  Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="32" customHeight="1">
+      <c r="A145" s="34" t="inlineStr">
+        <is>
+          <t>La gran noche del viaje, rearmada a pedido: el musical SALIÓ y entraron un PLAY de Broadway a las 19:30 y el CAFÉ WHA a las 23:45 — el sótano del Village donde debutaron Dylan y Hendrix, con reserva gratis ya pedida por Eventbrite. La cena temprana en Peter Luger (17:00) ahora existe exactamente para esto: porterhouse → telón → medianoche de soul y funk. Frankel's sigue afuera (a un porterhouse no se llega con un pastrami encima) y Westlight sigue opcional. ⚠️ La noche termina ~1:15-1:30: el domingo no tiene NADA fijo hasta las 16:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="30" customHeight="1">
+      <c r="A146" s="35" t="n"/>
+      <c r="B146" s="36" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="C146" s="37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D146" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E142" s="45" t="inlineStr">
-        <is>
-          <t>★★ VILLAGE VANGUARD — JOHN PATITUCCI TRIO con Chris Potter y Brian Blade, SET DE LAS 22:00. Movido acá desde el martes para que vayan LOS DOS (pedido de Juan). El sótano triangular de 1935, 123 asientos, la acústica que grabó a Coltrane. ✔ ENTRADAS COMPRADAS el 26/8: 2 × General Admission $45 (#18741454 y #18741456), a nombre de Juan Pablo Garicoïts. Falta solo el mínimo de UNA CONSUMICIÓN por cabeza en la mesa (vale gaseosa, jugo o agua) — se paga ahí, aceptan tarjeta.</t>
-        </is>
-      </c>
-      <c r="F142" s="43" t="inlineStr">
-        <is>
-          <t>Village Vanguard</t>
-        </is>
-      </c>
-      <c r="G142" s="40" t="inlineStr"/>
-      <c r="H142" s="41" t="inlineStr"/>
-      <c r="I142" s="41" t="inlineStr"/>
-    </row>
-    <row r="143" ht="32" customHeight="1">
-      <c r="A143" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  EL CANJE DE ESTA NOCHE: para meter el Vanguard con Thais, SALIÓ BILL'S PLACE. No hay otra noche donde entre (Bill Saxton toca solo viernes y sábado, y el sábado está tomado por Peter Luger + el play + el Café Wha). Con las entradas ya compradas y sin cambios ni transferencias, el canje quedó CERRADO: Bill's Place sale del viaje. // El Whitney es gratis hoy de 17 a 22h, pero choca con la Morgan y ustedes lo bajaron a 'quizás' mientras que la Morgan quedó en 2. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y el Whitney ahora cierra los martes. SI ALGO SALIERA MAL con el acomodo (llegar tarde y que no haya lugar): Mezzrow o Smalls quedan a cuatro cuadras ($25 con bebida, Smalls tiene jam de madrugada los viernes desde la 1:00), o el Blue Note — el 4 y 5 de septiembre toca Chief Adjuah.</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="22" customHeight="1">
-      <c r="A145" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 8 · Sábado 05/09 · Brooklyn, Peter Luger, un PLAY y Café Wha hasta la madrugada  —  base: The Beacon  ·  Ambos</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="32" customHeight="1">
-      <c r="A146" s="34" t="inlineStr">
-        <is>
-          <t>La gran noche del viaje, rearmada a pedido: el musical SALIÓ y entraron un PLAY de Broadway a las 19:30 y el CAFÉ WHA a las 23:45 — el sótano del Village donde debutaron Dylan y Hendrix, con reserva gratis ya pedida por Eventbrite. La cena temprana en Peter Luger (17:00) ahora existe exactamente para esto: porterhouse → telón → medianoche de soul y funk. Frankel's sigue afuera (a un porterhouse no se llega con un pastrami encima) y Westlight sigue opcional. ⚠️ La noche termina ~1:15-1:30: el domingo no tiene NADA fijo hasta las 16:00.</t>
-        </is>
-      </c>
+      <c r="E146" s="39" t="inlineStr">
+        <is>
+          <t>Salir 8:15: 1/2/3 desde 72 St + transbordo a A/C hasta High St son ~40-45 min REALES. Llegar temprano a DUMBO es la diferencia entre la foto y la cola de fotos.</t>
+        </is>
+      </c>
+      <c r="F146" s="37" t="inlineStr"/>
+      <c r="G146" s="40" t="inlineStr"/>
+      <c r="H146" s="41" t="inlineStr"/>
+      <c r="I146" s="41" t="inlineStr"/>
     </row>
     <row r="147" ht="30" customHeight="1">
       <c r="A147" s="35" t="n"/>
-      <c r="B147" s="36" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="C147" s="37" t="inlineStr">
+      <c r="B147" s="42" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D147" s="38" t="inlineStr">
+      <c r="C147" s="43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D147" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E147" s="39" t="inlineStr">
-        <is>
-          <t>Salir 8:15: 1/2/3 desde 72 St + transbordo a A/C hasta High St son ~40-45 min REALES. Llegar temprano a DUMBO es la diferencia entre la foto y la cola de fotos.</t>
-        </is>
-      </c>
-      <c r="F147" s="37" t="inlineStr"/>
+      <c r="E147" s="45" t="inlineStr">
+        <is>
+          <t>★ Brooklyn Bridge Park y DUMBO — muelles reconvertidos con el skyline de Lower Manhattan de frente, y la foto del Manhattan Bridge encuadrado en Washington y Water.</t>
+        </is>
+      </c>
+      <c r="F147" s="43" t="inlineStr">
+        <is>
+          <t>Brooklyn Bridge Park</t>
+        </is>
+      </c>
       <c r="G147" s="40" t="inlineStr"/>
       <c r="H147" s="41" t="inlineStr"/>
       <c r="I147" s="41" t="inlineStr"/>
     </row>
-    <row r="148" ht="30" customHeight="1">
+    <row r="148" ht="16" customHeight="1">
       <c r="A148" s="35" t="n"/>
-      <c r="B148" s="42" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C148" s="43" t="inlineStr">
+      <c r="B148" s="36" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="D148" s="44" t="inlineStr">
+      <c r="C148" s="37" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D148" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E148" s="45" t="inlineStr">
-        <is>
-          <t>★ Brooklyn Bridge Park y DUMBO — muelles reconvertidos con el skyline de Lower Manhattan de frente, y la foto del Manhattan Bridge encuadrado en Washington y Water.</t>
-        </is>
-      </c>
-      <c r="F148" s="43" t="inlineStr">
-        <is>
-          <t>Brooklyn Bridge Park</t>
-        </is>
-      </c>
-      <c r="G148" s="40" t="inlineStr"/>
+      <c r="E148" s="39" t="inlineStr">
+        <is>
+          <t>Brooklyn Heights Promenade — la postal clásica del skyline sobre el BQE.</t>
+        </is>
+      </c>
+      <c r="F148" s="37" t="inlineStr">
+        <is>
+          <t>Brooklyn Heights Promenade</t>
+        </is>
+      </c>
+      <c r="G148" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~8 min a pie · 0.6 km · estimado</t>
+        </is>
+      </c>
       <c r="H148" s="41" t="inlineStr"/>
       <c r="I148" s="41" t="inlineStr"/>
     </row>
-    <row r="149" ht="16" customHeight="1">
+    <row r="149" ht="30" customHeight="1">
       <c r="A149" s="35" t="n"/>
-      <c r="B149" s="36" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="C149" s="37" t="inlineStr">
+      <c r="B149" s="42" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="D149" s="38" t="inlineStr">
+      <c r="C149" s="43" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D149" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E149" s="39" t="inlineStr">
-        <is>
-          <t>Brooklyn Heights Promenade — la postal clásica del skyline sobre el BQE.</t>
-        </is>
-      </c>
-      <c r="F149" s="37" t="inlineStr">
-        <is>
-          <t>Brooklyn Heights Promenade</t>
-        </is>
-      </c>
-      <c r="G149" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~8 min a pie · 0.6 km · estimado</t>
-        </is>
-      </c>
+      <c r="E149" s="45" t="inlineStr">
+        <is>
+          <t>★ NEW YORK TRANSIT MUSEUM — una estación de subte clausurada de 1936 con 20 vagones históricos en las vías originales; se puede subir a todos. $10. Cierra lunes y martes, así que hoy es el día.</t>
+        </is>
+      </c>
+      <c r="F149" s="43" t="inlineStr">
+        <is>
+          <t>New York Transit Museum</t>
+        </is>
+      </c>
+      <c r="G149" s="40" t="inlineStr"/>
       <c r="H149" s="41" t="inlineStr"/>
       <c r="I149" s="41" t="inlineStr"/>
     </row>
-    <row r="150" ht="30" customHeight="1">
+    <row r="150" ht="16" customHeight="1">
       <c r="A150" s="35" t="n"/>
-      <c r="B150" s="42" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="C150" s="43" t="inlineStr">
+      <c r="B150" s="36" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="D150" s="44" t="inlineStr">
+      <c r="C150" s="37" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D150" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E150" s="45" t="inlineStr">
-        <is>
-          <t>★ NEW YORK TRANSIT MUSEUM — una estación de subte clausurada de 1936 con 20 vagones históricos en las vías originales; se puede subir a todos. $10. Cierra lunes y martes, así que hoy es el día.</t>
-        </is>
-      </c>
-      <c r="F150" s="43" t="inlineStr">
-        <is>
-          <t>New York Transit Museum</t>
-        </is>
-      </c>
+      <c r="E150" s="39" t="inlineStr">
+        <is>
+          <t>Almuerzo en Downtown Brooklyn.</t>
+        </is>
+      </c>
+      <c r="F150" s="37" t="inlineStr"/>
       <c r="G150" s="40" t="inlineStr"/>
       <c r="H150" s="41" t="inlineStr"/>
       <c r="I150" s="41" t="inlineStr"/>
@@ -26739,12 +26731,12 @@
       <c r="A151" s="35" t="n"/>
       <c r="B151" s="36" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C151" s="37" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="D151" s="38" t="inlineStr">
@@ -26754,7 +26746,7 @@
       </c>
       <c r="E151" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en Downtown Brooklyn.</t>
+          <t>Subte a Williamsburg.</t>
         </is>
       </c>
       <c r="F151" s="37" t="inlineStr"/>
@@ -26762,74 +26754,74 @@
       <c r="H151" s="41" t="inlineStr"/>
       <c r="I151" s="41" t="inlineStr"/>
     </row>
-    <row r="152" ht="16" customHeight="1">
+    <row r="152" ht="30" customHeight="1">
       <c r="A152" s="35" t="n"/>
-      <c r="B152" s="36" t="inlineStr">
-        <is>
-          <t>13:45</t>
-        </is>
-      </c>
-      <c r="C152" s="37" t="inlineStr">
+      <c r="B152" s="42" t="inlineStr">
         <is>
           <t>14:15</t>
         </is>
       </c>
-      <c r="D152" s="38" t="inlineStr">
+      <c r="C152" s="43" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D152" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E152" s="39" t="inlineStr">
-        <is>
-          <t>Subte a Williamsburg.</t>
-        </is>
-      </c>
-      <c r="F152" s="37" t="inlineStr"/>
+      <c r="E152" s="45" t="inlineStr">
+        <is>
+          <t>★ Domino Park — ex refinería de azúcar; el paseo elevado pasa entre la maquinaria industrial conservada, con el Williamsburg Bridge y Midtown enfrente.</t>
+        </is>
+      </c>
+      <c r="F152" s="43" t="inlineStr">
+        <is>
+          <t>Domino Park</t>
+        </is>
+      </c>
       <c r="G152" s="40" t="inlineStr"/>
       <c r="H152" s="41" t="inlineStr"/>
       <c r="I152" s="41" t="inlineStr"/>
     </row>
     <row r="153" ht="30" customHeight="1">
       <c r="A153" s="35" t="n"/>
-      <c r="B153" s="42" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="C153" s="43" t="inlineStr">
+      <c r="B153" s="36" t="inlineStr">
         <is>
           <t>15:15</t>
         </is>
       </c>
-      <c r="D153" s="44" t="inlineStr">
+      <c r="C153" s="37" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D153" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E153" s="45" t="inlineStr">
-        <is>
-          <t>★ Domino Park — ex refinería de azúcar; el paseo elevado pasa entre la maquinaria industrial conservada, con el Williamsburg Bridge y Midtown enfrente.</t>
-        </is>
-      </c>
-      <c r="F153" s="43" t="inlineStr">
-        <is>
-          <t>Domino Park</t>
-        </is>
-      </c>
+      <c r="E153" s="39" t="inlineStr">
+        <is>
+          <t>Paseo por Williamsburg: Bedford Ave, disquerías y vintage. OPCIONAL si quieren la panorámica: Westlight (piso 22, sin cover, un trago) — lo bajaron a 'quizás', así que es prescindible. NO comer nada: lo que viene lo merece.</t>
+        </is>
+      </c>
+      <c r="F153" s="37" t="inlineStr"/>
       <c r="G153" s="40" t="inlineStr"/>
       <c r="H153" s="41" t="inlineStr"/>
       <c r="I153" s="41" t="inlineStr"/>
     </row>
-    <row r="154" ht="30" customHeight="1">
+    <row r="154" ht="16" customHeight="1">
       <c r="A154" s="35" t="n"/>
       <c r="B154" s="36" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C154" s="37" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D154" s="38" t="inlineStr">
@@ -26839,7 +26831,7 @@
       </c>
       <c r="E154" s="39" t="inlineStr">
         <is>
-          <t>Paseo por Williamsburg: Bedford Ave, disquerías y vintage. OPCIONAL si quieren la panorámica: Westlight (piso 22, sin cover, un trago) — lo bajaron a 'quizás', así que es prescindible. NO comer nada: lo que viene lo merece.</t>
+          <t>Caminar por Bedford/Driggs hasta el pie del Williamsburg Bridge (~15 min).</t>
         </is>
       </c>
       <c r="F154" s="37" t="inlineStr"/>
@@ -26847,132 +26839,132 @@
       <c r="H154" s="41" t="inlineStr"/>
       <c r="I154" s="41" t="inlineStr"/>
     </row>
-    <row r="155" ht="16" customHeight="1">
+    <row r="155" ht="30" customHeight="1">
       <c r="A155" s="35" t="n"/>
-      <c r="B155" s="36" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="C155" s="37" t="inlineStr">
+      <c r="B155" s="42" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="D155" s="38" t="inlineStr">
+      <c r="C155" s="43" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D155" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E155" s="39" t="inlineStr">
-        <is>
-          <t>Caminar por Bedford/Driggs hasta el pie del Williamsburg Bridge (~15 min).</t>
-        </is>
-      </c>
-      <c r="F155" s="37" t="inlineStr"/>
+      <c r="E155" s="45" t="inlineStr">
+        <is>
+          <t>★★ PETER LUGER (178 Broadway) — el porterhouse for two de 1887, dry-aged en el sótano, con la tocineta gruesa de entrada. ~$160-200 los dos con sides y propina. ⚠️ SIN TARJETAS DE CRÉDITO: efectivo, débito US o cheque — llevar cash. Cena temprana a propósito: el teatro espera. RESERVA EN RESY YA.</t>
+        </is>
+      </c>
+      <c r="F155" s="43" t="inlineStr">
+        <is>
+          <t>Peter Luger Steak House</t>
+        </is>
+      </c>
       <c r="G155" s="40" t="inlineStr"/>
       <c r="H155" s="41" t="inlineStr"/>
       <c r="I155" s="41" t="inlineStr"/>
     </row>
     <row r="156" ht="30" customHeight="1">
       <c r="A156" s="35" t="n"/>
-      <c r="B156" s="42" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C156" s="43" t="inlineStr">
+      <c r="B156" s="36" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="D156" s="44" t="inlineStr">
+      <c r="C156" s="37" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D156" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E156" s="45" t="inlineStr">
-        <is>
-          <t>★★ PETER LUGER (178 Broadway) — el porterhouse for two de 1887, dry-aged en el sótano, con la tocineta gruesa de entrada. ~$160-200 los dos con sides y propina. ⚠️ SIN TARJETAS DE CRÉDITO: efectivo, débito US o cheque — llevar cash. Cena temprana a propósito: el teatro espera. RESERVA EN RESY YA.</t>
-        </is>
-      </c>
-      <c r="F156" s="43" t="inlineStr">
-        <is>
-          <t>Peter Luger Steak House</t>
-        </is>
-      </c>
+      <c r="E156" s="39" t="inlineStr">
+        <is>
+          <t>A la zona de teatros: subte J desde Marcy Av hasta Essex St y F hasta 42 St-Bryant Park (~35 min con transbordo), o directamente Uber al teatro (~20-25 min, $25-35 — un sábado a la noche el puente puede estar cargado).</t>
+        </is>
+      </c>
+      <c r="F156" s="37" t="inlineStr"/>
       <c r="G156" s="40" t="inlineStr"/>
       <c r="H156" s="41" t="inlineStr"/>
       <c r="I156" s="41" t="inlineStr"/>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="35" t="n"/>
-      <c r="B157" s="36" t="inlineStr">
-        <is>
-          <t>18:45</t>
-        </is>
-      </c>
-      <c r="C157" s="37" t="inlineStr">
+      <c r="B157" s="42" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="D157" s="38" t="inlineStr">
+      <c r="C157" s="43" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="D157" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E157" s="39" t="inlineStr">
-        <is>
-          <t>A la zona de teatros: subte J desde Marcy Av hasta Essex St y F hasta 42 St-Bryant Park (~35 min con transbordo), o directamente Uber al teatro (~20-25 min, $25-35 — un sábado a la noche el puente puede estar cargado).</t>
-        </is>
-      </c>
-      <c r="F157" s="37" t="inlineStr"/>
+      <c r="E157" s="45" t="inlineStr">
+        <is>
+          <t>★★ PLAY DE BROADWAY — mi recomendación: STRANGER THINGS: THE FIRST SHADOW (Marquis, desde ~$76): la maquinaria escénica que ganó el Tony — para quien viene de Mercer Labs, el mismo músculo llevado al teatro. Alternativas esa semana: Harry Potter and the Cursed Child, Paranormal Activity, The Imaginary Invalid. COMPRA FIRME esta semana y verificar el horario real de la función (19:00/19:30/20:00): tiene que terminar ~22:00 para lo que sigue.</t>
+        </is>
+      </c>
+      <c r="F157" s="43" t="inlineStr">
+        <is>
+          <t>Stranger Things: The First Shadow (play)</t>
+        </is>
+      </c>
       <c r="G157" s="40" t="inlineStr"/>
       <c r="H157" s="41" t="inlineStr"/>
       <c r="I157" s="41" t="inlineStr"/>
     </row>
-    <row r="158" ht="30" customHeight="1">
+    <row r="158" ht="16" customHeight="1">
       <c r="A158" s="35" t="n"/>
-      <c r="B158" s="42" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="C158" s="43" t="inlineStr">
+      <c r="B158" s="36" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D158" s="44" t="inlineStr">
+      <c r="C158" s="37" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="D158" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E158" s="45" t="inlineStr">
-        <is>
-          <t>★★ PLAY DE BROADWAY — mi recomendación: STRANGER THINGS: THE FIRST SHADOW (Marquis, desde ~$76): la maquinaria escénica que ganó el Tony — para quien viene de Mercer Labs, el mismo músculo llevado al teatro. Alternativas esa semana: Harry Potter and the Cursed Child, Paranormal Activity, The Imaginary Invalid. COMPRA FIRME esta semana y verificar el horario real de la función (19:00/19:30/20:00): tiene que terminar ~22:00 para lo que sigue.</t>
-        </is>
-      </c>
-      <c r="F158" s="43" t="inlineStr">
-        <is>
-          <t>Stranger Things: The First Shadow (play)</t>
-        </is>
-      </c>
+      <c r="E158" s="39" t="inlineStr">
+        <is>
+          <t>Subte 1 desde Times Sq hasta Christopher St (~15 min) y caminar al corazón del Village.</t>
+        </is>
+      </c>
+      <c r="F158" s="37" t="inlineStr"/>
       <c r="G158" s="40" t="inlineStr"/>
       <c r="H158" s="41" t="inlineStr"/>
       <c r="I158" s="41" t="inlineStr"/>
     </row>
-    <row r="159" ht="16" customHeight="1">
+    <row r="159" ht="30" customHeight="1">
       <c r="A159" s="35" t="n"/>
       <c r="B159" s="36" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="C159" s="37" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D159" s="38" t="inlineStr">
@@ -26982,7 +26974,7 @@
       </c>
       <c r="E159" s="39" t="inlineStr">
         <is>
-          <t>Subte 1 desde Times Sq hasta Christopher St (~15 min) y caminar al corazón del Village.</t>
+          <t>Paseo sin apuro por Bleecker y MacDougal — la esquina folk de los 60s de noche, un café o un trago corto. El único objetivo real: estar en la puerta del Wha a las 23:10.</t>
         </is>
       </c>
       <c r="F159" s="37" t="inlineStr"/>
@@ -26992,102 +26984,106 @@
     </row>
     <row r="160" ht="30" customHeight="1">
       <c r="A160" s="35" t="n"/>
-      <c r="B160" s="36" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="C160" s="37" t="inlineStr">
+      <c r="B160" s="42" t="inlineStr">
         <is>
           <t>23:15</t>
         </is>
       </c>
-      <c r="D160" s="38" t="inlineStr">
+      <c r="C160" s="43" t="inlineStr"/>
+      <c r="D160" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E160" s="39" t="inlineStr">
-        <is>
-          <t>Paseo sin apuro por Bleecker y MacDougal — la esquina folk de los 60s de noche, un café o un trago corto. El único objetivo real: estar en la puerta del Wha a las 23:10.</t>
-        </is>
-      </c>
-      <c r="F160" s="37" t="inlineStr"/>
+      <c r="E160" s="45" t="inlineStr">
+        <is>
+          <t>★★ CAFÉ WHA — LLEGAR 23:10-23:15: la reserva de Eventbrite NO garantiza admisión y a las 23:30 EN PUNTO liberan los asientos vacíos al standby. TODOS los de la reserva presentes. Set 2 de la house band 23:45-~1:15: soul y funk a máquina en el sótano donde debutaron Dylan, Hendrix y Springsteen. $20 por cabeza van a la cuenta + consumo. Vuelta: subte 1 Christopher St → 72 St (~25 min) o taxi.</t>
+        </is>
+      </c>
+      <c r="F160" s="43" t="inlineStr">
+        <is>
+          <t>Cafe Wha?</t>
+        </is>
+      </c>
       <c r="G160" s="40" t="inlineStr"/>
       <c r="H160" s="41" t="inlineStr"/>
       <c r="I160" s="41" t="inlineStr"/>
     </row>
-    <row r="161" ht="30" customHeight="1">
-      <c r="A161" s="35" t="n"/>
-      <c r="B161" s="42" t="inlineStr">
-        <is>
-          <t>23:15</t>
-        </is>
-      </c>
-      <c r="C161" s="43" t="inlineStr"/>
-      <c r="D161" s="44" t="inlineStr">
+    <row r="161" ht="32" customHeight="1">
+      <c r="A161" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  SOBRE PETER LUGER: la mesa de las 17:00 es la realista — y ahora es la única que funciona: el play manda. PLAN B si no hay mesa: correr Peter Luger al ALMUERZO del mismo día (12:45). // SI EL CANSANCIO GANA A LAS 22:00: el Café Wha es la pieza sacrificable — la reserva es gratis y no penaliza no ir; el play, pagado, no. // Sigue afuera: Bar LunÀtico y Barbès (Bed-Stuy/Park Slope), sin noche posible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="22" customHeight="1">
+      <c r="A163" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 9 · Domingo 06/09 · Checkout, Central Park, Roosevelt Island y vuelo  —  base: The Beacon (checkout) → EWR  ·  Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="32" customHeight="1">
+      <c r="A164" s="34" t="inlineStr">
+        <is>
+          <t>El día arranca con el CHECKOUT de The Beacon: hacerlo temprano y dejar las valijas en el bell desk libera el día entero. El vuelo sale 23:40, así que hay margen — pero es el domingo del fin de semana largo de Labor Day, la noche de mayor tráfico del año, y EWR va a estar cargado. Por eso todo queda dentro del eje Central Park - Upper East Side, a diez minutos de subte del hotel, y se sale con 2h45 de anticipación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="30" customHeight="1">
+      <c r="A165" s="35" t="n"/>
+      <c r="B165" s="36" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C165" s="37" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D165" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E161" s="45" t="inlineStr">
-        <is>
-          <t>★★ CAFÉ WHA — LLEGAR 23:10-23:15: la reserva de Eventbrite NO garantiza admisión y a las 23:30 EN PUNTO liberan los asientos vacíos al standby. TODOS los de la reserva presentes. Set 2 de la house band 23:45-~1:15: soul y funk a máquina en el sótano donde debutaron Dylan, Hendrix y Springsteen. $20 por cabeza van a la cuenta + consumo. Vuelta: subte 1 Christopher St → 72 St (~25 min) o taxi.</t>
-        </is>
-      </c>
-      <c r="F161" s="43" t="inlineStr">
-        <is>
-          <t>Cafe Wha?</t>
-        </is>
-      </c>
-      <c r="G161" s="40" t="inlineStr"/>
-      <c r="H161" s="41" t="inlineStr"/>
-      <c r="I161" s="41" t="inlineStr"/>
-    </row>
-    <row r="162" ht="32" customHeight="1">
-      <c r="A162" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  SOBRE PETER LUGER: la mesa de las 17:00 es la realista — y ahora es la única que funciona: el play manda. PLAN B si no hay mesa: correr Peter Luger al ALMUERZO del mismo día (12:45). // SI EL CANSANCIO GANA A LAS 22:00: el Café Wha es la pieza sacrificable — la reserva es gratis y no penaliza no ir; el play, pagado, no. // Sigue afuera: Bar LunÀtico y Barbès (Bed-Stuy/Park Slope), sin noche posible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="164" ht="22" customHeight="1">
-      <c r="A164" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 9 · Domingo 06/09 · Checkout, Central Park, Roosevelt Island y vuelo  —  base: The Beacon (checkout) → EWR  ·  Ambos</t>
-        </is>
-      </c>
-    </row>
-    <row r="165" ht="32" customHeight="1">
-      <c r="A165" s="34" t="inlineStr">
-        <is>
-          <t>El día arranca con el CHECKOUT de The Beacon: hacerlo temprano y dejar las valijas en el bell desk libera el día entero. El vuelo sale 23:40, así que hay margen — pero es el domingo del fin de semana largo de Labor Day, la noche de mayor tráfico del año, y EWR va a estar cargado. Por eso todo queda dentro del eje Central Park - Upper East Side, a diez minutos de subte del hotel, y se sale con 2h45 de anticipación.</t>
-        </is>
-      </c>
+      <c r="E165" s="39" t="inlineStr">
+        <is>
+          <t>Desayuno SIN despertador temprano: anoche terminó ~1:30 en el Village y lo único con hora fija hoy es el Guggenheim a las 16:00. Dormir un poco más está permitido.</t>
+        </is>
+      </c>
+      <c r="F165" s="37" t="inlineStr"/>
+      <c r="G165" s="40" t="inlineStr"/>
+      <c r="H165" s="41" t="inlineStr"/>
+      <c r="I165" s="41" t="inlineStr"/>
     </row>
     <row r="166" ht="30" customHeight="1">
       <c r="A166" s="35" t="n"/>
-      <c r="B166" s="36" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C166" s="37" t="inlineStr">
+      <c r="B166" s="42" t="inlineStr">
         <is>
           <t>09:45</t>
         </is>
       </c>
-      <c r="D166" s="38" t="inlineStr">
+      <c r="C166" s="43" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D166" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E166" s="39" t="inlineStr">
-        <is>
-          <t>Desayuno SIN despertador temprano: anoche terminó ~1:30 en el Village y lo único con hora fija hoy es el Guggenheim a las 16:00. Dormir un poco más está permitido.</t>
-        </is>
-      </c>
-      <c r="F166" s="37" t="inlineStr"/>
+      <c r="E166" s="45" t="inlineStr">
+        <is>
+          <t>★ CHECKOUT de The Beacon y dejar las valijas en el bell desk. El checkout formal suele ser 11:00-12:00, pero hacerlo antes libera el día.</t>
+        </is>
+      </c>
+      <c r="F166" s="43" t="inlineStr">
+        <is>
+          <t>Hotel The Beacon (3-6 sep)</t>
+        </is>
+      </c>
       <c r="G166" s="40" t="inlineStr"/>
       <c r="H166" s="41" t="inlineStr"/>
       <c r="I166" s="41" t="inlineStr"/>
@@ -27096,12 +27092,12 @@
       <c r="A167" s="35" t="n"/>
       <c r="B167" s="42" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C167" s="43" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D167" s="44" t="inlineStr">
@@ -27111,63 +27107,59 @@
       </c>
       <c r="E167" s="45" t="inlineStr">
         <is>
-          <t>★ CHECKOUT de The Beacon y dejar las valijas en el bell desk. El checkout formal suele ser 11:00-12:00, pero hacerlo antes libera el día.</t>
+          <t>★ CENTRAL PARK cruzando de oeste a este: Bethesda Terrace, el Ramble, Bow Bridge. Se entra por la 72 desde Broadway, a tres cuadras del hotel.</t>
         </is>
       </c>
       <c r="F167" s="43" t="inlineStr">
         <is>
-          <t>Hotel The Beacon (3-6 sep)</t>
-        </is>
-      </c>
-      <c r="G167" s="40" t="inlineStr"/>
+          <t>Central Park</t>
+        </is>
+      </c>
+      <c r="G167" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~20 min a pie (1.5 km) o 🚇 ~15 min · estimado</t>
+        </is>
+      </c>
       <c r="H167" s="41" t="inlineStr"/>
       <c r="I167" s="41" t="inlineStr"/>
     </row>
-    <row r="168" ht="30" customHeight="1">
+    <row r="168" ht="16" customHeight="1">
       <c r="A168" s="35" t="n"/>
-      <c r="B168" s="42" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="C168" s="43" t="inlineStr">
+      <c r="B168" s="36" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="D168" s="44" t="inlineStr">
+      <c r="C168" s="37" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D168" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E168" s="45" t="inlineStr">
-        <is>
-          <t>★ CENTRAL PARK cruzando de oeste a este: Bethesda Terrace, el Ramble, Bow Bridge. Se entra por la 72 desde Broadway, a tres cuadras del hotel.</t>
-        </is>
-      </c>
-      <c r="F168" s="43" t="inlineStr">
-        <is>
-          <t>Central Park</t>
-        </is>
-      </c>
-      <c r="G168" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~20 min a pie (1.5 km) o 🚇 ~15 min · estimado</t>
-        </is>
-      </c>
+      <c r="E168" s="39" t="inlineStr">
+        <is>
+          <t>Almuerzo en el Upper East Side, saliendo del parque por la Quinta.</t>
+        </is>
+      </c>
+      <c r="F168" s="37" t="inlineStr"/>
+      <c r="G168" s="40" t="inlineStr"/>
       <c r="H168" s="41" t="inlineStr"/>
       <c r="I168" s="41" t="inlineStr"/>
     </row>
-    <row r="169" ht="16" customHeight="1">
+    <row r="169" ht="30" customHeight="1">
       <c r="A169" s="35" t="n"/>
       <c r="B169" s="36" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C169" s="37" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="D169" s="38" t="inlineStr">
@@ -27177,7 +27169,7 @@
       </c>
       <c r="E169" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en el Upper East Side, saliendo del parque por la Quinta.</t>
+          <t>Bajar a 59 St y 2ª Av: subte 6 desde 68 St-Hunter College (el 4/5 exprés NO para ahí), o caminando por la Quinta si el día está lindo.</t>
         </is>
       </c>
       <c r="F169" s="37" t="inlineStr"/>
@@ -27187,56 +27179,60 @@
     </row>
     <row r="170" ht="30" customHeight="1">
       <c r="A170" s="35" t="n"/>
-      <c r="B170" s="36" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C170" s="37" t="inlineStr">
+      <c r="B170" s="42" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="D170" s="38" t="inlineStr">
+      <c r="C170" s="43" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D170" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E170" s="39" t="inlineStr">
-        <is>
-          <t>Bajar a 59 St y 2ª Av: subte 6 desde 68 St-Hunter College (el 4/5 exprés NO para ahí), o caminando por la Quinta si el día está lindo.</t>
-        </is>
-      </c>
-      <c r="F170" s="37" t="inlineStr"/>
+      <c r="E170" s="45" t="inlineStr">
+        <is>
+          <t>★ ROOSEVELT ISLAND TRAMWAY ($3, OMNY) — cruza el East River a 76 metros de altura con el Queensboro Bridge al lado. Es la vista de $50 por el precio de un viaje de subte.</t>
+        </is>
+      </c>
+      <c r="F170" s="43" t="inlineStr">
+        <is>
+          <t>Roosevelt Island Tramway</t>
+        </is>
+      </c>
       <c r="G170" s="40" t="inlineStr"/>
       <c r="H170" s="41" t="inlineStr"/>
       <c r="I170" s="41" t="inlineStr"/>
     </row>
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="35" t="n"/>
-      <c r="B171" s="42" t="inlineStr">
-        <is>
-          <t>13:50</t>
-        </is>
-      </c>
-      <c r="C171" s="43" t="inlineStr">
+      <c r="B171" s="36" t="inlineStr">
         <is>
           <t>14:25</t>
         </is>
       </c>
-      <c r="D171" s="44" t="inlineStr">
+      <c r="C171" s="37" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D171" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E171" s="45" t="inlineStr">
-        <is>
-          <t>★ ROOSEVELT ISLAND TRAMWAY ($3, OMNY) — cruza el East River a 76 metros de altura con el Queensboro Bridge al lado. Es la vista de $50 por el precio de un viaje de subte.</t>
-        </is>
-      </c>
-      <c r="F171" s="43" t="inlineStr">
-        <is>
-          <t>Roosevelt Island Tramway</t>
+      <c r="E171" s="39" t="inlineStr">
+        <is>
+          <t>FDR Four Freedoms Park — del teleférico son ~20 min a pie por el borde del río. La última obra de Louis Kahn: granito, plátanos y una sala abierta al río apuntando a Manhattan. Gratis y vacía. Se pasa por las ruinas del Smallpox Hospital.</t>
+        </is>
+      </c>
+      <c r="F171" s="37" t="inlineStr">
+        <is>
+          <t>FDR Four Freedoms Park</t>
         </is>
       </c>
       <c r="G171" s="40" t="inlineStr"/>
@@ -27247,12 +27243,12 @@
       <c r="A172" s="35" t="n"/>
       <c r="B172" s="36" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C172" s="37" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="D172" s="38" t="inlineStr">
@@ -27262,70 +27258,70 @@
       </c>
       <c r="E172" s="39" t="inlineStr">
         <is>
-          <t>FDR Four Freedoms Park — del teleférico son ~20 min a pie por el borde del río. La última obra de Louis Kahn: granito, plátanos y una sala abierta al río apuntando a Manhattan. Gratis y vacía. Se pasa por las ruinas del Smallpox Hospital.</t>
-        </is>
-      </c>
-      <c r="F172" s="37" t="inlineStr">
-        <is>
-          <t>FDR Four Freedoms Park</t>
-        </is>
-      </c>
+          <t>SALIR 15:05 (no más tarde): caminata al teleférico + cruce + subte 4/5/6 de 59 St a 86 St suman ~50 min, y la ventana pay-what-you-wish del Guggenheim arranca 16:00 y el museo cierra 17:30 — llegar puntuales ES la visita.</t>
+        </is>
+      </c>
+      <c r="F172" s="37" t="inlineStr"/>
       <c r="G172" s="40" t="inlineStr"/>
       <c r="H172" s="41" t="inlineStr"/>
       <c r="I172" s="41" t="inlineStr"/>
     </row>
     <row r="173" ht="30" customHeight="1">
       <c r="A173" s="35" t="n"/>
-      <c r="B173" s="36" t="inlineStr">
-        <is>
-          <t>15:05</t>
-        </is>
-      </c>
-      <c r="C173" s="37" t="inlineStr">
+      <c r="B173" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D173" s="38" t="inlineStr">
+      <c r="C173" s="43" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D173" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E173" s="39" t="inlineStr">
-        <is>
-          <t>SALIR 15:05 (no más tarde): caminata al teleférico + cruce + subte 4/5/6 de 59 St a 86 St suman ~50 min, y la ventana pay-what-you-wish del Guggenheim arranca 16:00 y el museo cierra 17:30 — llegar puntuales ES la visita.</t>
-        </is>
-      </c>
-      <c r="F173" s="37" t="inlineStr"/>
+      <c r="E173" s="45" t="inlineStr">
+        <is>
+          <t>★ GUGGENHEIM — pay-what-you-wish domingos 16:00-17:30 (sugerido $10, mínimo $1). El edificio de Frank Lloyd Wright vale la visita solo: se sube en ascensor y se baja caminando la rampa. ⚠️ LLAMAR ANTES: la rotonda estaría en montaje hasta el 18 de septiembre y el pay-what-you-wish no está confirmado en fuente oficial.</t>
+        </is>
+      </c>
+      <c r="F173" s="43" t="inlineStr">
+        <is>
+          <t>Guggenheim</t>
+        </is>
+      </c>
       <c r="G173" s="40" t="inlineStr"/>
       <c r="H173" s="41" t="inlineStr"/>
       <c r="I173" s="41" t="inlineStr"/>
     </row>
-    <row r="174" ht="30" customHeight="1">
+    <row r="174" ht="16" customHeight="1">
       <c r="A174" s="35" t="n"/>
-      <c r="B174" s="42" t="inlineStr">
-        <is>
-          <t>16:00</t>
-        </is>
-      </c>
-      <c r="C174" s="43" t="inlineStr">
+      <c r="B174" s="36" t="inlineStr">
         <is>
           <t>17:45</t>
         </is>
       </c>
-      <c r="D174" s="44" t="inlineStr">
+      <c r="C174" s="37" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="D174" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E174" s="45" t="inlineStr">
-        <is>
-          <t>★ GUGGENHEIM — pay-what-you-wish domingos 16:00-17:30 (sugerido $10, mínimo $1). El edificio de Frank Lloyd Wright vale la visita solo: se sube en ascensor y se baja caminando la rampa. ⚠️ LLAMAR ANTES: la rotonda estaría en montaje hasta el 18 de septiembre y el pay-what-you-wish no está confirmado en fuente oficial.</t>
-        </is>
-      </c>
-      <c r="F174" s="43" t="inlineStr">
-        <is>
-          <t>Guggenheim</t>
+      <c r="E174" s="39" t="inlineStr">
+        <is>
+          <t>Volver caminando por Central Park hasta el hotel (~25 min) o subte 86 St → 1 a 79 St.</t>
+        </is>
+      </c>
+      <c r="F174" s="37" t="inlineStr">
+        <is>
+          <t>Hotel The Beacon (3-6 sep)</t>
         </is>
       </c>
       <c r="G174" s="40" t="inlineStr"/>
@@ -27336,12 +27332,12 @@
       <c r="A175" s="35" t="n"/>
       <c r="B175" s="36" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C175" s="37" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="D175" s="38" t="inlineStr">
@@ -27351,14 +27347,10 @@
       </c>
       <c r="E175" s="39" t="inlineStr">
         <is>
-          <t>Volver caminando por Central Park hasta el hotel (~25 min) o subte 86 St → 1 a 79 St.</t>
-        </is>
-      </c>
-      <c r="F175" s="37" t="inlineStr">
-        <is>
-          <t>Hotel The Beacon (3-6 sep)</t>
-        </is>
-      </c>
+          <t>Retirar las valijas del bell desk. Cena tranquila cerca del hotel: es la última.</t>
+        </is>
+      </c>
+      <c r="F175" s="37" t="inlineStr"/>
       <c r="G175" s="40" t="inlineStr"/>
       <c r="H175" s="41" t="inlineStr"/>
       <c r="I175" s="41" t="inlineStr"/>
@@ -27367,12 +27359,12 @@
       <c r="A176" s="35" t="n"/>
       <c r="B176" s="36" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C176" s="37" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="D176" s="38" t="inlineStr">
@@ -27382,7 +27374,7 @@
       </c>
       <c r="E176" s="39" t="inlineStr">
         <is>
-          <t>Retirar las valijas del bell desk. Cena tranquila cerca del hotel: es la última.</t>
+          <t>Salir de The Beacon. Subte 1/2/3 desde 72 St hasta 34 St-Penn Station: ~10 min, $3.</t>
         </is>
       </c>
       <c r="F176" s="37" t="inlineStr"/>
@@ -27390,16 +27382,16 @@
       <c r="H176" s="41" t="inlineStr"/>
       <c r="I176" s="41" t="inlineStr"/>
     </row>
-    <row r="177" ht="16" customHeight="1">
+    <row r="177" ht="30" customHeight="1">
       <c r="A177" s="35" t="n"/>
       <c r="B177" s="36" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C177" s="37" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="D177" s="38" t="inlineStr">
@@ -27409,7 +27401,7 @@
       </c>
       <c r="E177" s="39" t="inlineStr">
         <is>
-          <t>Salir de The Beacon. Subte 1/2/3 desde 72 St hasta 34 St-Penn Station: ~10 min, $3.</t>
+          <t>NJ Transit Penn Station → EWR, llega 20:38. $17,25 (incluye el AirTrain). VERIFICAR el horario dominical en njtransit.com unos días antes.</t>
         </is>
       </c>
       <c r="F177" s="37" t="inlineStr"/>
@@ -27417,16 +27409,16 @@
       <c r="H177" s="41" t="inlineStr"/>
       <c r="I177" s="41" t="inlineStr"/>
     </row>
-    <row r="178" ht="30" customHeight="1">
+    <row r="178" ht="16" customHeight="1">
       <c r="A178" s="35" t="n"/>
       <c r="B178" s="36" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C178" s="37" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="D178" s="38" t="inlineStr">
@@ -27436,7 +27428,7 @@
       </c>
       <c r="E178" s="39" t="inlineStr">
         <is>
-          <t>NJ Transit Penn Station → EWR, llega 20:38. $17,25 (incluye el AirTrain). VERIFICAR el horario dominical en njtransit.com unos días antes.</t>
+          <t>AirTrain hasta la terminal: 10-15 min.</t>
         </is>
       </c>
       <c r="F178" s="37" t="inlineStr"/>
@@ -27444,18 +27436,14 @@
       <c r="H178" s="41" t="inlineStr"/>
       <c r="I178" s="41" t="inlineStr"/>
     </row>
-    <row r="179" ht="16" customHeight="1">
+    <row r="179" ht="30" customHeight="1">
       <c r="A179" s="35" t="n"/>
       <c r="B179" s="36" t="inlineStr">
         <is>
-          <t>20:45</t>
-        </is>
-      </c>
-      <c r="C179" s="37" t="inlineStr">
-        <is>
           <t>20:55</t>
         </is>
       </c>
+      <c r="C179" s="37" t="inlineStr"/>
       <c r="D179" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
@@ -27463,7 +27451,7 @@
       </c>
       <c r="E179" s="39" t="inlineStr">
         <is>
-          <t>AirTrain hasta la terminal: 10-15 min.</t>
+          <t>En terminal. Faltan 2h45 para el vuelo de las 23:40 — correcto para un internacional en el domingo de Labor Day, que es la noche de más tráfico del año en EWR.</t>
         </is>
       </c>
       <c r="F179" s="37" t="inlineStr"/>
@@ -27471,31 +27459,8 @@
       <c r="H179" s="41" t="inlineStr"/>
       <c r="I179" s="41" t="inlineStr"/>
     </row>
-    <row r="180" ht="30" customHeight="1">
-      <c r="A180" s="35" t="n"/>
-      <c r="B180" s="36" t="inlineStr">
-        <is>
-          <t>20:55</t>
-        </is>
-      </c>
-      <c r="C180" s="37" t="inlineStr"/>
-      <c r="D180" s="38" t="inlineStr">
-        <is>
-          <t>Ambos</t>
-        </is>
-      </c>
-      <c r="E180" s="39" t="inlineStr">
-        <is>
-          <t>En terminal. Faltan 2h45 para el vuelo de las 23:40 — correcto para un internacional en el domingo de Labor Day, que es la noche de más tráfico del año en EWR.</t>
-        </is>
-      </c>
-      <c r="F180" s="37" t="inlineStr"/>
-      <c r="G180" s="40" t="inlineStr"/>
-      <c r="H180" s="41" t="inlineStr"/>
-      <c r="I180" s="41" t="inlineStr"/>
-    </row>
-    <row r="181" ht="32" customHeight="1">
-      <c r="A181" s="46" t="inlineStr">
+    <row r="180" ht="32" customHeight="1">
+      <c r="A180" s="46" t="inlineStr">
         <is>
           <t>ALTERNATIVA / OJO:  COLCHÓN: si algo se atrasa, el tren siguiente sale 20:55 y llega a EWR 21:16, o sea terminal ~21:35 y 2h05 antes del vuelo. Es el último que yo tomaría. // Si prefieren un último día sin moverse, salteen el teleférico y estiren Central Park hasta el Guggenheim: el parque solo da para toda la mañana y la tarde. Y si el Guggenheim tiene la rotonda cerrada, el Whitney abre los domingos. Lo que NO conviene hoy es meter algo nuevo y grande.</t>
         </is>
@@ -27510,31 +27475,31 @@
     <mergeCell ref="A46:I46"/>
     <mergeCell ref="A27:I27"/>
     <mergeCell ref="A145:I145"/>
+    <mergeCell ref="A163:I163"/>
     <mergeCell ref="A101:I101"/>
     <mergeCell ref="A86:I86"/>
     <mergeCell ref="A47:I47"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A85:I85"/>
-    <mergeCell ref="A181:I181"/>
     <mergeCell ref="A126:I126"/>
+    <mergeCell ref="A144:I144"/>
     <mergeCell ref="A125:I125"/>
-    <mergeCell ref="A165:I165"/>
+    <mergeCell ref="A180:I180"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A68:I68"/>
     <mergeCell ref="A28:I28"/>
+    <mergeCell ref="A161:I161"/>
     <mergeCell ref="A44:I44"/>
     <mergeCell ref="A102:I102"/>
     <mergeCell ref="A67:I67"/>
     <mergeCell ref="A83:I83"/>
-    <mergeCell ref="A143:I143"/>
+    <mergeCell ref="A142:I142"/>
     <mergeCell ref="A123:I123"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A146:I146"/>
-    <mergeCell ref="A162:I162"/>
     <mergeCell ref="A6:I6"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H183" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H182" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,Reservado,Confirmado,Descartado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Stone St entra: el almuerzo del jueves se muda a la calle adoquinada [fa78a1]
Era imprescindible y no estaba en ningun dia. Reemplaza el almuerzo en
Brookfield Place, que no tenia nada especial, por la traza holandesa de
1660 con las mesas afuera, a 831 m del museo del 11-S.

El costo, dicho: 10 min de ida y 12 de vuelta a One World dejan 38 minutos
para comer, y su mejor hora es el after office de 5 a 8, no el mediodia.
Las otras dos ubicaciones posibles se descartaron con numeros: el domingo
entre Mercer Labs y The Crown son 1097 m de desvio en una ventana de 25
minutos contra el atardecer, y despues del Oculus hay que estar en Queens
40 minutos mas tarde.

Quedan 36 de 38 imprescindibles agendados. Los otros dos son MoMA PS1
—pendiente de decision— y Roosevelt Island, que en los hechos se cumple el
domingo: el bloque del teleferico y el del FDR Park estan en la isla, solo
que ninguno lleva ese pid.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/NYC_2026_Planificador.xlsx
+++ b/NYC_2026_Planificador.xlsx
@@ -20806,9 +20806,9 @@
         </is>
       </c>
       <c r="R193" s="16" t="inlineStr"/>
-      <c r="S193" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="S193" s="17" t="inlineStr">
+        <is>
+          <t>Día 6 · jue 3/9</t>
         </is>
       </c>
       <c r="T193" s="18" t="inlineStr">
@@ -30318,7 +30318,7 @@
     <row r="102" ht="32" customHeight="1">
       <c r="A102" s="34" t="inlineStr">
         <is>
-          <t>La mañana y la primera tarde son el World Trade Center completo — memorial, museo y One World Observatory en una sola bajada. OJO: One World es EL MIRADOR DE DÍA a propósito — su vista es el puerto y el agua, que de noche es negra; los arcos de atardecer van en Top of the Rock (lunes) y SUMMIT (viernes). THAIS ESTÁ EN NYC CON SU EQUIPO este jueves y SE LIBERA A LAS 16:00: se encuentran por Manhattan y se van juntos al Museum of the Moving Image, que es GRATIS los jueves de 14 a 18 — estaba caído del plan y ustedes lo tienen 2/2: RECUPERADO. El día cierra con check-in, cena y Dizzy's. Siguen afuera MoMA PS1, Astoria y Gantry (no hay hueco), y el Staten Island Ferry pasó a la alternativa nocturna de hoy.</t>
+          <t>La mañana y la primera tarde son el World Trade Center completo — memorial, museo y One World Observatory en una sola bajada. OJO: One World es EL MIRADOR DE DÍA a propósito — su vista es el puerto y el agua, que de noche es negra; los arcos de atardecer van en Top of the Rock (lunes) y SUMMIT (viernes). THAIS ESTÁ EN NYC CON SU EQUIPO este jueves y SE LIBERA A LAS 16:00: se encuentran por Manhattan y se van juntos al Museum of the Moving Image, que es GRATIS los jueves de 14 a 18 — estaba caído del plan y ustedes lo tienen 2/2: RECUPERADO. El día cierra con check-in, cena y Dizzy's. Siguen afuera MoMA PS1, Astoria y Gantry (no hay hueco), y el Staten Island Ferry pasó a la alternativa nocturna de hoy. ENTRA STONE ST, que era imprescindible y no estaba en ningún día: el almuerzo se corre de Brookfield Place a la calle adoquinada, a 10 minutos del museo y 12 de One World. Se pagan 22 minutos de caminata y quedan 38 para comer — alcanza para un mediodía, aunque su mejor hora sea el after office de 5 a 8 y no la del almuerzo.</t>
         </is>
       </c>
     </row>
@@ -30542,11 +30542,19 @@
       </c>
       <c r="E110" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo cruzando West St: Hudson Eats o Le District, en Brookfield Place, con el yate harbor de fondo.</t>
-        </is>
-      </c>
-      <c r="F110" s="37" t="inlineStr"/>
-      <c r="G110" s="40" t="inlineStr"/>
+          <t>★ ALMUERZO EN STONE ST — 10 min a pie desde el museo, hacia el sureste. Calle adoquinada peatonal de 1660, la traza holandesa que sobrevivió al fuego de 1835: mesas afuera, sin autos, entre edificios de piedra. Se come rápido y se sigue: One World es a las 13:45 y son 12 min de vuelta. Plan B si llueve o no hay mesa: Hudson Eats o Le District en Brookfield Place, cruzando West St.</t>
+        </is>
+      </c>
+      <c r="F110" s="37" t="inlineStr">
+        <is>
+          <t>Stone St</t>
+        </is>
+      </c>
+      <c r="G110" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~14 min a pie · 1.1 km · estimado</t>
+        </is>
+      </c>
       <c r="H110" s="41" t="inlineStr"/>
       <c r="I110" s="41" t="inlineStr"/>
     </row>
@@ -30579,7 +30587,7 @@
       </c>
       <c r="G111" s="40" t="inlineStr">
         <is>
-          <t>🚶 ~4 min a pie · 0.2 km · estimado</t>
+          <t>🚶 ~20 min a pie (1.2 km) o 🚇 ~15 min · estimado</t>
         </is>
       </c>
       <c r="H111" s="41" t="inlineStr"/>

</xml_diff>

<commit_message>
Entran los tres museos al miercoles: Historia Natural, Frick a voluntad y MoMA [dcbe39]
Sale el Vessel (del High Line Juan quiere solo la caminata) y con las dos horas
que libera entran los tres museos que no se podian soltar:

  10:00 Historia Natural a la apertura   (era 11:30)
  13:30 Frick, arranque exacto de su ventana pay-what-you-wish del miercoles
  15:40 MoMA hasta que cierra 17:30

El almuerzo se resigna a pedido de Juan: se come de parado cruzando Central Park.
El Vessel no se pierde, esta el viernes con Thais. El Top of the Rock queda
fuera del viaje: su unica tarde era esta.

Accion abierta para hoy: comprar online el ticket del Frick ($5 minimo, garantiza
la entrada; en persona es mas barato pero sin garantia de lugar).

66 chequeos en verde.
</commit_message>
<xml_diff>
--- a/NYC_2026_Planificador.xlsx
+++ b/NYC_2026_Planificador.xlsx
@@ -5572,9 +5572,9 @@
           <t>1 E 70th St</t>
         </is>
       </c>
-      <c r="S38" s="16" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="S38" s="17" t="inlineStr">
+        <is>
+          <t>Día 5 · mié 2/9</t>
         </is>
       </c>
       <c r="T38" s="18" t="inlineStr">
@@ -21115,9 +21115,9 @@
           <t>20 Hudson Yards</t>
         </is>
       </c>
-      <c r="S195" s="17" t="inlineStr">
-        <is>
-          <t>Día 5 · mié 2/9</t>
+      <c r="S195" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="T195" s="18" t="inlineStr">
@@ -21414,7 +21414,7 @@
       </c>
       <c r="S198" s="17" t="inlineStr">
         <is>
-          <t>Día 5 · mié 2/9, Día 7 · vie 4/9</t>
+          <t>Día 7 · vie 4/9</t>
         </is>
       </c>
       <c r="T198" s="18" t="inlineStr">
@@ -21913,7 +21913,7 @@
       </c>
       <c r="S203" s="17" t="inlineStr">
         <is>
-          <t>Día 5 · mié 2/9, Día 7 · vie 4/9</t>
+          <t>Día 7 · vie 4/9</t>
         </is>
       </c>
       <c r="T203" s="18" t="inlineStr">
@@ -32651,7 +32651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I184"/>
+  <dimension ref="A1:I183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34764,14 +34764,14 @@
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="33" t="inlineStr">
         <is>
-          <t>DÍA 5 · Miércoles 02/09 · JP solo · High Line al amanecer, Vessel, Historia Natural, MoMA y McBride en Central Park  —  base: JGStay SoHo (YA NO se vuelve a New Jersey)  ·  Solo JP</t>
+          <t>DÍA 5 · Miércoles 02/09 · JP solo · High Line al amanecer, Historia Natural, Frick a voluntad, MoMA y McBride en Central Park  —  base: JGStay SoHo (YA NO se vuelve a New Jersey)  ·  Solo JP</t>
         </is>
       </c>
     </row>
     <row r="87" ht="32" customHeight="1">
       <c r="A87" s="34" t="inlineStr">
         <is>
-          <t>REARMADO EL 1/9 con dos cambios de Juan. UNO: ya no vuelve a New Jersey — se queda en el JGStay SoHo hasta el jueves y de ahí lleva las maletas a The Beacon. Eso borra la única vuelta nocturna del viaje, o sea que hoy NO hay tren que atrapar: el SummerStage se ve entero y sin mirar el reloj, y mañana se arranca a las 7:30 desde SoHo en vez de a las 5:45 desde Branchburg. DOS: Juan quiere el HIGH LINE A LAS 7 DE LA MAÑANA, cuando abre y está vacío. ⚠️ EL ENGANCHE QUE NO CIERRA SOLO: el Vessel abre a las 10:00, así que entre el final del High Line y el Vessel hay un hueco de una hora larga — se llena con el desayuno en Hudson Yards, que además reemplaza al del hotel (7-9 AM), que hoy se pierde por salir temprano. Y entra el MoMA, que quedó pendiente del lunes: cierra 17:30 y encaja justo antes del SummerStage. CERRADOS hoy: el MET (por eso fue ayer) y el Frick pierde su ventana a voluntad — ver alternativas.</t>
+          <t>REARMADO EL 1/9, SEGUNDA PASADA. Juan sacó el Vessel (del High Line quiere SOLO la caminata) y con eso se liberaron casi dos horas: ahora entran los TRES museos que no se podían soltar. El día pasó de apretado a encastrado, y el que lo hace posible es el Vessel que se fue. LA LLAVE DEL DÍA es la ventana pay-what-you-wish del FRICK, miércoles 13:30-17:30, la única de la semana: el plan la toma a las 13:30 EN PUNTO, apenas abre, y de ahí sale con tiempo para el MoMA antes de que cierre a las 17:30. Los tres horarios encajan sin margen para improvisar: AMNH abre 10:00, Frick a voluntad 13:30, MoMA cierra 17:30. Correrse media hora en el primero se paga en el último. ⚠️ HAY QUE COMPRAR EL TICKET DEL FRICK HOY: online el mínimo son $5 y GARANTIZA la entrada; en persona se puede pagar menos pero sin garantía de lugar, y un miércoles de septiembre a las 13:30 es la hora pico de la ventana. Por $5 no vale el riesgo de quedarse afuera. EL ALMUERZO SE RESIGNA, por decisión de Juan: se come algo de parado cruzando Central Park entre el museo y el Frick. Es la media hora que hace entrar todo. EL VESSEL NO SE PIERDE: está el viernes con Thais, que lo tiene 2/2 — sacarlo hoy lo mueve, no lo borra. Y como ya no hay tren a New Jersey, el SummerStage se ve entero. CERRADO hoy: el MET (por eso fue ayer).</t>
         </is>
       </c>
     </row>
@@ -34794,7 +34794,7 @@
       </c>
       <c r="E88" s="39" t="inlineStr">
         <is>
-          <t>Salir del JGStay. Subte 1 desde Canal St hasta Christopher St, o A/C/E hasta 14 St (~12 min). Hoy se pierde el desayuno incluido del hotel (7-9 AM): se desayuna a media mañana en Hudson Yards.</t>
+          <t>Salir del JGStay. Subte 1 desde Canal St hasta Christopher St, o A/C/E hasta 14 St (~12 min). Hoy se pierde el desayuno incluido del hotel (7-9 AM): se desayuna a media mañana en el Upper West Side, antes de que abra el museo.</t>
         </is>
       </c>
       <c r="F88" s="37" t="inlineStr">
@@ -34815,7 +34815,7 @@
       </c>
       <c r="C89" s="43" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="D89" s="44" t="inlineStr">
@@ -34825,7 +34825,7 @@
       </c>
       <c r="E89" s="45" t="inlineStr">
         <is>
-          <t>★★ THE HIGH LINE AL AMANECER — abre 7:00 y esta es LA hora: vacío, con el sol bajo entre los edificios y sin las hordas de la tarde. Entrar por Gansevoort St (extremo SUR) y caminar los 2,3 km hacia el norte, sin apuro. Incluye el Buda de arenisca de 9 metros de Tuan Andrew Nguyen.</t>
+          <t>★★ THE HIGH LINE AL AMANECER — abre 7:00 y esta es LA hora: vacío, con el sol bajo entre los edificios y sin las hordas de la tarde. Entrar por Gansevoort St (extremo SUR) y caminar los 2,3 km hacia el norte, sin apuro: hoy hay casi dos horas para hacerlo lento. Incluye el Buda de arenisca de 9 metros de Tuan Andrew Nguyen. SI QUIERE SUMAR 20 MINUTOS: Little Island está a 5 min de la entrada de Gansevoort y también abre temprano (6:00).</t>
         </is>
       </c>
       <c r="F89" s="43" t="inlineStr">
@@ -34841,12 +34841,12 @@
       <c r="A90" s="35" t="n"/>
       <c r="B90" s="36" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:50</t>
         </is>
       </c>
       <c r="C90" s="37" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="D90" s="38" t="inlineStr">
@@ -34856,19 +34856,11 @@
       </c>
       <c r="E90" s="39" t="inlineStr">
         <is>
-          <t>Little Island — el parque flotante de Heatherwick sobre 132 macetas de hormigón, a la altura de la calle 13. Abre 6:00, así que a esta hora también está vacío. Media hora y se sigue al norte.</t>
-        </is>
-      </c>
-      <c r="F90" s="37" t="inlineStr">
-        <is>
-          <t>Little Island</t>
-        </is>
-      </c>
-      <c r="G90" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~15 min a pie · 1.1 km · estimado</t>
-        </is>
-      </c>
+          <t>Subte al Upper West Side: A/C desde 34 St-Penn Station hasta 81 St-Museum of Natural History, directo y sin transbordo (~20 min). El High Line termina justo ahí arriba.</t>
+        </is>
+      </c>
+      <c r="F90" s="37" t="inlineStr"/>
+      <c r="G90" s="40" t="inlineStr"/>
       <c r="H90" s="41" t="inlineStr"/>
       <c r="I90" s="41" t="inlineStr"/>
     </row>
@@ -34876,7 +34868,7 @@
       <c r="A91" s="35" t="n"/>
       <c r="B91" s="36" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:20</t>
         </is>
       </c>
       <c r="C91" s="37" t="inlineStr">
@@ -34891,19 +34883,11 @@
       </c>
       <c r="E91" s="39" t="inlineStr">
         <is>
-          <t>Desayuno en Hudson Yards, al pie del Vessel — acá se llena el hueco hasta que abra. The Shops tiene opciones rápidas; si prefieren algo mejor, Mercado Little Spain de José Andrés está en la planta baja.</t>
-        </is>
-      </c>
-      <c r="F91" s="37" t="inlineStr">
-        <is>
-          <t>Hudson Yards</t>
-        </is>
-      </c>
-      <c r="G91" s="40" t="inlineStr">
-        <is>
-          <t>🚇 ~15 min en subte · 2.5 km (a pie 35 min) · estimado</t>
-        </is>
-      </c>
+          <t>Desayuno en el Upper West Side, sobre Amsterdam o Columbus, a metros del museo. Acá se llena el hueco hasta que abra el AMNH y se recupera el desayuno del hotel que se perdió por madrugar.</t>
+        </is>
+      </c>
+      <c r="F91" s="37" t="inlineStr"/>
+      <c r="G91" s="40" t="inlineStr"/>
       <c r="H91" s="41" t="inlineStr"/>
       <c r="I91" s="41" t="inlineStr"/>
     </row>
@@ -34916,7 +34900,7 @@
       </c>
       <c r="C92" s="43" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D92" s="44" t="inlineStr">
@@ -34926,19 +34910,15 @@
       </c>
       <c r="E92" s="45" t="inlineStr">
         <is>
-          <t>★ THE VESSEL — abre 10:00 EN PUNTO y conviene ser de los primeros: la escalera infinita de Heatherwick, 154 tramos y 2.500 escalones, $10. Reabierto con redes; hay ascensor cada 15 min. Subir es la única forma de entenderla.</t>
+          <t>★ AMERICAN MUSEUM OF NATURAL HISTORY — ENTRAR A LA APERTURA, 10:00 en punto: son 2h45 y el día no da más. Dinosaurios (4º piso, lo mejor), la ballena azul y el Gilder Center nuevo de Studio Gang. $37. Thais lo marcó 0: es de hoy o no es. A las 12:45 hay que estar saliendo.</t>
         </is>
       </c>
       <c r="F92" s="43" t="inlineStr">
         <is>
-          <t>The Vessel</t>
-        </is>
-      </c>
-      <c r="G92" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~7 min a pie · 0.5 km · estimado</t>
-        </is>
-      </c>
+          <t>American Museum of Natural History</t>
+        </is>
+      </c>
+      <c r="G92" s="40" t="inlineStr"/>
       <c r="H92" s="41" t="inlineStr"/>
       <c r="I92" s="41" t="inlineStr"/>
     </row>
@@ -34946,12 +34926,12 @@
       <c r="A93" s="35" t="n"/>
       <c r="B93" s="36" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="C93" s="37" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D93" s="38" t="inlineStr">
@@ -34961,7 +34941,7 @@
       </c>
       <c r="E93" s="39" t="inlineStr">
         <is>
-          <t>Subte a Historia Natural: 7 desde 34 St-Hudson Yards hasta Times Sq y 1/2/3 hasta 79 St, o A/C desde 34 St-Penn hasta 81 St (~30 min).</t>
+          <t>ALMUERZO DE PARADO cruzando Central Park — 1,3 km a pie, unos 18 min: bajar por Central Park West hasta la 72, cruzar el parque por Terrace Drive y salir a la Quinta. Comprar algo antes de entrar (hay carritos en CPW, o el café del propio museo) y comerlo caminando: esta media hora es la que hace entrar los tres museos. Al Frick no se entra con comida.</t>
         </is>
       </c>
       <c r="F93" s="37" t="inlineStr"/>
@@ -34973,12 +34953,12 @@
       <c r="A94" s="35" t="n"/>
       <c r="B94" s="42" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C94" s="43" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="D94" s="44" t="inlineStr">
@@ -34988,15 +34968,19 @@
       </c>
       <c r="E94" s="45" t="inlineStr">
         <is>
-          <t>★ AMERICAN MUSEUM OF NATURAL HISTORY — dinosaurios, la ballena azul y el Gilder Center nuevo de Studio Gang. $37. Abre 10-17:30. Thais lo marcó 0: es de hoy.</t>
+          <t>★ THE FRICK COLLECTION, A VOLUNTAD — 13:30 EN PUNTO, cuando arranca la ventana pay-what-you-wish de los miércoles, la única de la semana. Reabrió en 2025 tras cinco años de obra: Vermeer, Rembrandt y Bellini colgados en la mansión del magnate, como en una casa. Es el museo más placentero de NYC. TICKET COMPRADO ONLINE ($5 mínimo, garantiza la entrada). 1h45 alcanza bien: es chico a propósito.</t>
         </is>
       </c>
       <c r="F94" s="43" t="inlineStr">
         <is>
-          <t>American Museum of Natural History</t>
-        </is>
-      </c>
-      <c r="G94" s="40" t="inlineStr"/>
+          <t>The Frick Collection</t>
+        </is>
+      </c>
+      <c r="G94" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~25 min a pie (1.6 km) o 🚇 ~15 min · estimado</t>
+        </is>
+      </c>
       <c r="H94" s="41" t="inlineStr"/>
       <c r="I94" s="41" t="inlineStr"/>
     </row>
@@ -35004,12 +34988,12 @@
       <c r="A95" s="35" t="n"/>
       <c r="B95" s="36" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C95" s="37" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="D95" s="38" t="inlineStr">
@@ -35019,7 +35003,7 @@
       </c>
       <c r="E95" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en el Upper West Side, saliendo del museo. Amsterdam o Columbus tienen de todo; Gray's Papaya está en Broadway y 72 si quieren el pancho de parado.</t>
+          <t>Del Frick al MoMA: 1,4 km bajando por la Quinta Avenida, ~18 min a pie, con el Central Park a la derecha y las vidrieras a la izquierda. Es de los mejores paseos de Manhattan y va cuesta abajo. Alternativa si están las piernas cansadas: subte 6 desde 68 St hasta 51 St.</t>
         </is>
       </c>
       <c r="F95" s="37" t="inlineStr"/>
@@ -35027,60 +35011,60 @@
       <c r="H95" s="41" t="inlineStr"/>
       <c r="I95" s="41" t="inlineStr"/>
     </row>
-    <row r="96" ht="16" customHeight="1">
+    <row r="96" ht="30" customHeight="1">
       <c r="A96" s="35" t="n"/>
-      <c r="B96" s="36" t="inlineStr">
-        <is>
-          <t>15:15</t>
-        </is>
-      </c>
-      <c r="C96" s="37" t="inlineStr">
+      <c r="B96" s="42" t="inlineStr">
         <is>
           <t>15:40</t>
         </is>
       </c>
-      <c r="D96" s="38" t="inlineStr">
+      <c r="C96" s="43" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="D96" s="44" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E96" s="39" t="inlineStr">
-        <is>
-          <t>Subte B/C o D desde 81 St hasta 7 Av / 47-50 Sts (~15 min). Caminar al MoMA.</t>
-        </is>
-      </c>
-      <c r="F96" s="37" t="inlineStr"/>
+      <c r="E96" s="45" t="inlineStr">
+        <is>
+          <t>★ MoMA — QUEDÓ PENDIENTE DEL LUNES y hoy es su última chance del viaje: cierra 17:30, así que son 1h50. SIN VUELTAS, DERECHO AL 5º PISO: ahí están la noche estrellada de Van Gogh, Les Demoiselles d'Avignon y los Monet grandes. Si sobra tiempo, el 4º (Warhol, Rothko). QUÉ HAY AHORA: «Frida and Diego: The Last Dream», que cierra el 12 de septiembre. $30. (El viernes gratis de UNIQLO es SOLO para residentes del Estado de NY: no aplica.)</t>
+        </is>
+      </c>
+      <c r="F96" s="43" t="inlineStr">
+        <is>
+          <t>MoMA</t>
+        </is>
+      </c>
       <c r="G96" s="40" t="inlineStr"/>
       <c r="H96" s="41" t="inlineStr"/>
       <c r="I96" s="41" t="inlineStr"/>
     </row>
     <row r="97" ht="30" customHeight="1">
       <c r="A97" s="35" t="n"/>
-      <c r="B97" s="42" t="inlineStr">
-        <is>
-          <t>15:40</t>
-        </is>
-      </c>
-      <c r="C97" s="43" t="inlineStr">
+      <c r="B97" s="36" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="D97" s="44" t="inlineStr">
+      <c r="C97" s="37" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="D97" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E97" s="45" t="inlineStr">
-        <is>
-          <t>★ MoMA — QUEDÓ PENDIENTE DEL LUNES y hoy es el día: cierra 17:30, así que entrando 15:40 quedan casi dos horas, que alcanzan para las salas de arriba. Van Gogh, Picasso, Rothko, Warhol. QUÉ HAY AHORA: «Frida and Diego: The Last Dream», que cierra el 12 de septiembre. El cine está incluido en la entrada. $30.</t>
-        </is>
-      </c>
-      <c r="F97" s="43" t="inlineStr">
-        <is>
-          <t>MoMA</t>
-        </is>
-      </c>
+      <c r="E97" s="39" t="inlineStr">
+        <is>
+          <t>Del MoMA a Rumsey Playfield: 1,3 km, ~16 min a pie subiendo por la Quinta y entrando al parque por la 69. Con el cartel de hoy conviene estar temprano.</t>
+        </is>
+      </c>
+      <c r="F97" s="37" t="inlineStr"/>
       <c r="G97" s="40" t="inlineStr"/>
       <c r="H97" s="41" t="inlineStr"/>
       <c r="I97" s="41" t="inlineStr"/>
@@ -35089,12 +35073,12 @@
       <c r="A98" s="35" t="n"/>
       <c r="B98" s="36" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C98" s="37" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="D98" s="38" t="inlineStr">
@@ -35104,7 +35088,7 @@
       </c>
       <c r="E98" s="39" t="inlineStr">
         <is>
-          <t>Del MoMA a Rumsey Playfield: subte F desde 57 St hasta 63 St-Lexington y caminar, o los 20 minutos a pie por la Quinta y entrando por la 69. Con el cartel de hoy conviene estar temprano.</t>
+          <t>Entrar a Rumsey Playfield y buscar lugar. Puertas 18:00 y con este cartel se llena: cuanto antes, mejor lugar. LA CENA ES ACÁ — hoy el almuerzo fue de parado, así que esta es la comida de verdad del día: hay puestos adentro, o se compra algo en el camino por la Quinta.</t>
         </is>
       </c>
       <c r="F98" s="37" t="inlineStr"/>
@@ -35114,120 +35098,124 @@
     </row>
     <row r="99" ht="30" customHeight="1">
       <c r="A99" s="35" t="n"/>
-      <c r="B99" s="36" t="inlineStr">
-        <is>
-          <t>18:10</t>
-        </is>
-      </c>
-      <c r="C99" s="37" t="inlineStr">
+      <c r="B99" s="42" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="D99" s="38" t="inlineStr">
+      <c r="C99" s="43" t="inlineStr">
+        <is>
+          <t>22:05</t>
+        </is>
+      </c>
+      <c r="D99" s="44" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E99" s="39" t="inlineStr">
-        <is>
-          <t>Entrar a Rumsey Playfield y buscar lugar. Puertas 18:00 y con este cartel se llena: cuanto antes, mejor lugar. Comer algo acá o de camino — hoy la cena es lo que se consiga.</t>
-        </is>
-      </c>
-      <c r="F99" s="37" t="inlineStr"/>
+      <c r="E99" s="45" t="inlineStr">
+        <is>
+          <t>★★ SUMMERSTAGE: Christian McBride + SAMARA JOY + Mei Semones — Verve 70 aniversario y Getz/Gilberto. GRATIS, sin ticket, Rumsey Playfield, 19:00-22:00. Y SE VE ENTERO: ya no hay tren a New Jersey que atrapar, que era lo que obligaba a salir corriendo.</t>
+        </is>
+      </c>
+      <c r="F99" s="43" t="inlineStr">
+        <is>
+          <t>SummerStage: Christian McBride (gratis)</t>
+        </is>
+      </c>
       <c r="G99" s="40" t="inlineStr"/>
       <c r="H99" s="41" t="inlineStr"/>
       <c r="I99" s="41" t="inlineStr"/>
     </row>
     <row r="100" ht="30" customHeight="1">
       <c r="A100" s="35" t="n"/>
-      <c r="B100" s="42" t="inlineStr">
-        <is>
-          <t>19:00</t>
-        </is>
-      </c>
-      <c r="C100" s="43" t="inlineStr">
+      <c r="B100" s="36" t="inlineStr">
         <is>
           <t>22:05</t>
         </is>
       </c>
-      <c r="D100" s="44" t="inlineStr">
+      <c r="C100" s="37" t="inlineStr"/>
+      <c r="D100" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E100" s="45" t="inlineStr">
-        <is>
-          <t>★★ SUMMERSTAGE: Christian McBride + SAMARA JOY + Mei Semones — Verve 70 aniversario y Getz/Gilberto. GRATIS, sin ticket, Rumsey Playfield, 19:00-22:00. Y AHORA SE VE ENTERO: ya no hay tren a New Jersey que atrapar, que era lo que obligaba a salir corriendo.</t>
-        </is>
-      </c>
-      <c r="F100" s="43" t="inlineStr">
-        <is>
-          <t>SummerStage: Christian McBride (gratis)</t>
+      <c r="E100" s="39" t="inlineStr">
+        <is>
+          <t>Al JGStay sin apuro: subte B/C desde 72 St hasta W 4 St y caminar, o 1 hasta Canal (~35 min). Dormir en SoHo y no en Branchburg cambia el jueves entero.</t>
+        </is>
+      </c>
+      <c r="F100" s="37" t="inlineStr">
+        <is>
+          <t>JGSTAY SoHo (JP: 31 ago-2 sep)</t>
         </is>
       </c>
       <c r="G100" s="40" t="inlineStr"/>
       <c r="H100" s="41" t="inlineStr"/>
       <c r="I100" s="41" t="inlineStr"/>
     </row>
-    <row r="101" ht="30" customHeight="1">
-      <c r="A101" s="35" t="n"/>
-      <c r="B101" s="36" t="inlineStr">
-        <is>
-          <t>22:05</t>
-        </is>
-      </c>
-      <c r="C101" s="37" t="inlineStr"/>
-      <c r="D101" s="38" t="inlineStr">
+    <row r="101" ht="32" customHeight="1">
+      <c r="A101" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  LO QUE HAY QUE HACER HOY, ANTES DE DORMIR: comprar el ticket del Frick para mañana 13:30. Son $5 (el mínimo online del pay-what-you-wish) y es lo único que garantiza la entrada. Sin eso, hay que hacer la cola en persona y jugarse a que haya lugar en la hora más pedida de la única ventana semanal. // EL DÍA NO TIENE COLCHÓN, y conviene saber dónde se corta si algo se estira: el que se achica es el MoMA, porque es el último y cierra a las 17:30 pase lo que pase. Salir del AMNH 12:45 no es negociable; salir del Frick 15:15 tampoco. Si el High Line a las 7 resulta demasiado madrugón después de anoche, se puede entrar 8:30 y empezar el día en el museo: el AMNH abre 10:00 igual y nada se mueve — lo único que se acorta es el desayuno. // EL VESSEL SE FUE DE HOY y está bien que así sea: Thais lo tiene 2/2 y está en el plan del viernes, con el High Line y Little Island. Hoy Juan hace solo la caminata, que es lo que quería. // TOP OF THE ROCK: ya no entra en ningún lado. Su gracia es el atardecer y el viernes el SUMMIT —mejor mirador— ya lo tiene reservado. Si igual lo quieren, la única forma es soltar el MoMA de hoy, y el MoMA no tiene otra fecha. // Si el Frick resulta corto y sobran 20 minutos, el Guggenheim está 14 cuadras al norte por la Quinta — pero OJO, la rotonda está en montaje hasta el 17 de septiembre: es entrar a ver el edificio a medio armar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 6 · Jueves 03/09 · Traslado + World Trade Center completo + ferry con Thais  —  base: JGStay SoHo → The Beacon  ·  Solo JP</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="32" customHeight="1">
+      <c r="A104" s="34" t="inlineStr">
+        <is>
+          <t>REARMADO EL 1/9: Juan ya no duerme en New Jersey, así que el día arranca en el JGStay SoHo a las 7:30 con desayuno incluido en vez de a las 6:20 en Branchburg — hora y media más de sueño, un Uber menos y un tren menos. Las maletas van en el subte 1, directo de Canal St a 72 St, y quedan en el bell desk del Beacon antes de las 9. La mañana y la primera tarde son el World Trade Center completo — memorial, museo y One World Observatory en una sola bajada. OJO: One World es EL MIRADOR DE DÍA a propósito — su vista es el puerto y el agua, que de noche es negra; los arcos de atardecer van en Top of the Rock (lunes) y SUMMIT (viernes). THAIS ESTÁ EN NYC CON SU EQUIPO este jueves y SE LIBERA A LAS 16:00: se encuentran por Manhattan y se van juntos al Museum of the Moving Image, que es GRATIS los jueves de 14 a 18 — estaba caído del plan y ustedes lo tienen 2/2: RECUPERADO. El día cierra con check-in, cena y Dizzy's. Siguen afuera MoMA PS1, Astoria y Gantry (no hay hueco), y el Staten Island Ferry pasó a la alternativa nocturna de hoy. ENTRA STONE ST, que era imprescindible y no estaba en ningún día: el almuerzo se corre de Brookfield Place a la calle adoquinada, a 10 minutos del museo y 12 de One World. Se pagan 22 minutos de caminata y quedan 38 para comer — alcanza para un mediodía, aunque su mejor hora sea el after office de 5 a 8 y no la del almuerzo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="30" customHeight="1">
+      <c r="A105" s="35" t="n"/>
+      <c r="B105" s="36" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="C105" s="37" t="inlineStr">
+        <is>
+          <t>08:05</t>
+        </is>
+      </c>
+      <c r="D105" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E101" s="39" t="inlineStr">
-        <is>
-          <t>Al JGStay sin apuro: subte B/C desde 72 St hasta W 4 St y caminar, o 1 hasta Canal (~35 min). Dormir en SoHo y no en Branchburg cambia el jueves entero.</t>
-        </is>
-      </c>
-      <c r="F101" s="37" t="inlineStr">
+      <c r="E105" s="39" t="inlineStr">
+        <is>
+          <t>Desayuno incluido en el JGStay (7-9 AM) y CHECKOUT con las maletas. Hoy ya no se madruga a las 5:45 en Branchburg: se duerme en SoHo y se sale a las 7:30. Una hora y media más de sueño y un tren menos.</t>
+        </is>
+      </c>
+      <c r="F105" s="37" t="inlineStr">
         <is>
           <t>JGSTAY SoHo (JP: 31 ago-2 sep)</t>
         </is>
       </c>
-      <c r="G101" s="40" t="inlineStr"/>
-      <c r="H101" s="41" t="inlineStr"/>
-      <c r="I101" s="41" t="inlineStr"/>
-    </row>
-    <row r="102" ht="32" customHeight="1">
-      <c r="A102" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  EL FRICK SE CAE, y hay que decirlo: hoy era su ventana pay-what-you-wish de 13:30 a 17:30, la única de la semana, y el día quedó lleno con el High Line temprano, el Vessel y el MoMA pendiente. Si lo quieren recuperar, la única forma es soltar el MoMA o el AMNH — el Frick fuera de esa ventana son $30 por cabeza. // SI PREFIEREN EL TOP OF THE ROCK EN VEZ DEL MoMA: abre 8:00-24:00, así que entra en el mismo hueco de las 15:40. PERO su gracia es el atardecer (hoy ~19:26) y a esa hora están en el SummerStage, así que sería subir con luz plana. El MoMA cierra 17:30 y hoy es su única chance del viaje; el Top of the Rock, en cambio, compite con el SUMMIT del viernes, que ya tiene el atardecer reservado y es mejor mirador. Por eso el plan pone el MoMA. // Si el High Line a las 7 resulta demasiado madrugón después de anoche, se puede entrar 8:30 y correr todo una hora: el Vessel abre 10:00 igual y el resto del día no se mueve.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="22" customHeight="1">
-      <c r="A104" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 6 · Jueves 03/09 · Traslado + World Trade Center completo + ferry con Thais  —  base: JGStay SoHo → The Beacon  ·  Solo JP</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="32" customHeight="1">
-      <c r="A105" s="34" t="inlineStr">
-        <is>
-          <t>REARMADO EL 1/9: Juan ya no duerme en New Jersey, así que el día arranca en el JGStay SoHo a las 7:30 con desayuno incluido en vez de a las 6:20 en Branchburg — hora y media más de sueño, un Uber menos y un tren menos. Las maletas van en el subte 1, directo de Canal St a 72 St, y quedan en el bell desk del Beacon antes de las 9. La mañana y la primera tarde son el World Trade Center completo — memorial, museo y One World Observatory en una sola bajada. OJO: One World es EL MIRADOR DE DÍA a propósito — su vista es el puerto y el agua, que de noche es negra; los arcos de atardecer van en Top of the Rock (lunes) y SUMMIT (viernes). THAIS ESTÁ EN NYC CON SU EQUIPO este jueves y SE LIBERA A LAS 16:00: se encuentran por Manhattan y se van juntos al Museum of the Moving Image, que es GRATIS los jueves de 14 a 18 — estaba caído del plan y ustedes lo tienen 2/2: RECUPERADO. El día cierra con check-in, cena y Dizzy's. Siguen afuera MoMA PS1, Astoria y Gantry (no hay hueco), y el Staten Island Ferry pasó a la alternativa nocturna de hoy. ENTRA STONE ST, que era imprescindible y no estaba en ningún día: el almuerzo se corre de Brookfield Place a la calle adoquinada, a 10 minutos del museo y 12 de One World. Se pagan 22 minutos de caminata y quedan 38 para comer — alcanza para un mediodía, aunque su mejor hora sea el after office de 5 a 8 y no la del almuerzo.</t>
-        </is>
-      </c>
+      <c r="G105" s="40" t="inlineStr"/>
+      <c r="H105" s="41" t="inlineStr"/>
+      <c r="I105" s="41" t="inlineStr"/>
     </row>
     <row r="106" ht="30" customHeight="1">
       <c r="A106" s="35" t="n"/>
       <c r="B106" s="36" t="inlineStr">
         <is>
-          <t>07:30</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="C106" s="37" t="inlineStr">
         <is>
-          <t>08:05</t>
+          <t>08:35</t>
         </is>
       </c>
       <c r="D106" s="38" t="inlineStr">
@@ -35237,99 +35225,95 @@
       </c>
       <c r="E106" s="39" t="inlineStr">
         <is>
-          <t>Desayuno incluido en el JGStay (7-9 AM) y CHECKOUT con las maletas. Hoy ya no se madruga a las 5:45 en Branchburg: se duerme en SoHo y se sale a las 7:30. Una hora y media más de sueño y un tren menos.</t>
-        </is>
-      </c>
-      <c r="F106" s="37" t="inlineStr">
-        <is>
-          <t>JGSTAY SoHo (JP: 31 ago-2 sep)</t>
-        </is>
-      </c>
+          <t>Subte 1 desde Canal St derecho hasta 72 St (~25 min). Con maletas, el 1 es el que conviene: es directo y no hay que hacer transbordo.</t>
+        </is>
+      </c>
+      <c r="F106" s="37" t="inlineStr"/>
       <c r="G106" s="40" t="inlineStr"/>
       <c r="H106" s="41" t="inlineStr"/>
       <c r="I106" s="41" t="inlineStr"/>
     </row>
     <row r="107" ht="30" customHeight="1">
       <c r="A107" s="35" t="n"/>
-      <c r="B107" s="36" t="inlineStr">
-        <is>
-          <t>08:05</t>
-        </is>
-      </c>
-      <c r="C107" s="37" t="inlineStr">
+      <c r="B107" s="42" t="inlineStr">
         <is>
           <t>08:35</t>
         </is>
       </c>
-      <c r="D107" s="38" t="inlineStr">
+      <c r="C107" s="43" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="D107" s="44" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E107" s="39" t="inlineStr">
-        <is>
-          <t>Subte 1 desde Canal St derecho hasta 72 St (~25 min). Con maletas, el 1 es el que conviene: es directo y no hay que hacer transbordo.</t>
-        </is>
-      </c>
-      <c r="F107" s="37" t="inlineStr"/>
+      <c r="E107" s="45" t="inlineStr">
+        <is>
+          <t>★ THE BEACON — dejar las maletas en el bell desk. El check-in formal es a la tarde, con Thais, pero el equipaje se recibe desde temprano. Confirmalo por mail.</t>
+        </is>
+      </c>
+      <c r="F107" s="43" t="inlineStr">
+        <is>
+          <t>Hotel The Beacon (3-6 sep)</t>
+        </is>
+      </c>
       <c r="G107" s="40" t="inlineStr"/>
       <c r="H107" s="41" t="inlineStr"/>
       <c r="I107" s="41" t="inlineStr"/>
     </row>
     <row r="108" ht="30" customHeight="1">
       <c r="A108" s="35" t="n"/>
-      <c r="B108" s="42" t="inlineStr">
-        <is>
-          <t>08:35</t>
-        </is>
-      </c>
-      <c r="C108" s="43" t="inlineStr">
+      <c r="B108" s="36" t="inlineStr">
         <is>
           <t>09:05</t>
         </is>
       </c>
-      <c r="D108" s="44" t="inlineStr">
+      <c r="C108" s="37" t="inlineStr">
+        <is>
+          <t>09:50</t>
+        </is>
+      </c>
+      <c r="D108" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E108" s="45" t="inlineStr">
-        <is>
-          <t>★ THE BEACON — dejar las maletas en el bell desk. El check-in formal es a la tarde, con Thais, pero el equipaje se recibe desde temprano. Confirmalo por mail.</t>
-        </is>
-      </c>
-      <c r="F108" s="43" t="inlineStr">
-        <is>
-          <t>Hotel The Beacon (3-6 sep)</t>
-        </is>
-      </c>
+      <c r="E108" s="39" t="inlineStr">
+        <is>
+          <t>Subte 1 directo desde 72 St hasta WTC Cortlandt (~30 min), otra vez sin transbordo. Alternativa: 2/3 express hasta Chambers St y 5 min a pie.</t>
+        </is>
+      </c>
+      <c r="F108" s="37" t="inlineStr"/>
       <c r="G108" s="40" t="inlineStr"/>
       <c r="H108" s="41" t="inlineStr"/>
       <c r="I108" s="41" t="inlineStr"/>
     </row>
     <row r="109" ht="30" customHeight="1">
       <c r="A109" s="35" t="n"/>
-      <c r="B109" s="36" t="inlineStr">
-        <is>
-          <t>09:05</t>
-        </is>
-      </c>
-      <c r="C109" s="37" t="inlineStr">
+      <c r="B109" s="42" t="inlineStr">
         <is>
           <t>09:50</t>
         </is>
       </c>
-      <c r="D109" s="38" t="inlineStr">
+      <c r="C109" s="43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D109" s="44" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E109" s="39" t="inlineStr">
-        <is>
-          <t>Subte 1 directo desde 72 St hasta WTC Cortlandt (~30 min), otra vez sin transbordo. Alternativa: 2/3 express hasta Chambers St y 5 min a pie.</t>
-        </is>
-      </c>
-      <c r="F109" s="37" t="inlineStr"/>
+      <c r="E109" s="45" t="inlineStr">
+        <is>
+          <t>★ 9/11 MEMORIAL (la plaza) — las dos fuentes en las huellas de las torres y el Survivor Tree. Gratis, abierto desde las 8:00. Verlo ANTES del museo ordena la visita.</t>
+        </is>
+      </c>
+      <c r="F109" s="43" t="inlineStr"/>
       <c r="G109" s="40" t="inlineStr"/>
       <c r="H109" s="41" t="inlineStr"/>
       <c r="I109" s="41" t="inlineStr"/>
@@ -35338,12 +35322,12 @@
       <c r="A110" s="35" t="n"/>
       <c r="B110" s="42" t="inlineStr">
         <is>
-          <t>09:50</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="C110" s="43" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="D110" s="44" t="inlineStr">
@@ -35353,75 +35337,83 @@
       </c>
       <c r="E110" s="45" t="inlineStr">
         <is>
-          <t>★ 9/11 MEMORIAL (la plaza) — las dos fuentes en las huellas de las torres y el Survivor Tree. Gratis, abierto desde las 8:00. Verlo ANTES del museo ordena la visita.</t>
-        </is>
-      </c>
-      <c r="F110" s="43" t="inlineStr"/>
+          <t>★★ 9/11 MEMORIAL MUSEUM — $36, TIMED TICKET OBLIGATORIO comprado online antes (el museo no vende en puerta sin reserva). 2 horas largas; es duro y muy bien hecho. Thais lo marcó 0: por eso va en la mañana de JP solo.</t>
+        </is>
+      </c>
+      <c r="F110" s="43" t="inlineStr">
+        <is>
+          <t>9/11 Memorial Museum</t>
+        </is>
+      </c>
       <c r="G110" s="40" t="inlineStr"/>
       <c r="H110" s="41" t="inlineStr"/>
       <c r="I110" s="41" t="inlineStr"/>
     </row>
     <row r="111" ht="30" customHeight="1">
       <c r="A111" s="35" t="n"/>
-      <c r="B111" s="42" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="C111" s="43" t="inlineStr">
+      <c r="B111" s="36" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="D111" s="44" t="inlineStr">
+      <c r="C111" s="37" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D111" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E111" s="45" t="inlineStr">
-        <is>
-          <t>★★ 9/11 MEMORIAL MUSEUM — $36, TIMED TICKET OBLIGATORIO comprado online antes (el museo no vende en puerta sin reserva). 2 horas largas; es duro y muy bien hecho. Thais lo marcó 0: por eso va en la mañana de JP solo.</t>
-        </is>
-      </c>
-      <c r="F111" s="43" t="inlineStr">
-        <is>
-          <t>9/11 Memorial Museum</t>
-        </is>
-      </c>
-      <c r="G111" s="40" t="inlineStr"/>
+      <c r="E111" s="39" t="inlineStr">
+        <is>
+          <t>★ ALMUERZO EN STONE ST — 10 min a pie desde el museo, hacia el sureste. Calle adoquinada peatonal de 1660, la traza holandesa que sobrevivió al fuego de 1835: mesas afuera, sin autos, entre edificios de piedra. Se come rápido y se sigue: One World es a las 13:45 y son 12 min de vuelta. Plan B si llueve o no hay mesa: Hudson Eats o Le District en Brookfield Place, cruzando West St.</t>
+        </is>
+      </c>
+      <c r="F111" s="37" t="inlineStr">
+        <is>
+          <t>Stone St</t>
+        </is>
+      </c>
+      <c r="G111" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~14 min a pie · 1.1 km · estimado</t>
+        </is>
+      </c>
       <c r="H111" s="41" t="inlineStr"/>
       <c r="I111" s="41" t="inlineStr"/>
     </row>
     <row r="112" ht="30" customHeight="1">
       <c r="A112" s="35" t="n"/>
-      <c r="B112" s="36" t="inlineStr">
-        <is>
-          <t>12:45</t>
-        </is>
-      </c>
-      <c r="C112" s="37" t="inlineStr">
+      <c r="B112" s="42" t="inlineStr">
         <is>
           <t>13:45</t>
         </is>
       </c>
-      <c r="D112" s="38" t="inlineStr">
+      <c r="C112" s="43" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D112" s="44" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E112" s="39" t="inlineStr">
-        <is>
-          <t>★ ALMUERZO EN STONE ST — 10 min a pie desde el museo, hacia el sureste. Calle adoquinada peatonal de 1660, la traza holandesa que sobrevivió al fuego de 1835: mesas afuera, sin autos, entre edificios de piedra. Se come rápido y se sigue: One World es a las 13:45 y son 12 min de vuelta. Plan B si llueve o no hay mesa: Hudson Eats o Le District en Brookfield Place, cruzando West St.</t>
-        </is>
-      </c>
-      <c r="F112" s="37" t="inlineStr">
-        <is>
-          <t>Stone St</t>
+      <c r="E112" s="45" t="inlineStr">
+        <is>
+          <t>★★ ONE WORLD OBSERVATORY — piso 102, el punto más alto del hemisferio occidental, con el puerto y Brooklyn dominando la vista. $44+fee, ventana de entrada de 15 min: sacar el timed ticket online. JP lo subió a 2 en la última pasada.</t>
+        </is>
+      </c>
+      <c r="F112" s="43" t="inlineStr">
+        <is>
+          <t>One World Observatory</t>
         </is>
       </c>
       <c r="G112" s="40" t="inlineStr">
         <is>
-          <t>🚶 ~14 min a pie · 1.1 km · estimado</t>
+          <t>🚶 ~20 min a pie (1.2 km) o 🚇 ~15 min · estimado</t>
         </is>
       </c>
       <c r="H112" s="41" t="inlineStr"/>
@@ -35429,34 +35421,34 @@
     </row>
     <row r="113" ht="30" customHeight="1">
       <c r="A113" s="35" t="n"/>
-      <c r="B113" s="42" t="inlineStr">
-        <is>
-          <t>13:45</t>
-        </is>
-      </c>
-      <c r="C113" s="43" t="inlineStr">
+      <c r="B113" s="36" t="inlineStr">
         <is>
           <t>15:15</t>
         </is>
       </c>
-      <c r="D113" s="44" t="inlineStr">
+      <c r="C113" s="37" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D113" s="38" t="inlineStr">
         <is>
           <t>Solo JP</t>
         </is>
       </c>
-      <c r="E113" s="45" t="inlineStr">
-        <is>
-          <t>★★ ONE WORLD OBSERVATORY — piso 102, el punto más alto del hemisferio occidental, con el puerto y Brooklyn dominando la vista. $44+fee, ventana de entrada de 15 min: sacar el timed ticket online. JP lo subió a 2 en la última pasada.</t>
-        </is>
-      </c>
-      <c r="F113" s="43" t="inlineStr">
-        <is>
-          <t>One World Observatory</t>
+      <c r="E113" s="39" t="inlineStr">
+        <is>
+          <t>El Oculus en un VISTAZO (5 min — ya estás ahí, y el tiempo no da para más) y R/W desde Cortlandt St hacia el norte.</t>
+        </is>
+      </c>
+      <c r="F113" s="37" t="inlineStr">
+        <is>
+          <t>Oculus / WTC Transportation Hub</t>
         </is>
       </c>
       <c r="G113" s="40" t="inlineStr">
         <is>
-          <t>🚶 ~20 min a pie (1.2 km) o 🚇 ~15 min · estimado</t>
+          <t>🚶 ~4 min a pie · 0.3 km · estimado</t>
         </is>
       </c>
       <c r="H113" s="41" t="inlineStr"/>
@@ -35464,36 +35456,28 @@
     </row>
     <row r="114" ht="30" customHeight="1">
       <c r="A114" s="35" t="n"/>
-      <c r="B114" s="36" t="inlineStr">
-        <is>
-          <t>15:15</t>
-        </is>
-      </c>
-      <c r="C114" s="37" t="inlineStr">
+      <c r="B114" s="42" t="inlineStr">
         <is>
           <t>16:00</t>
         </is>
       </c>
-      <c r="D114" s="38" t="inlineStr">
-        <is>
-          <t>Solo JP</t>
-        </is>
-      </c>
-      <c r="E114" s="39" t="inlineStr">
-        <is>
-          <t>El Oculus en un VISTAZO (5 min — ya estás ahí, y el tiempo no da para más) y R/W desde Cortlandt St hacia el norte.</t>
-        </is>
-      </c>
-      <c r="F114" s="37" t="inlineStr">
-        <is>
-          <t>Oculus / WTC Transportation Hub</t>
-        </is>
-      </c>
-      <c r="G114" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~4 min a pie · 0.3 km · estimado</t>
-        </is>
-      </c>
+      <c r="C114" s="43" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D114" s="44" t="inlineStr">
+        <is>
+          <t>Ambos</t>
+        </is>
+      </c>
+      <c r="E114" s="45" t="inlineStr">
+        <is>
+          <t>★ ENCUENTRO CON THAIS. Lo que MÁS rinde: verse DIRECTO en la puerta del MoMI a las 16:20 (36-01 35 Ave, N/W hasta 36 Av) — cada uno llega por su lado y el museo gana 10-15 min. Si prefieren encontrarse antes en Manhattan: Lexington Av-59 St 16:00 y N/W juntos (JP puede llegar 16:05-16:10 si el WTC se estiró: avisale que es ±10).</t>
+        </is>
+      </c>
+      <c r="F114" s="43" t="inlineStr"/>
+      <c r="G114" s="40" t="inlineStr"/>
       <c r="H114" s="41" t="inlineStr"/>
       <c r="I114" s="41" t="inlineStr"/>
     </row>
@@ -35501,12 +35485,12 @@
       <c r="A115" s="35" t="n"/>
       <c r="B115" s="42" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>16:30</t>
         </is>
       </c>
       <c r="C115" s="43" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="D115" s="44" t="inlineStr">
@@ -35516,46 +35500,46 @@
       </c>
       <c r="E115" s="45" t="inlineStr">
         <is>
-          <t>★ ENCUENTRO CON THAIS. Lo que MÁS rinde: verse DIRECTO en la puerta del MoMI a las 16:20 (36-01 35 Ave, N/W hasta 36 Av) — cada uno llega por su lado y el museo gana 10-15 min. Si prefieren encontrarse antes en Manhattan: Lexington Av-59 St 16:00 y N/W juntos (JP puede llegar 16:05-16:10 si el WTC se estiró: avisale que es ±10).</t>
-        </is>
-      </c>
-      <c r="F115" s="43" t="inlineStr"/>
-      <c r="G115" s="40" t="inlineStr"/>
+          <t>★★ MUSEUM OF THE MOVING IMAGE — GRATIS los jueves 14-18, sus únicas horas del jueves. RECUPERADO: había quedado afuera del plan y ustedes lo tienen 2/2. Una hora y media alcanza para Behind the Screen y los Muppets originales de Jim Henson. Cierra 18:00 EN PUNTO. (N/W hasta 36 Av + 8 min a pie.)</t>
+        </is>
+      </c>
+      <c r="F115" s="43" t="inlineStr">
+        <is>
+          <t>Museum of the Moving Image</t>
+        </is>
+      </c>
+      <c r="G115" s="40" t="inlineStr">
+        <is>
+          <t>🚇 ~40 min en subte · 11.5 km (a pie 155 min) · estimado</t>
+        </is>
+      </c>
       <c r="H115" s="41" t="inlineStr"/>
       <c r="I115" s="41" t="inlineStr"/>
     </row>
-    <row r="116" ht="30" customHeight="1">
+    <row r="116" ht="16" customHeight="1">
       <c r="A116" s="35" t="n"/>
-      <c r="B116" s="42" t="inlineStr">
-        <is>
-          <t>16:30</t>
-        </is>
-      </c>
-      <c r="C116" s="43" t="inlineStr">
+      <c r="B116" s="36" t="inlineStr">
         <is>
           <t>18:05</t>
         </is>
       </c>
-      <c r="D116" s="44" t="inlineStr">
+      <c r="C116" s="37" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="D116" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E116" s="45" t="inlineStr">
-        <is>
-          <t>★★ MUSEUM OF THE MOVING IMAGE — GRATIS los jueves 14-18, sus únicas horas del jueves. RECUPERADO: había quedado afuera del plan y ustedes lo tienen 2/2. Una hora y media alcanza para Behind the Screen y los Muppets originales de Jim Henson. Cierra 18:00 EN PUNTO. (N/W hasta 36 Av + 8 min a pie.)</t>
-        </is>
-      </c>
-      <c r="F116" s="43" t="inlineStr">
-        <is>
-          <t>Museum of the Moving Image</t>
-        </is>
-      </c>
-      <c r="G116" s="40" t="inlineStr">
-        <is>
-          <t>🚇 ~40 min en subte · 11.5 km (a pie 155 min) · estimado</t>
-        </is>
-      </c>
+      <c r="E116" s="39" t="inlineStr">
+        <is>
+          <t>Subte N/W desde 36 Av hasta Times Sq y 1/2/3 hasta 72 St (~45 min).</t>
+        </is>
+      </c>
+      <c r="F116" s="37" t="inlineStr"/>
+      <c r="G116" s="40" t="inlineStr"/>
       <c r="H116" s="41" t="inlineStr"/>
       <c r="I116" s="41" t="inlineStr"/>
     </row>
@@ -35563,12 +35547,12 @@
       <c r="A117" s="35" t="n"/>
       <c r="B117" s="36" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C117" s="37" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="D117" s="38" t="inlineStr">
@@ -35578,24 +35562,28 @@
       </c>
       <c r="E117" s="39" t="inlineStr">
         <is>
-          <t>Subte N/W desde 36 Av hasta Times Sq y 1/2/3 hasta 72 St (~45 min).</t>
-        </is>
-      </c>
-      <c r="F117" s="37" t="inlineStr"/>
+          <t>The Beacon: check-in formal y subir las maletas.</t>
+        </is>
+      </c>
+      <c r="F117" s="37" t="inlineStr">
+        <is>
+          <t>Hotel The Beacon (3-6 sep)</t>
+        </is>
+      </c>
       <c r="G117" s="40" t="inlineStr"/>
       <c r="H117" s="41" t="inlineStr"/>
       <c r="I117" s="41" t="inlineStr"/>
     </row>
-    <row r="118" ht="16" customHeight="1">
+    <row r="118" ht="30" customHeight="1">
       <c r="A118" s="35" t="n"/>
       <c r="B118" s="36" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>19:15</t>
         </is>
       </c>
       <c r="C118" s="37" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="D118" s="38" t="inlineStr">
@@ -35605,134 +35593,130 @@
       </c>
       <c r="E118" s="39" t="inlineStr">
         <is>
-          <t>The Beacon: check-in formal y subir las maletas.</t>
-        </is>
-      </c>
-      <c r="F118" s="37" t="inlineStr">
-        <is>
-          <t>Hotel The Beacon (3-6 sep)</t>
-        </is>
-      </c>
+          <t>Cena RÁPIDA en el Upper West Side, bajando por Broadway o Columbus. Hoy se come temprano y liviano: la noche tiene tres paradas y todas valen.</t>
+        </is>
+      </c>
+      <c r="F118" s="37" t="inlineStr"/>
       <c r="G118" s="40" t="inlineStr"/>
       <c r="H118" s="41" t="inlineStr"/>
       <c r="I118" s="41" t="inlineStr"/>
     </row>
     <row r="119" ht="30" customHeight="1">
       <c r="A119" s="35" t="n"/>
-      <c r="B119" s="36" t="inlineStr">
-        <is>
-          <t>19:15</t>
-        </is>
-      </c>
-      <c r="C119" s="37" t="inlineStr">
+      <c r="B119" s="42" t="inlineStr">
         <is>
           <t>19:55</t>
         </is>
       </c>
-      <c r="D119" s="38" t="inlineStr">
+      <c r="C119" s="43" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="D119" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E119" s="39" t="inlineStr">
-        <is>
-          <t>Cena RÁPIDA en el Upper West Side, bajando por Broadway o Columbus. Hoy se come temprano y liviano: la noche tiene tres paradas y todas valen.</t>
-        </is>
-      </c>
-      <c r="F119" s="37" t="inlineStr"/>
-      <c r="G119" s="40" t="inlineStr"/>
+      <c r="E119" s="45" t="inlineStr">
+        <is>
+          <t>★ LINCOLN CENTER DE NOCHE (gratis, 20 min) — OJO, VERIFICADO el 27/8 y cambia lo que van a encontrar: esta noche la Josie Robertson Plaza NO está tranquila. El Met proyecta Tristan und Isolde (actos II y III) a las 20:00 en pantalla gigante, gratis y sin reserva, y despejan la plaza desde las 18:00 para armar 2.500 sillas. O sea: llegan justo cuando se está llenando. La fuente y los chandeliers siguen ahí, pero con multitud y pantalla. Puede ser mejor que el plan original —hay ambiente de estreno— o puede ser un quilombo: decidan en el momento. Si prefieren el Lincoln Center vacío, el espejo de agua con el Henry Moore está del lado norte, detrás del Vivian Beaumont, y ahí no hay nadie.</t>
+        </is>
+      </c>
+      <c r="F119" s="43" t="inlineStr">
+        <is>
+          <t>Lincoln Center (campus y plaza)</t>
+        </is>
+      </c>
+      <c r="G119" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~20 min a pie (1.3 km) o 🚇 ~15 min · estimado</t>
+        </is>
+      </c>
       <c r="H119" s="41" t="inlineStr"/>
       <c r="I119" s="41" t="inlineStr"/>
     </row>
-    <row r="120" ht="30" customHeight="1">
+    <row r="120" ht="16" customHeight="1">
       <c r="A120" s="35" t="n"/>
-      <c r="B120" s="42" t="inlineStr">
-        <is>
-          <t>19:55</t>
-        </is>
-      </c>
-      <c r="C120" s="43" t="inlineStr">
+      <c r="B120" s="36" t="inlineStr">
         <is>
           <t>20:20</t>
         </is>
       </c>
-      <c r="D120" s="44" t="inlineStr">
+      <c r="C120" s="37" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="D120" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E120" s="45" t="inlineStr">
-        <is>
-          <t>★ LINCOLN CENTER DE NOCHE (gratis, 20 min) — OJO, VERIFICADO el 27/8 y cambia lo que van a encontrar: esta noche la Josie Robertson Plaza NO está tranquila. El Met proyecta Tristan und Isolde (actos II y III) a las 20:00 en pantalla gigante, gratis y sin reserva, y despejan la plaza desde las 18:00 para armar 2.500 sillas. O sea: llegan justo cuando se está llenando. La fuente y los chandeliers siguen ahí, pero con multitud y pantalla. Puede ser mejor que el plan original —hay ambiente de estreno— o puede ser un quilombo: decidan en el momento. Si prefieren el Lincoln Center vacío, el espejo de agua con el Henry Moore está del lado norte, detrás del Vivian Beaumont, y ahí no hay nadie.</t>
-        </is>
-      </c>
-      <c r="F120" s="43" t="inlineStr">
-        <is>
-          <t>Lincoln Center (campus y plaza)</t>
-        </is>
-      </c>
-      <c r="G120" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~20 min a pie (1.3 km) o 🚇 ~15 min · estimado</t>
-        </is>
-      </c>
+      <c r="E120" s="39" t="inlineStr">
+        <is>
+          <t>Caminar seis cuadras por Broadway hasta Columbus Circle (~8 min).</t>
+        </is>
+      </c>
+      <c r="F120" s="37" t="inlineStr"/>
+      <c r="G120" s="40" t="inlineStr"/>
       <c r="H120" s="41" t="inlineStr"/>
       <c r="I120" s="41" t="inlineStr"/>
     </row>
-    <row r="121" ht="16" customHeight="1">
+    <row r="121" ht="30" customHeight="1">
       <c r="A121" s="35" t="n"/>
-      <c r="B121" s="36" t="inlineStr">
-        <is>
-          <t>20:20</t>
-        </is>
-      </c>
-      <c r="C121" s="37" t="inlineStr">
+      <c r="B121" s="42" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="D121" s="38" t="inlineStr">
+      <c r="C121" s="43" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="D121" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E121" s="39" t="inlineStr">
-        <is>
-          <t>Caminar seis cuadras por Broadway hasta Columbus Circle (~8 min).</t>
-        </is>
-      </c>
-      <c r="F121" s="37" t="inlineStr"/>
+      <c r="E121" s="45" t="inlineStr">
+        <is>
+          <t>★★ MO LOUNGE, PISO 35 DEL MANDARIN ORIENTAL (80 Columbus Circle) — el dato del amigo de Juan, con una corrección: es el piso 35, no el 60 (el hotel ocupa del 35 al 54). Ventanales de piso a techo sobre Central Park con la ciudad encendida abajo. Coctel ~$26-32, sin cover. RESERVAR por SevenRooms desde su web. Si prefieren algo más íntimo, en ese MISMO piso está The Bar (ex speakeasy The Office, 45 asientos, mar-sáb 17-1h).</t>
+        </is>
+      </c>
+      <c r="F121" s="43" t="inlineStr">
+        <is>
+          <t>MO Lounge — Mandarin Oriental (piso 35)</t>
+        </is>
+      </c>
       <c r="G121" s="40" t="inlineStr"/>
       <c r="H121" s="41" t="inlineStr"/>
       <c r="I121" s="41" t="inlineStr"/>
     </row>
     <row r="122" ht="30" customHeight="1">
       <c r="A122" s="35" t="n"/>
-      <c r="B122" s="42" t="inlineStr">
-        <is>
-          <t>20:30</t>
-        </is>
-      </c>
-      <c r="C122" s="43" t="inlineStr">
+      <c r="B122" s="36" t="inlineStr">
         <is>
           <t>20:55</t>
         </is>
       </c>
-      <c r="D122" s="44" t="inlineStr">
+      <c r="C122" s="37" t="inlineStr">
+        <is>
+          <t>21:00</t>
+        </is>
+      </c>
+      <c r="D122" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E122" s="45" t="inlineStr">
-        <is>
-          <t>★★ MO LOUNGE, PISO 35 DEL MANDARIN ORIENTAL (80 Columbus Circle) — el dato del amigo de Juan, con una corrección: es el piso 35, no el 60 (el hotel ocupa del 35 al 54). Ventanales de piso a techo sobre Central Park con la ciudad encendida abajo. Coctel ~$26-32, sin cover. RESERVAR por SevenRooms desde su web. Si prefieren algo más íntimo, en ese MISMO piso está The Bar (ex speakeasy The Office, 45 asientos, mar-sáb 17-1h).</t>
-        </is>
-      </c>
-      <c r="F122" s="43" t="inlineStr">
-        <is>
-          <t>MO Lounge — Mandarin Oriental (piso 35)</t>
-        </is>
-      </c>
+      <c r="E122" s="39" t="inlineStr">
+        <is>
+          <t>Bajar en ascensor: Dizzy's está EN EL MISMO EDIFICIO (10 Columbus Circle, piso 5). Cero calle, cero frío.</t>
+        </is>
+      </c>
+      <c r="F122" s="37" t="inlineStr"/>
       <c r="G122" s="40" t="inlineStr"/>
       <c r="H122" s="41" t="inlineStr"/>
       <c r="I122" s="41" t="inlineStr"/>
@@ -35741,14 +35725,10 @@
       <c r="A123" s="35" t="n"/>
       <c r="B123" s="36" t="inlineStr">
         <is>
-          <t>20:55</t>
-        </is>
-      </c>
-      <c r="C123" s="37" t="inlineStr">
-        <is>
           <t>21:00</t>
         </is>
       </c>
+      <c r="C123" s="37" t="inlineStr"/>
       <c r="D123" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
@@ -35756,72 +35736,76 @@
       </c>
       <c r="E123" s="39" t="inlineStr">
         <is>
-          <t>Bajar en ascensor: Dizzy's está EN EL MISMO EDIFICIO (10 Columbus Circle, piso 5). Cero calle, cero frío.</t>
-        </is>
-      </c>
-      <c r="F123" s="37" t="inlineStr"/>
+          <t>★ Dizzy's Club — ventanales sobre Central Park detrás del escenario, un piso abajo del cóctel. SEAMOS HONESTOS: JP lleva ~17 horas en pie con 5 de sueño. Decidan A LAS 20:00, arriba en el Mandarin: si están enteros, bajan; si no, se quedan con la vista y el trago, que ya es un cierre precioso. El set Late Night (~22:45) cuesta una fracción — variante para valientes.</t>
+        </is>
+      </c>
+      <c r="F123" s="37" t="inlineStr">
+        <is>
+          <t>Dizzy's Club (Jazz at Lincoln Center)</t>
+        </is>
+      </c>
       <c r="G123" s="40" t="inlineStr"/>
       <c r="H123" s="41" t="inlineStr"/>
       <c r="I123" s="41" t="inlineStr"/>
     </row>
-    <row r="124" ht="30" customHeight="1">
-      <c r="A124" s="35" t="n"/>
-      <c r="B124" s="36" t="inlineStr">
-        <is>
-          <t>21:00</t>
-        </is>
-      </c>
-      <c r="C124" s="37" t="inlineStr"/>
-      <c r="D124" s="38" t="inlineStr">
+    <row r="124" ht="32" customHeight="1">
+      <c r="A124" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  ⚠️ EL PROBLEMA DE LA NOCHE ANTERIOR: si JP viaja desde New Jersey el jueves, significa que durmió allá el miércoles — y el miércoles el SummerStage termina a las 22:00 en Central Park. Llegando a Penn ~22:25 se toma el directo de las 22:48, que deja en Raritan ~0:04, más Uber: llegada al hotel ~0:25 y despertador a las 5:45. Son cinco horas de sueño antes de un día completo. Tres salidas: (a) salir del SummerStage a las 21:15, después del set principal; (b) quedarse una noche más en el JGStay y que Thais lleve las maletas el jueves (implica tocar la reserva); (c) tomar el tren de las 7:13 en vez del de 6:55 y arrancar 20 minutos más tarde. Verificá los horarios exactos de la tarde-noche en njtransit.com: solo tengo confirmado el directo de las 22:48. // EL FERRY, SI LES DUELE (lo tienen 2/2): al salir del MoMI, W directo hasta Whitehall (~50 min), ferry ~19:15 — el atardecer (~19:22) de ida y la Estatua y el skyline ILUMINADOS de vuelta; check-in ~21:15, cena tarde cerca del hotel, y Dizzy's tiene set Late Night los jueves ~22:45 como consuelo. Es MÁS día: elíjanlo solo si llegan enteros. // Siguen afuera: MoMA PS1, Astoria y Gantry (sin hueco); ya habían salido Noguchi, Astoria Park y Socrates por interés bajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 7 · Viernes 04/09 · Vessel + High Line, SUMMIT al atardecer y el VANGUARD de a dos  —  base: The Beacon  ·  Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="32" customHeight="1">
+      <c r="A127" s="34" t="inlineStr">
+        <is>
+          <t>Salieron el West Village, Washington Square y el Whitney; entraron el High Line, THE VESSEL (al pie del arranque, $10 y 45 min), la Morgan (hoy GRATIS 17-20) y SUMMIT — que se movió AL ATARDECER por el pedido de ustedes: entrada 18:10, luz plena, la puesta ~19:21 multiplicada por los espejos de Kusama (es EL lugar de la ciudad para ese momento) y la noche encendida hasta las 20:15. EL PAGO, dicho honesto: la Morgan se hace en una hora entrando 17:00 en punto, y la cena de hoy es un bocado rápido — por eso el almuerzo en Chelsea Market es EL fuerte del día. SALIÓ GRAND CENTRAL: estaba a las 16:20 con el argumento de que JP ya lo vio el lunes y Thais no — pero ella lo tiene en 0, así que eran 40 minutos para alguien que no lo quiere. Sin esa parada tampoco hace falta cortar Chelsea a las 15:50: se sale 16:25 derecho a la Morgan y la tarde de galerías y almuerzo gana una hora larga.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="35" t="n"/>
+      <c r="B128" s="36" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C128" s="37" t="inlineStr">
+        <is>
+          <t>09:40</t>
+        </is>
+      </c>
+      <c r="D128" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E124" s="39" t="inlineStr">
-        <is>
-          <t>★ Dizzy's Club — ventanales sobre Central Park detrás del escenario, un piso abajo del cóctel. SEAMOS HONESTOS: JP lleva ~17 horas en pie con 5 de sueño. Decidan A LAS 20:00, arriba en el Mandarin: si están enteros, bajan; si no, se quedan con la vista y el trago, que ya es un cierre precioso. El set Late Night (~22:45) cuesta una fracción — variante para valientes.</t>
-        </is>
-      </c>
-      <c r="F124" s="37" t="inlineStr">
-        <is>
-          <t>Dizzy's Club (Jazz at Lincoln Center)</t>
-        </is>
-      </c>
-      <c r="G124" s="40" t="inlineStr"/>
-      <c r="H124" s="41" t="inlineStr"/>
-      <c r="I124" s="41" t="inlineStr"/>
-    </row>
-    <row r="125" ht="32" customHeight="1">
-      <c r="A125" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  ⚠️ EL PROBLEMA DE LA NOCHE ANTERIOR: si JP viaja desde New Jersey el jueves, significa que durmió allá el miércoles — y el miércoles el SummerStage termina a las 22:00 en Central Park. Llegando a Penn ~22:25 se toma el directo de las 22:48, que deja en Raritan ~0:04, más Uber: llegada al hotel ~0:25 y despertador a las 5:45. Son cinco horas de sueño antes de un día completo. Tres salidas: (a) salir del SummerStage a las 21:15, después del set principal; (b) quedarse una noche más en el JGStay y que Thais lleve las maletas el jueves (implica tocar la reserva); (c) tomar el tren de las 7:13 en vez del de 6:55 y arrancar 20 minutos más tarde. Verificá los horarios exactos de la tarde-noche en njtransit.com: solo tengo confirmado el directo de las 22:48. // EL FERRY, SI LES DUELE (lo tienen 2/2): al salir del MoMI, W directo hasta Whitehall (~50 min), ferry ~19:15 — el atardecer (~19:22) de ida y la Estatua y el skyline ILUMINADOS de vuelta; check-in ~21:15, cena tarde cerca del hotel, y Dizzy's tiene set Late Night los jueves ~22:45 como consuelo. Es MÁS día: elíjanlo solo si llegan enteros. // Siguen afuera: MoMA PS1, Astoria y Gantry (sin hueco); ya habían salido Noguchi, Astoria Park y Socrates por interés bajo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="22" customHeight="1">
-      <c r="A127" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 7 · Viernes 04/09 · Vessel + High Line, SUMMIT al atardecer y el VANGUARD de a dos  —  base: The Beacon  ·  Ambos</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="32" customHeight="1">
-      <c r="A128" s="34" t="inlineStr">
-        <is>
-          <t>Salieron el West Village, Washington Square y el Whitney; entraron el High Line, THE VESSEL (al pie del arranque, $10 y 45 min), la Morgan (hoy GRATIS 17-20) y SUMMIT — que se movió AL ATARDECER por el pedido de ustedes: entrada 18:10, luz plena, la puesta ~19:21 multiplicada por los espejos de Kusama (es EL lugar de la ciudad para ese momento) y la noche encendida hasta las 20:15. EL PAGO, dicho honesto: la Morgan se hace en una hora entrando 17:00 en punto, y la cena de hoy es un bocado rápido — por eso el almuerzo en Chelsea Market es EL fuerte del día. SALIÓ GRAND CENTRAL: estaba a las 16:20 con el argumento de que JP ya lo vio el lunes y Thais no — pero ella lo tiene en 0, así que eran 40 minutos para alguien que no lo quiere. Sin esa parada tampoco hace falta cortar Chelsea a las 15:50: se sale 16:25 derecho a la Morgan y la tarde de galerías y almuerzo gana una hora larga.</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="16" customHeight="1">
+      <c r="E128" s="39" t="inlineStr">
+        <is>
+          <t>Subte a Hudson Yards.</t>
+        </is>
+      </c>
+      <c r="F128" s="37" t="inlineStr"/>
+      <c r="G128" s="40" t="inlineStr"/>
+      <c r="H128" s="41" t="inlineStr"/>
+      <c r="I128" s="41" t="inlineStr"/>
+    </row>
+    <row r="129" ht="30" customHeight="1">
       <c r="A129" s="35" t="n"/>
       <c r="B129" s="36" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="C129" s="37" t="inlineStr">
         <is>
-          <t>09:40</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D129" s="38" t="inlineStr">
@@ -35831,7 +35815,7 @@
       </c>
       <c r="E129" s="39" t="inlineStr">
         <is>
-          <t>Subte a Hudson Yards.</t>
+          <t>La plaza de Hudson Yards mientras abre el Vessel: The Shops y el Shed desde afuera. Sacar el timed ticket de las 10:00 online antes.</t>
         </is>
       </c>
       <c r="F129" s="37" t="inlineStr"/>
@@ -35841,27 +35825,31 @@
     </row>
     <row r="130" ht="30" customHeight="1">
       <c r="A130" s="35" t="n"/>
-      <c r="B130" s="36" t="inlineStr">
-        <is>
-          <t>09:40</t>
-        </is>
-      </c>
-      <c r="C130" s="37" t="inlineStr">
+      <c r="B130" s="42" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="D130" s="38" t="inlineStr">
+      <c r="C130" s="43" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="D130" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E130" s="39" t="inlineStr">
-        <is>
-          <t>La plaza de Hudson Yards mientras abre el Vessel: The Shops y el Shed desde afuera. Sacar el timed ticket de las 10:00 online antes.</t>
-        </is>
-      </c>
-      <c r="F130" s="37" t="inlineStr"/>
+      <c r="E130" s="45" t="inlineStr">
+        <is>
+          <t>★ THE VESSEL — la escalera infinita de Heatherwick: 154 tramos, 2.500 escalones, $10. Reabierto con redes; algunos tramos altos hacia el Hudson siguen cerrados, y hay ascensor cada 15 min. Subir es la única forma de entenderla. Si Thais prefiere no subir, la plaza está al pie.</t>
+        </is>
+      </c>
+      <c r="F130" s="43" t="inlineStr">
+        <is>
+          <t>The Vessel</t>
+        </is>
+      </c>
       <c r="G130" s="40" t="inlineStr"/>
       <c r="H130" s="41" t="inlineStr"/>
       <c r="I130" s="41" t="inlineStr"/>
@@ -35870,12 +35858,12 @@
       <c r="A131" s="35" t="n"/>
       <c r="B131" s="42" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="C131" s="43" t="inlineStr">
         <is>
-          <t>10:50</t>
+          <t>12:20</t>
         </is>
       </c>
       <c r="D131" s="44" t="inlineStr">
@@ -35885,48 +35873,52 @@
       </c>
       <c r="E131" s="45" t="inlineStr">
         <is>
-          <t>★ THE VESSEL — la escalera infinita de Heatherwick: 154 tramos, 2.500 escalones, $10. Reabierto con redes; algunos tramos altos hacia el Hudson siguen cerrados, y hay ascensor cada 15 min. Subir es la única forma de entenderla. Si Thais prefiere no subir, la plaza está al pie.</t>
+          <t>★ THE HIGH LINE completo, de norte a sur (2,3 km) — arranca ahí mismo, en 30th y 10ª. Vía ferroviaria elevada convertida en parque lineal. Incluye el Buda de arenisca de 9 metros de Tuan Andrew Nguyen.</t>
         </is>
       </c>
       <c r="F131" s="43" t="inlineStr">
         <is>
-          <t>The Vessel</t>
-        </is>
-      </c>
-      <c r="G131" s="40" t="inlineStr"/>
+          <t>The High Line</t>
+        </is>
+      </c>
+      <c r="G131" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~12 min a pie · 0.9 km · estimado</t>
+        </is>
+      </c>
       <c r="H131" s="41" t="inlineStr"/>
       <c r="I131" s="41" t="inlineStr"/>
     </row>
     <row r="132" ht="30" customHeight="1">
       <c r="A132" s="35" t="n"/>
-      <c r="B132" s="42" t="inlineStr">
-        <is>
-          <t>10:50</t>
-        </is>
-      </c>
-      <c r="C132" s="43" t="inlineStr">
+      <c r="B132" s="36" t="inlineStr">
         <is>
           <t>12:20</t>
         </is>
       </c>
-      <c r="D132" s="44" t="inlineStr">
+      <c r="C132" s="37" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D132" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E132" s="45" t="inlineStr">
-        <is>
-          <t>★ THE HIGH LINE completo, de norte a sur (2,3 km) — arranca ahí mismo, en 30th y 10ª. Vía ferroviaria elevada convertida en parque lineal. Incluye el Buda de arenisca de 9 metros de Tuan Andrew Nguyen.</t>
-        </is>
-      </c>
-      <c r="F132" s="43" t="inlineStr">
-        <is>
-          <t>The High Line</t>
+      <c r="E132" s="39" t="inlineStr">
+        <is>
+          <t>Little Island — el parque flotante de Heatherwick sobre 132 macetas de hormigón, al final del High Line. Gratis.</t>
+        </is>
+      </c>
+      <c r="F132" s="37" t="inlineStr">
+        <is>
+          <t>Little Island</t>
         </is>
       </c>
       <c r="G132" s="40" t="inlineStr">
         <is>
-          <t>🚶 ~12 min a pie · 0.9 km · estimado</t>
+          <t>🚶 ~15 min a pie · 1.1 km · estimado</t>
         </is>
       </c>
       <c r="H132" s="41" t="inlineStr"/>
@@ -35934,63 +35926,63 @@
     </row>
     <row r="133" ht="30" customHeight="1">
       <c r="A133" s="35" t="n"/>
-      <c r="B133" s="36" t="inlineStr">
-        <is>
-          <t>12:20</t>
-        </is>
-      </c>
-      <c r="C133" s="37" t="inlineStr">
+      <c r="B133" s="42" t="inlineStr">
         <is>
           <t>13:00</t>
         </is>
       </c>
-      <c r="D133" s="38" t="inlineStr">
+      <c r="C133" s="43" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="D133" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E133" s="39" t="inlineStr">
-        <is>
-          <t>Little Island — el parque flotante de Heatherwick sobre 132 macetas de hormigón, al final del High Line. Gratis.</t>
-        </is>
-      </c>
-      <c r="F133" s="37" t="inlineStr">
-        <is>
-          <t>Little Island</t>
-        </is>
-      </c>
-      <c r="G133" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~15 min a pie · 1.1 km · estimado</t>
-        </is>
-      </c>
+      <c r="E133" s="45" t="inlineStr">
+        <is>
+          <t>Galerías de Chelsea COMPLETAS — W 19th a W 27th entre la 10ª y la 11ª, concentradas en W 24th y W 21st (Gagosian, Pace, Zwirner). Gratis, se entra y se sale. El recorte del Vessel se devolvió: SUMMIT pasó al atardecer y la tarde se estiró.</t>
+        </is>
+      </c>
+      <c r="F133" s="43" t="inlineStr"/>
+      <c r="G133" s="40" t="inlineStr"/>
       <c r="H133" s="41" t="inlineStr"/>
       <c r="I133" s="41" t="inlineStr"/>
     </row>
     <row r="134" ht="30" customHeight="1">
       <c r="A134" s="35" t="n"/>
-      <c r="B134" s="42" t="inlineStr">
-        <is>
-          <t>13:00</t>
-        </is>
-      </c>
-      <c r="C134" s="43" t="inlineStr">
+      <c r="B134" s="36" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="D134" s="44" t="inlineStr">
+      <c r="C134" s="37" t="inlineStr">
+        <is>
+          <t>16:25</t>
+        </is>
+      </c>
+      <c r="D134" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E134" s="45" t="inlineStr">
-        <is>
-          <t>Galerías de Chelsea COMPLETAS — W 19th a W 27th entre la 10ª y la 11ª, concentradas en W 24th y W 21st (Gagosian, Pace, Zwirner). Gratis, se entra y se sale. El recorte del Vessel se devolvió: SUMMIT pasó al atardecer y la tarde se estiró.</t>
-        </is>
-      </c>
-      <c r="F134" s="43" t="inlineStr"/>
-      <c r="G134" s="40" t="inlineStr"/>
+      <c r="E134" s="39" t="inlineStr">
+        <is>
+          <t>Almuerzo en Chelsea Market — COMER FUERTE: es la comida grande del día, la cena de hoy es un bocado rápido entre el SUMMIT y el Vanguard. Los Tacos No.1 o Very Fresh Noodles. Ahora hay casi DOS HORAS: sin apuro, y si quedaron galerías de Chelsea sin ver, se vuelve. ★ HEATONIST está ADENTRO de este mismo mercado (12-18:45): más de 100 salsas picantes para probar, con el lineup de Hot Ones. Si el sábado no llegan a la de Williamsburg, esta es la misma cata en menos metros.</t>
+        </is>
+      </c>
+      <c r="F134" s="37" t="inlineStr">
+        <is>
+          <t>Chelsea Market</t>
+        </is>
+      </c>
+      <c r="G134" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~7 min a pie · 0.5 km · estimado</t>
+        </is>
+      </c>
       <c r="H134" s="41" t="inlineStr"/>
       <c r="I134" s="41" t="inlineStr"/>
     </row>
@@ -35998,12 +35990,12 @@
       <c r="A135" s="35" t="n"/>
       <c r="B135" s="36" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C135" s="37" t="inlineStr">
         <is>
-          <t>16:25</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D135" s="38" t="inlineStr">
@@ -36013,134 +36005,126 @@
       </c>
       <c r="E135" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en Chelsea Market — COMER FUERTE: es la comida grande del día, la cena de hoy es un bocado rápido entre el SUMMIT y el Vanguard. Los Tacos No.1 o Very Fresh Noodles. Ahora hay casi DOS HORAS: sin apuro, y si quedaron galerías de Chelsea sin ver, se vuelve. ★ HEATONIST está ADENTRO de este mismo mercado (12-18:45): más de 100 salsas picantes para probar, con el lineup de Hot Ones. Si el sábado no llegan a la de Williamsburg, esta es la misma cata en menos metros.</t>
-        </is>
-      </c>
-      <c r="F135" s="37" t="inlineStr">
-        <is>
-          <t>Chelsea Market</t>
-        </is>
-      </c>
-      <c r="G135" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~7 min a pie · 0.5 km · estimado</t>
-        </is>
-      </c>
+          <t>A la Morgan: L desde 14 St-8 Av hasta Union Sq y 6 hasta 33 St, o A/C/E hasta 34 St-Penn y siete cuadras a pie (~30 min). Salir 16:25 deja margen para entrar 17:00 EN PUNTO.</t>
+        </is>
+      </c>
+      <c r="F135" s="37" t="inlineStr"/>
+      <c r="G135" s="40" t="inlineStr"/>
       <c r="H135" s="41" t="inlineStr"/>
       <c r="I135" s="41" t="inlineStr"/>
     </row>
     <row r="136" ht="30" customHeight="1">
       <c r="A136" s="35" t="n"/>
-      <c r="B136" s="36" t="inlineStr">
-        <is>
-          <t>16:25</t>
-        </is>
-      </c>
-      <c r="C136" s="37" t="inlineStr">
+      <c r="B136" s="42" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="D136" s="38" t="inlineStr">
+      <c r="C136" s="43" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="D136" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E136" s="39" t="inlineStr">
-        <is>
-          <t>A la Morgan: L desde 14 St-8 Av hasta Union Sq y 6 hasta 33 St, o A/C/E hasta 34 St-Penn y siete cuadras a pie (~30 min). Salir 16:25 deja margen para entrar 17:00 EN PUNTO.</t>
-        </is>
-      </c>
-      <c r="F136" s="37" t="inlineStr"/>
+      <c r="E136" s="45" t="inlineStr">
+        <is>
+          <t>★ MORGAN LIBRARY — GRATIS los viernes 17-20h: entrar 17:00 EN PUNTO y hacerla en una hora — la biblioteca son tres salas gloriosas (estanterías de nogal, la Biblia de Gutenberg): alcanza. RESERVA OBLIGATORIA, se libera el viernes 28 de agosto. Está a 8 min a pie de One Vanderbilt.</t>
+        </is>
+      </c>
+      <c r="F136" s="43" t="inlineStr">
+        <is>
+          <t>The Morgan Library &amp; Museum</t>
+        </is>
+      </c>
       <c r="G136" s="40" t="inlineStr"/>
       <c r="H136" s="41" t="inlineStr"/>
       <c r="I136" s="41" t="inlineStr"/>
     </row>
-    <row r="137" ht="30" customHeight="1">
+    <row r="137" ht="16" customHeight="1">
       <c r="A137" s="35" t="n"/>
-      <c r="B137" s="42" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C137" s="43" t="inlineStr">
+      <c r="B137" s="36" t="inlineStr">
         <is>
           <t>18:00</t>
         </is>
       </c>
-      <c r="D137" s="44" t="inlineStr">
+      <c r="C137" s="37" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="D137" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E137" s="45" t="inlineStr">
-        <is>
-          <t>★ MORGAN LIBRARY — GRATIS los viernes 17-20h: entrar 17:00 EN PUNTO y hacerla en una hora — la biblioteca son tres salas gloriosas (estanterías de nogal, la Biblia de Gutenberg): alcanza. RESERVA OBLIGATORIA, se libera el viernes 28 de agosto. Está a 8 min a pie de One Vanderbilt.</t>
-        </is>
-      </c>
-      <c r="F137" s="43" t="inlineStr">
-        <is>
-          <t>The Morgan Library &amp; Museum</t>
-        </is>
-      </c>
+      <c r="E137" s="39" t="inlineStr">
+        <is>
+          <t>Caminar las seis cuadras de la Morgan a One Vanderbilt (~8-10 min).</t>
+        </is>
+      </c>
+      <c r="F137" s="37" t="inlineStr"/>
       <c r="G137" s="40" t="inlineStr"/>
       <c r="H137" s="41" t="inlineStr"/>
       <c r="I137" s="41" t="inlineStr"/>
     </row>
-    <row r="138" ht="16" customHeight="1">
+    <row r="138" ht="30" customHeight="1">
       <c r="A138" s="35" t="n"/>
-      <c r="B138" s="36" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="C138" s="37" t="inlineStr">
+      <c r="B138" s="42" t="inlineStr">
         <is>
           <t>18:10</t>
         </is>
       </c>
-      <c r="D138" s="38" t="inlineStr">
+      <c r="C138" s="43" t="inlineStr">
+        <is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="D138" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E138" s="39" t="inlineStr">
-        <is>
-          <t>Caminar las seis cuadras de la Morgan a One Vanderbilt (~8-10 min).</t>
-        </is>
-      </c>
-      <c r="F138" s="37" t="inlineStr"/>
+      <c r="E138" s="45" t="inlineStr">
+        <is>
+          <t>★★ SUMMIT ONE VANDERBILT — EL ARCO COMPLETO: entrada 18:10 con luz, el atardecer ~19:21 multiplicado por los espejos infinitos de Kusama, y la noche encendida hasta ~20:15. Ticket ATARDECER $57-63 — es la franja que primero se agota: reservar YA. NO está en ningún pase.</t>
+        </is>
+      </c>
+      <c r="F138" s="43" t="inlineStr">
+        <is>
+          <t>SUMMIT One Vanderbilt</t>
+        </is>
+      </c>
       <c r="G138" s="40" t="inlineStr"/>
       <c r="H138" s="41" t="inlineStr"/>
       <c r="I138" s="41" t="inlineStr"/>
     </row>
     <row r="139" ht="30" customHeight="1">
       <c r="A139" s="35" t="n"/>
-      <c r="B139" s="42" t="inlineStr">
-        <is>
-          <t>18:10</t>
-        </is>
-      </c>
-      <c r="C139" s="43" t="inlineStr">
+      <c r="B139" s="36" t="inlineStr">
         <is>
           <t>20:20</t>
         </is>
       </c>
-      <c r="D139" s="44" t="inlineStr">
+      <c r="C139" s="37" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="D139" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E139" s="45" t="inlineStr">
-        <is>
-          <t>★★ SUMMIT ONE VANDERBILT — EL ARCO COMPLETO: entrada 18:10 con luz, el atardecer ~19:21 multiplicado por los espejos infinitos de Kusama, y la noche encendida hasta ~20:15. Ticket ATARDECER $57-63 — es la franja que primero se agota: reservar YA. NO está en ningún pase.</t>
-        </is>
-      </c>
-      <c r="F139" s="43" t="inlineStr">
-        <is>
-          <t>SUMMIT One Vanderbilt</t>
-        </is>
-      </c>
+      <c r="E139" s="39" t="inlineStr">
+        <is>
+          <t>Bajar AL VILLAGE PRIMERO y cenar allá: 4/5/6 o 7 hasta 14 St-Union Sq y 1 hasta Christopher St (~25 min). Cenar cerca de Grand Central y bajar después llega justo; hacerlo al revés deja margen.</t>
+        </is>
+      </c>
+      <c r="F139" s="37" t="inlineStr"/>
       <c r="G139" s="40" t="inlineStr"/>
       <c r="H139" s="41" t="inlineStr"/>
       <c r="I139" s="41" t="inlineStr"/>
@@ -36149,12 +36133,12 @@
       <c r="A140" s="35" t="n"/>
       <c r="B140" s="36" t="inlineStr">
         <is>
-          <t>20:20</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C140" s="37" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="D140" s="38" t="inlineStr">
@@ -36164,7 +36148,7 @@
       </c>
       <c r="E140" s="39" t="inlineStr">
         <is>
-          <t>Bajar AL VILLAGE PRIMERO y cenar allá: 4/5/6 o 7 hasta 14 St-Union Sq y 1 hasta Christopher St (~25 min). Cenar cerca de Grand Central y bajar después llega justo; hacerlo al revés deja margen.</t>
+          <t>Cena en el West Village, a cinco minutos del club. El Vanguard NO sirve NADA de comida (lo dicen así: 'ni un maní') y no se permite entrar comida: lo que no cenen ahora, no se cena. 40 minutos alcanzan.</t>
         </is>
       </c>
       <c r="F140" s="37" t="inlineStr"/>
@@ -36176,12 +36160,12 @@
       <c r="A141" s="35" t="n"/>
       <c r="B141" s="36" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>21:30</t>
         </is>
       </c>
       <c r="C141" s="37" t="inlineStr">
         <is>
-          <t>21:30</t>
+          <t>22:00</t>
         </is>
       </c>
       <c r="D141" s="38" t="inlineStr">
@@ -36191,7 +36175,7 @@
       </c>
       <c r="E141" s="39" t="inlineStr">
         <is>
-          <t>Cena en el West Village, a cinco minutos del club. El Vanguard NO sirve NADA de comida (lo dicen así: 'ni un maní') y no se permite entrar comida: lo que no cenen ahora, no se cena. 40 minutos alcanzan.</t>
+          <t>EN LA PUERTA DEL VANGUARD a las 21:30 EN PUNTO: el acomodo del segundo set arranca a esa hora y los asientos son POR ORDEN DE LLEGADA — la entrada es General Admission, no numerada. Con 123 asientos, los diez minutos de diferencia son estar frente al piano o contra la columna. El ticket lo dice: el acomodo tardío, con entrada o sin ella, queda a criterio del encargado.</t>
         </is>
       </c>
       <c r="F141" s="37" t="inlineStr"/>
@@ -36201,199 +36185,199 @@
     </row>
     <row r="142" ht="30" customHeight="1">
       <c r="A142" s="35" t="n"/>
-      <c r="B142" s="36" t="inlineStr">
-        <is>
-          <t>21:30</t>
-        </is>
-      </c>
-      <c r="C142" s="37" t="inlineStr">
+      <c r="B142" s="42" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D142" s="38" t="inlineStr">
+      <c r="C142" s="43" t="inlineStr"/>
+      <c r="D142" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E142" s="39" t="inlineStr">
-        <is>
-          <t>EN LA PUERTA DEL VANGUARD a las 21:30 EN PUNTO: el acomodo del segundo set arranca a esa hora y los asientos son POR ORDEN DE LLEGADA — la entrada es General Admission, no numerada. Con 123 asientos, los diez minutos de diferencia son estar frente al piano o contra la columna. El ticket lo dice: el acomodo tardío, con entrada o sin ella, queda a criterio del encargado.</t>
-        </is>
-      </c>
-      <c r="F142" s="37" t="inlineStr"/>
+      <c r="E142" s="45" t="inlineStr">
+        <is>
+          <t>★★ VILLAGE VANGUARD — JOHN PATITUCCI TRIO con Chris Potter y Brian Blade, SET DE LAS 22:00. Movido acá desde el martes para que vayan LOS DOS (pedido de Juan). El sótano triangular de 1935, 123 asientos, la acústica que grabó a Coltrane. ✔ ENTRADAS COMPRADAS el 26/8: 2 × General Admission $45 (#18741454 y #18741456), a nombre de Juan Pablo Garicoïts. Falta solo el mínimo de UNA CONSUMICIÓN por cabeza en la mesa (vale gaseosa, jugo o agua) — se paga ahí, aceptan tarjeta.</t>
+        </is>
+      </c>
+      <c r="F142" s="43" t="inlineStr">
+        <is>
+          <t>Village Vanguard</t>
+        </is>
+      </c>
       <c r="G142" s="40" t="inlineStr"/>
       <c r="H142" s="41" t="inlineStr"/>
       <c r="I142" s="41" t="inlineStr"/>
     </row>
-    <row r="143" ht="30" customHeight="1">
-      <c r="A143" s="35" t="n"/>
-      <c r="B143" s="42" t="inlineStr">
-        <is>
-          <t>22:00</t>
-        </is>
-      </c>
-      <c r="C143" s="43" t="inlineStr"/>
-      <c r="D143" s="44" t="inlineStr">
+    <row r="143" ht="32" customHeight="1">
+      <c r="A143" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  ⚠️ OJO CON LA MAÑANA, y es nuevo: Juan hizo el HIGH LINE, LITTLE ISLAND y el VESSEL el miércoles temprano, solo. Los tres siguen en el plan de hoy porque THAIS NO LOS VIO —el Vessel además lo tienen 2/2 y es imprescindible— así que sacarlos la perjudica a ella. Decidan en el momento: si Juan la acompaña igual, el High Line de día con ella es otro paseo y no se pierde nada; si prefieren no repetir, esa mañana libera de 9:15 a 13:00 y ahí entran las galerías de Chelsea con calma, o el Whitney, que hoy es gratis de 17 a 22 pero abre 10:30. // EL CANJE DE ESTA NOCHE: para meter el Vanguard con Thais, SALIÓ BILL'S PLACE. No hay otra noche donde entre (Bill Saxton toca solo viernes y sábado, y el sábado está tomado por Peter Luger + el play + el Café Wha). Con las entradas ya compradas y sin cambios ni transferencias, el canje quedó CERRADO: Bill's Place sale del viaje. // EL WHITNEY, con los números verificados el 27/8: gratis todos los viernes de 17:00 a 22:00 (normal $30), y hoy pasan por Meatpacking, que es donde está. Coincide barrio, día y franja. El problema es el reloj y es serio: la Morgan también es hoy 17:00-20:00 y el SUMMIT entra 18:10. Meter el Whitney obliga a recortar el High Line o a soltar la Morgan, que ustedes tienen en 2 y el Whitney en 'quizás'. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y hay que sacarlo antes. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y el Whitney ahora cierra los martes. SI ALGO SALIERA MAL con el acomodo (llegar tarde y que no haya lugar): Mezzrow o Smalls quedan a cuatro cuadras ($25 con bebida, Smalls tiene jam de madrugada los viernes desde la 1:00), o el Blue Note — el 4 y 5 de septiembre toca Chief Adjuah.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 8 · Sábado 05/09 · Brooklyn, Peter Luger, un PLAY y Café Wha hasta la madrugada  —  base: The Beacon  ·  Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="32" customHeight="1">
+      <c r="A146" s="34" t="inlineStr">
+        <is>
+          <t>La gran noche del viaje, rearmada a pedido: el musical SALIÓ y entraron un PLAY de Broadway a las 19:30 y el CAFÉ WHA a las 23:45 — el sótano del Village donde debutaron Dylan y Hendrix, con reserva gratis ya pedida por Eventbrite. La cena temprana en Peter Luger (17:00) ahora existe exactamente para esto: porterhouse → telón → medianoche de soul y funk. Frankel's sigue afuera (a un porterhouse no se llega con un pastrami encima) y Westlight sigue opcional. ⚠️ La noche termina ~1:15-1:30: el domingo no tiene NADA fijo hasta las 16:00.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="30" customHeight="1">
+      <c r="A147" s="35" t="n"/>
+      <c r="B147" s="36" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="C147" s="37" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D147" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E143" s="45" t="inlineStr">
-        <is>
-          <t>★★ VILLAGE VANGUARD — JOHN PATITUCCI TRIO con Chris Potter y Brian Blade, SET DE LAS 22:00. Movido acá desde el martes para que vayan LOS DOS (pedido de Juan). El sótano triangular de 1935, 123 asientos, la acústica que grabó a Coltrane. ✔ ENTRADAS COMPRADAS el 26/8: 2 × General Admission $45 (#18741454 y #18741456), a nombre de Juan Pablo Garicoïts. Falta solo el mínimo de UNA CONSUMICIÓN por cabeza en la mesa (vale gaseosa, jugo o agua) — se paga ahí, aceptan tarjeta.</t>
-        </is>
-      </c>
-      <c r="F143" s="43" t="inlineStr">
-        <is>
-          <t>Village Vanguard</t>
-        </is>
-      </c>
-      <c r="G143" s="40" t="inlineStr"/>
-      <c r="H143" s="41" t="inlineStr"/>
-      <c r="I143" s="41" t="inlineStr"/>
-    </row>
-    <row r="144" ht="32" customHeight="1">
-      <c r="A144" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  ⚠️ OJO CON LA MAÑANA, y es nuevo: Juan hizo el HIGH LINE, LITTLE ISLAND y el VESSEL el miércoles temprano, solo. Los tres siguen en el plan de hoy porque THAIS NO LOS VIO —el Vessel además lo tienen 2/2 y es imprescindible— así que sacarlos la perjudica a ella. Decidan en el momento: si Juan la acompaña igual, el High Line de día con ella es otro paseo y no se pierde nada; si prefieren no repetir, esa mañana libera de 9:15 a 13:00 y ahí entran las galerías de Chelsea con calma, o el Whitney, que hoy es gratis de 17 a 22 pero abre 10:30. // EL CANJE DE ESTA NOCHE: para meter el Vanguard con Thais, SALIÓ BILL'S PLACE. No hay otra noche donde entre (Bill Saxton toca solo viernes y sábado, y el sábado está tomado por Peter Luger + el play + el Café Wha). Con las entradas ya compradas y sin cambios ni transferencias, el canje quedó CERRADO: Bill's Place sale del viaje. // EL WHITNEY, con los números verificados el 27/8: gratis todos los viernes de 17:00 a 22:00 (normal $30), y hoy pasan por Meatpacking, que es donde está. Coincide barrio, día y franja. El problema es el reloj y es serio: la Morgan también es hoy 17:00-20:00 y el SUMMIT entra 18:10. Meter el Whitney obliga a recortar el High Line o a soltar la Morgan, que ustedes tienen en 2 y el Whitney en 'quizás'. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y hay que sacarlo antes. Si igual lo prefieren, el ticket gratis es OBLIGATORIO y el Whitney ahora cierra los martes. SI ALGO SALIERA MAL con el acomodo (llegar tarde y que no haya lugar): Mezzrow o Smalls quedan a cuatro cuadras ($25 con bebida, Smalls tiene jam de madrugada los viernes desde la 1:00), o el Blue Note — el 4 y 5 de septiembre toca Chief Adjuah.</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="22" customHeight="1">
-      <c r="A146" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 8 · Sábado 05/09 · Brooklyn, Peter Luger, un PLAY y Café Wha hasta la madrugada  —  base: The Beacon  ·  Ambos</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="32" customHeight="1">
-      <c r="A147" s="34" t="inlineStr">
-        <is>
-          <t>La gran noche del viaje, rearmada a pedido: el musical SALIÓ y entraron un PLAY de Broadway a las 19:30 y el CAFÉ WHA a las 23:45 — el sótano del Village donde debutaron Dylan y Hendrix, con reserva gratis ya pedida por Eventbrite. La cena temprana en Peter Luger (17:00) ahora existe exactamente para esto: porterhouse → telón → medianoche de soul y funk. Frankel's sigue afuera (a un porterhouse no se llega con un pastrami encima) y Westlight sigue opcional. ⚠️ La noche termina ~1:15-1:30: el domingo no tiene NADA fijo hasta las 16:00.</t>
-        </is>
-      </c>
+      <c r="E147" s="39" t="inlineStr">
+        <is>
+          <t>Salir 8:15: 1/2/3 desde 72 St + transbordo a A/C hasta High St son ~40-45 min REALES. Llegar temprano a DUMBO es la diferencia entre la foto y la cola de fotos.</t>
+        </is>
+      </c>
+      <c r="F147" s="37" t="inlineStr"/>
+      <c r="G147" s="40" t="inlineStr"/>
+      <c r="H147" s="41" t="inlineStr"/>
+      <c r="I147" s="41" t="inlineStr"/>
     </row>
     <row r="148" ht="30" customHeight="1">
       <c r="A148" s="35" t="n"/>
-      <c r="B148" s="36" t="inlineStr">
-        <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="C148" s="37" t="inlineStr">
+      <c r="B148" s="42" t="inlineStr">
         <is>
           <t>09:00</t>
         </is>
       </c>
-      <c r="D148" s="38" t="inlineStr">
+      <c r="C148" s="43" t="inlineStr">
+        <is>
+          <t>10:30</t>
+        </is>
+      </c>
+      <c r="D148" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E148" s="39" t="inlineStr">
-        <is>
-          <t>Salir 8:15: 1/2/3 desde 72 St + transbordo a A/C hasta High St son ~40-45 min REALES. Llegar temprano a DUMBO es la diferencia entre la foto y la cola de fotos.</t>
-        </is>
-      </c>
-      <c r="F148" s="37" t="inlineStr"/>
+      <c r="E148" s="45" t="inlineStr">
+        <is>
+          <t>★ Brooklyn Bridge Park y DUMBO — muelles reconvertidos con el skyline de Lower Manhattan de frente, y la foto del Manhattan Bridge encuadrado en Washington y Water.</t>
+        </is>
+      </c>
+      <c r="F148" s="43" t="inlineStr">
+        <is>
+          <t>Brooklyn Bridge Park</t>
+        </is>
+      </c>
       <c r="G148" s="40" t="inlineStr"/>
       <c r="H148" s="41" t="inlineStr"/>
       <c r="I148" s="41" t="inlineStr"/>
     </row>
-    <row r="149" ht="30" customHeight="1">
+    <row r="149" ht="16" customHeight="1">
       <c r="A149" s="35" t="n"/>
-      <c r="B149" s="42" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C149" s="43" t="inlineStr">
+      <c r="B149" s="36" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="D149" s="44" t="inlineStr">
+      <c r="C149" s="37" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="D149" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E149" s="45" t="inlineStr">
-        <is>
-          <t>★ Brooklyn Bridge Park y DUMBO — muelles reconvertidos con el skyline de Lower Manhattan de frente, y la foto del Manhattan Bridge encuadrado en Washington y Water.</t>
-        </is>
-      </c>
-      <c r="F149" s="43" t="inlineStr">
-        <is>
-          <t>Brooklyn Bridge Park</t>
-        </is>
-      </c>
-      <c r="G149" s="40" t="inlineStr"/>
+      <c r="E149" s="39" t="inlineStr">
+        <is>
+          <t>Brooklyn Heights Promenade — la postal clásica del skyline sobre el BQE.</t>
+        </is>
+      </c>
+      <c r="F149" s="37" t="inlineStr">
+        <is>
+          <t>Brooklyn Heights Promenade</t>
+        </is>
+      </c>
+      <c r="G149" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~8 min a pie · 0.6 km · estimado</t>
+        </is>
+      </c>
       <c r="H149" s="41" t="inlineStr"/>
       <c r="I149" s="41" t="inlineStr"/>
     </row>
-    <row r="150" ht="16" customHeight="1">
+    <row r="150" ht="30" customHeight="1">
       <c r="A150" s="35" t="n"/>
-      <c r="B150" s="36" t="inlineStr">
-        <is>
-          <t>10:30</t>
-        </is>
-      </c>
-      <c r="C150" s="37" t="inlineStr">
+      <c r="B150" s="42" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="D150" s="38" t="inlineStr">
+      <c r="C150" s="43" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="D150" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E150" s="39" t="inlineStr">
-        <is>
-          <t>Brooklyn Heights Promenade — la postal clásica del skyline sobre el BQE.</t>
-        </is>
-      </c>
-      <c r="F150" s="37" t="inlineStr">
-        <is>
-          <t>Brooklyn Heights Promenade</t>
-        </is>
-      </c>
-      <c r="G150" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~8 min a pie · 0.6 km · estimado</t>
-        </is>
-      </c>
+      <c r="E150" s="45" t="inlineStr">
+        <is>
+          <t>★ NEW YORK TRANSIT MUSEUM — una estación de subte clausurada de 1936 con 20 vagones históricos en las vías originales; se puede subir a todos. $10. Cierra lunes y martes, así que hoy es el día.</t>
+        </is>
+      </c>
+      <c r="F150" s="43" t="inlineStr">
+        <is>
+          <t>New York Transit Museum</t>
+        </is>
+      </c>
+      <c r="G150" s="40" t="inlineStr"/>
       <c r="H150" s="41" t="inlineStr"/>
       <c r="I150" s="41" t="inlineStr"/>
     </row>
-    <row r="151" ht="30" customHeight="1">
+    <row r="151" ht="16" customHeight="1">
       <c r="A151" s="35" t="n"/>
-      <c r="B151" s="42" t="inlineStr">
-        <is>
-          <t>11:15</t>
-        </is>
-      </c>
-      <c r="C151" s="43" t="inlineStr">
+      <c r="B151" s="36" t="inlineStr">
         <is>
           <t>12:45</t>
         </is>
       </c>
-      <c r="D151" s="44" t="inlineStr">
+      <c r="C151" s="37" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D151" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E151" s="45" t="inlineStr">
-        <is>
-          <t>★ NEW YORK TRANSIT MUSEUM — una estación de subte clausurada de 1936 con 20 vagones históricos en las vías originales; se puede subir a todos. $10. Cierra lunes y martes, así que hoy es el día.</t>
-        </is>
-      </c>
-      <c r="F151" s="43" t="inlineStr">
-        <is>
-          <t>New York Transit Museum</t>
-        </is>
-      </c>
+      <c r="E151" s="39" t="inlineStr">
+        <is>
+          <t>Almuerzo en Downtown Brooklyn.</t>
+        </is>
+      </c>
+      <c r="F151" s="37" t="inlineStr"/>
       <c r="G151" s="40" t="inlineStr"/>
       <c r="H151" s="41" t="inlineStr"/>
       <c r="I151" s="41" t="inlineStr"/>
@@ -36402,12 +36386,12 @@
       <c r="A152" s="35" t="n"/>
       <c r="B152" s="36" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="C152" s="37" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>14:15</t>
         </is>
       </c>
       <c r="D152" s="38" t="inlineStr">
@@ -36417,7 +36401,7 @@
       </c>
       <c r="E152" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en Downtown Brooklyn.</t>
+          <t>Subte a Williamsburg.</t>
         </is>
       </c>
       <c r="F152" s="37" t="inlineStr"/>
@@ -36425,74 +36409,82 @@
       <c r="H152" s="41" t="inlineStr"/>
       <c r="I152" s="41" t="inlineStr"/>
     </row>
-    <row r="153" ht="16" customHeight="1">
+    <row r="153" ht="30" customHeight="1">
       <c r="A153" s="35" t="n"/>
-      <c r="B153" s="36" t="inlineStr">
-        <is>
-          <t>13:45</t>
-        </is>
-      </c>
-      <c r="C153" s="37" t="inlineStr">
+      <c r="B153" s="42" t="inlineStr">
         <is>
           <t>14:15</t>
         </is>
       </c>
-      <c r="D153" s="38" t="inlineStr">
+      <c r="C153" s="43" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D153" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E153" s="39" t="inlineStr">
-        <is>
-          <t>Subte a Williamsburg.</t>
-        </is>
-      </c>
-      <c r="F153" s="37" t="inlineStr"/>
+      <c r="E153" s="45" t="inlineStr">
+        <is>
+          <t>★ Domino Park — ex refinería de azúcar; el paseo elevado pasa entre la maquinaria industrial conservada, con el Williamsburg Bridge y Midtown enfrente.</t>
+        </is>
+      </c>
+      <c r="F153" s="43" t="inlineStr">
+        <is>
+          <t>Domino Park</t>
+        </is>
+      </c>
       <c r="G153" s="40" t="inlineStr"/>
       <c r="H153" s="41" t="inlineStr"/>
       <c r="I153" s="41" t="inlineStr"/>
     </row>
     <row r="154" ht="30" customHeight="1">
       <c r="A154" s="35" t="n"/>
-      <c r="B154" s="42" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="C154" s="43" t="inlineStr">
+      <c r="B154" s="36" t="inlineStr">
         <is>
           <t>15:15</t>
         </is>
       </c>
-      <c r="D154" s="44" t="inlineStr">
+      <c r="C154" s="37" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D154" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E154" s="45" t="inlineStr">
-        <is>
-          <t>★ Domino Park — ex refinería de azúcar; el paseo elevado pasa entre la maquinaria industrial conservada, con el Williamsburg Bridge y Midtown enfrente.</t>
-        </is>
-      </c>
-      <c r="F154" s="43" t="inlineStr">
-        <is>
-          <t>Domino Park</t>
-        </is>
-      </c>
-      <c r="G154" s="40" t="inlineStr"/>
+      <c r="E154" s="39" t="inlineStr">
+        <is>
+          <t>Paseo por Williamsburg: Bedford Ave, disquerías y vintage. ★ ACÁ ENTRA HEATONIST (121 Wythe Ave, a una cuadra de Bedford): la tienda insignia de salsas picantes, con más de 100 para probar en el local y el lineup completo de Hot Ones. Abre 12-19 todos los días, así que a esta hora está abierta y les queda de camino al Williamsburg Bridge. OPCIONAL si quieren la panorámica: Westlight (piso 22, sin cover, un trago) — lo bajaron a 'quizás'. NO comer nada: lo que viene lo merece.</t>
+        </is>
+      </c>
+      <c r="F154" s="37" t="inlineStr">
+        <is>
+          <t>HEATONIST Williamsburg</t>
+        </is>
+      </c>
+      <c r="G154" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~20 min a pie (1.2 km) o 🚇 ~15 min · estimado</t>
+        </is>
+      </c>
       <c r="H154" s="41" t="inlineStr"/>
       <c r="I154" s="41" t="inlineStr"/>
     </row>
-    <row r="155" ht="30" customHeight="1">
+    <row r="155" ht="16" customHeight="1">
       <c r="A155" s="35" t="n"/>
       <c r="B155" s="36" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>16:45</t>
         </is>
       </c>
       <c r="C155" s="37" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="D155" s="38" t="inlineStr">
@@ -36502,148 +36494,140 @@
       </c>
       <c r="E155" s="39" t="inlineStr">
         <is>
-          <t>Paseo por Williamsburg: Bedford Ave, disquerías y vintage. ★ ACÁ ENTRA HEATONIST (121 Wythe Ave, a una cuadra de Bedford): la tienda insignia de salsas picantes, con más de 100 para probar en el local y el lineup completo de Hot Ones. Abre 12-19 todos los días, así que a esta hora está abierta y les queda de camino al Williamsburg Bridge. OPCIONAL si quieren la panorámica: Westlight (piso 22, sin cover, un trago) — lo bajaron a 'quizás'. NO comer nada: lo que viene lo merece.</t>
-        </is>
-      </c>
-      <c r="F155" s="37" t="inlineStr">
-        <is>
-          <t>HEATONIST Williamsburg</t>
-        </is>
-      </c>
-      <c r="G155" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~20 min a pie (1.2 km) o 🚇 ~15 min · estimado</t>
-        </is>
-      </c>
+          <t>Caminar por Bedford/Driggs hasta el pie del Williamsburg Bridge (~15 min).</t>
+        </is>
+      </c>
+      <c r="F155" s="37" t="inlineStr"/>
+      <c r="G155" s="40" t="inlineStr"/>
       <c r="H155" s="41" t="inlineStr"/>
       <c r="I155" s="41" t="inlineStr"/>
     </row>
-    <row r="156" ht="16" customHeight="1">
+    <row r="156" ht="30" customHeight="1">
       <c r="A156" s="35" t="n"/>
-      <c r="B156" s="36" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="C156" s="37" t="inlineStr">
+      <c r="B156" s="42" t="inlineStr">
         <is>
           <t>17:00</t>
         </is>
       </c>
-      <c r="D156" s="38" t="inlineStr">
+      <c r="C156" s="43" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="D156" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E156" s="39" t="inlineStr">
-        <is>
-          <t>Caminar por Bedford/Driggs hasta el pie del Williamsburg Bridge (~15 min).</t>
-        </is>
-      </c>
-      <c r="F156" s="37" t="inlineStr"/>
+      <c r="E156" s="45" t="inlineStr">
+        <is>
+          <t>★★ PETER LUGER (178 Broadway) — el porterhouse for two de 1887, dry-aged en el sótano, con la tocineta gruesa de entrada. ~$160-200 los dos con sides y propina. ⚠️ SIN TARJETAS DE CRÉDITO: efectivo, débito US o cheque — llevar cash. Cena temprana a propósito: el teatro espera. RESERVA EN RESY YA.</t>
+        </is>
+      </c>
+      <c r="F156" s="43" t="inlineStr">
+        <is>
+          <t>Peter Luger Steak House</t>
+        </is>
+      </c>
       <c r="G156" s="40" t="inlineStr"/>
       <c r="H156" s="41" t="inlineStr"/>
       <c r="I156" s="41" t="inlineStr"/>
     </row>
     <row r="157" ht="30" customHeight="1">
       <c r="A157" s="35" t="n"/>
-      <c r="B157" s="42" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="C157" s="43" t="inlineStr">
+      <c r="B157" s="36" t="inlineStr">
         <is>
           <t>18:45</t>
         </is>
       </c>
-      <c r="D157" s="44" t="inlineStr">
+      <c r="C157" s="37" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="D157" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E157" s="45" t="inlineStr">
-        <is>
-          <t>★★ PETER LUGER (178 Broadway) — el porterhouse for two de 1887, dry-aged en el sótano, con la tocineta gruesa de entrada. ~$160-200 los dos con sides y propina. ⚠️ SIN TARJETAS DE CRÉDITO: efectivo, débito US o cheque — llevar cash. Cena temprana a propósito: el teatro espera. RESERVA EN RESY YA.</t>
-        </is>
-      </c>
-      <c r="F157" s="43" t="inlineStr">
-        <is>
-          <t>Peter Luger Steak House</t>
-        </is>
-      </c>
+      <c r="E157" s="39" t="inlineStr">
+        <is>
+          <t>A la zona de teatros: subte J desde Marcy Av hasta Essex St y F hasta 42 St-Bryant Park (~35 min con transbordo), o directamente Uber al teatro (~20-25 min, $25-35 — un sábado a la noche el puente puede estar cargado).</t>
+        </is>
+      </c>
+      <c r="F157" s="37" t="inlineStr"/>
       <c r="G157" s="40" t="inlineStr"/>
       <c r="H157" s="41" t="inlineStr"/>
       <c r="I157" s="41" t="inlineStr"/>
     </row>
     <row r="158" ht="30" customHeight="1">
       <c r="A158" s="35" t="n"/>
-      <c r="B158" s="36" t="inlineStr">
-        <is>
-          <t>18:45</t>
-        </is>
-      </c>
-      <c r="C158" s="37" t="inlineStr">
+      <c r="B158" s="42" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="D158" s="38" t="inlineStr">
+      <c r="C158" s="43" t="inlineStr">
+        <is>
+          <t>22:00</t>
+        </is>
+      </c>
+      <c r="D158" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E158" s="39" t="inlineStr">
-        <is>
-          <t>A la zona de teatros: subte J desde Marcy Av hasta Essex St y F hasta 42 St-Bryant Park (~35 min con transbordo), o directamente Uber al teatro (~20-25 min, $25-35 — un sábado a la noche el puente puede estar cargado).</t>
-        </is>
-      </c>
-      <c r="F158" s="37" t="inlineStr"/>
+      <c r="E158" s="45" t="inlineStr">
+        <is>
+          <t>★★ PLAY DE BROADWAY — mi recomendación: STRANGER THINGS: THE FIRST SHADOW (Marquis, desde ~$76): la maquinaria escénica que ganó el Tony — para quien viene de Mercer Labs, el mismo músculo llevado al teatro. Alternativas esa semana: Harry Potter and the Cursed Child, Paranormal Activity, The Imaginary Invalid. COMPRA FIRME esta semana y verificar el horario real de la función (19:00/19:30/20:00): tiene que terminar ~22:00 para lo que sigue.</t>
+        </is>
+      </c>
+      <c r="F158" s="43" t="inlineStr">
+        <is>
+          <t>Stranger Things: The First Shadow (play)</t>
+        </is>
+      </c>
       <c r="G158" s="40" t="inlineStr"/>
       <c r="H158" s="41" t="inlineStr"/>
       <c r="I158" s="41" t="inlineStr"/>
     </row>
-    <row r="159" ht="30" customHeight="1">
+    <row r="159" ht="16" customHeight="1">
       <c r="A159" s="35" t="n"/>
-      <c r="B159" s="42" t="inlineStr">
-        <is>
-          <t>19:30</t>
-        </is>
-      </c>
-      <c r="C159" s="43" t="inlineStr">
+      <c r="B159" s="36" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="D159" s="44" t="inlineStr">
+      <c r="C159" s="37" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="D159" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E159" s="45" t="inlineStr">
-        <is>
-          <t>★★ PLAY DE BROADWAY — mi recomendación: STRANGER THINGS: THE FIRST SHADOW (Marquis, desde ~$76): la maquinaria escénica que ganó el Tony — para quien viene de Mercer Labs, el mismo músculo llevado al teatro. Alternativas esa semana: Harry Potter and the Cursed Child, Paranormal Activity, The Imaginary Invalid. COMPRA FIRME esta semana y verificar el horario real de la función (19:00/19:30/20:00): tiene que terminar ~22:00 para lo que sigue.</t>
-        </is>
-      </c>
-      <c r="F159" s="43" t="inlineStr">
-        <is>
-          <t>Stranger Things: The First Shadow (play)</t>
-        </is>
-      </c>
+      <c r="E159" s="39" t="inlineStr">
+        <is>
+          <t>Subte 1 desde Times Sq hasta Christopher St (~15 min) y caminar al corazón del Village.</t>
+        </is>
+      </c>
+      <c r="F159" s="37" t="inlineStr"/>
       <c r="G159" s="40" t="inlineStr"/>
       <c r="H159" s="41" t="inlineStr"/>
       <c r="I159" s="41" t="inlineStr"/>
     </row>
-    <row r="160" ht="16" customHeight="1">
+    <row r="160" ht="30" customHeight="1">
       <c r="A160" s="35" t="n"/>
       <c r="B160" s="36" t="inlineStr">
         <is>
-          <t>22:00</t>
+          <t>22:30</t>
         </is>
       </c>
       <c r="C160" s="37" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>23:15</t>
         </is>
       </c>
       <c r="D160" s="38" t="inlineStr">
@@ -36653,7 +36637,7 @@
       </c>
       <c r="E160" s="39" t="inlineStr">
         <is>
-          <t>Subte 1 desde Times Sq hasta Christopher St (~15 min) y caminar al corazón del Village.</t>
+          <t>Paseo sin apuro por Bleecker y MacDougal — la esquina folk de los 60s de noche, un café o un trago corto. El único objetivo real: estar en la puerta del Wha a las 23:10.</t>
         </is>
       </c>
       <c r="F160" s="37" t="inlineStr"/>
@@ -36663,102 +36647,106 @@
     </row>
     <row r="161" ht="30" customHeight="1">
       <c r="A161" s="35" t="n"/>
-      <c r="B161" s="36" t="inlineStr">
-        <is>
-          <t>22:30</t>
-        </is>
-      </c>
-      <c r="C161" s="37" t="inlineStr">
+      <c r="B161" s="42" t="inlineStr">
         <is>
           <t>23:15</t>
         </is>
       </c>
-      <c r="D161" s="38" t="inlineStr">
+      <c r="C161" s="43" t="inlineStr"/>
+      <c r="D161" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E161" s="39" t="inlineStr">
-        <is>
-          <t>Paseo sin apuro por Bleecker y MacDougal — la esquina folk de los 60s de noche, un café o un trago corto. El único objetivo real: estar en la puerta del Wha a las 23:10.</t>
-        </is>
-      </c>
-      <c r="F161" s="37" t="inlineStr"/>
+      <c r="E161" s="45" t="inlineStr">
+        <is>
+          <t>★★ CAFÉ WHA — LLEGAR 23:10-23:15: la reserva de Eventbrite NO garantiza admisión y a las 23:30 EN PUNTO liberan los asientos vacíos al standby. TODOS los de la reserva presentes. Set 2 de la house band 23:45-~1:15: soul y funk a máquina en el sótano donde debutaron Dylan, Hendrix y Springsteen. $20 por cabeza van a la cuenta + consumo. Vuelta: subte 1 Christopher St → 72 St (~25 min) o taxi.</t>
+        </is>
+      </c>
+      <c r="F161" s="43" t="inlineStr">
+        <is>
+          <t>Cafe Wha?</t>
+        </is>
+      </c>
       <c r="G161" s="40" t="inlineStr"/>
       <c r="H161" s="41" t="inlineStr"/>
       <c r="I161" s="41" t="inlineStr"/>
     </row>
-    <row r="162" ht="30" customHeight="1">
-      <c r="A162" s="35" t="n"/>
-      <c r="B162" s="42" t="inlineStr">
-        <is>
-          <t>23:15</t>
-        </is>
-      </c>
-      <c r="C162" s="43" t="inlineStr"/>
-      <c r="D162" s="44" t="inlineStr">
+    <row r="162" ht="32" customHeight="1">
+      <c r="A162" s="46" t="inlineStr">
+        <is>
+          <t>ALTERNATIVA / OJO:  SOBRE PETER LUGER: la mesa de las 17:00 es la realista — y ahora es la única que funciona: el play manda. PLAN B si no hay mesa: correr Peter Luger al ALMUERZO del mismo día (12:45). // SI EL CANSANCIO GANA A LAS 22:00: el Café Wha es la pieza sacrificable — la reserva es gratis y no penaliza no ir; el play, pagado, no. // Sigue afuera: Bar LunÀtico y Barbès (Bed-Stuy/Park Slope), sin noche posible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="22" customHeight="1">
+      <c r="A164" s="33" t="inlineStr">
+        <is>
+          <t>DÍA 9 · Domingo 06/09 · Checkout, Central Park, Roosevelt Island, MoMA PS1 y vuelo  —  base: The Beacon (checkout) → EWR  ·  Ambos</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="32" customHeight="1">
+      <c r="A165" s="34" t="inlineStr">
+        <is>
+          <t>El día arranca con el CHECKOUT de The Beacon: hacerlo temprano y dejar las valijas en el bell desk libera el día entero. El vuelo sale 23:40, así que hay margen — pero es el domingo del fin de semana largo de Labor Day, la noche de mayor tráfico del año, y EWR va a estar cargado. Por eso todo queda cerca y se sale con 2h45 de anticipación. EL CAMBIO DEL ÚLTIMO DÍA: entra MOMA PS1 y sale el Guggenheim. Se verificó el 27/8 que la rotonda del Guggenheim está cerrada hasta el 17/9 —no se camina la rampa, que es la razón para ir— y PS1 resultó ser gratis, abierto hasta las 18 los domingos, a 1,2 km de Roosevelt Island y con «Greater New York 2026» en pie hasta el 7/9. Era el último imprescindible que quedaba afuera del viaje. El Guggenheim queda escrito como alternativa por si cambian de idea.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="30" customHeight="1">
+      <c r="A166" s="35" t="n"/>
+      <c r="B166" s="36" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C166" s="37" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="D166" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E162" s="45" t="inlineStr">
-        <is>
-          <t>★★ CAFÉ WHA — LLEGAR 23:10-23:15: la reserva de Eventbrite NO garantiza admisión y a las 23:30 EN PUNTO liberan los asientos vacíos al standby. TODOS los de la reserva presentes. Set 2 de la house band 23:45-~1:15: soul y funk a máquina en el sótano donde debutaron Dylan, Hendrix y Springsteen. $20 por cabeza van a la cuenta + consumo. Vuelta: subte 1 Christopher St → 72 St (~25 min) o taxi.</t>
-        </is>
-      </c>
-      <c r="F162" s="43" t="inlineStr">
-        <is>
-          <t>Cafe Wha?</t>
-        </is>
-      </c>
-      <c r="G162" s="40" t="inlineStr"/>
-      <c r="H162" s="41" t="inlineStr"/>
-      <c r="I162" s="41" t="inlineStr"/>
-    </row>
-    <row r="163" ht="32" customHeight="1">
-      <c r="A163" s="46" t="inlineStr">
-        <is>
-          <t>ALTERNATIVA / OJO:  SOBRE PETER LUGER: la mesa de las 17:00 es la realista — y ahora es la única que funciona: el play manda. PLAN B si no hay mesa: correr Peter Luger al ALMUERZO del mismo día (12:45). // SI EL CANSANCIO GANA A LAS 22:00: el Café Wha es la pieza sacrificable — la reserva es gratis y no penaliza no ir; el play, pagado, no. // Sigue afuera: Bar LunÀtico y Barbès (Bed-Stuy/Park Slope), sin noche posible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="165" ht="22" customHeight="1">
-      <c r="A165" s="33" t="inlineStr">
-        <is>
-          <t>DÍA 9 · Domingo 06/09 · Checkout, Central Park, Roosevelt Island, MoMA PS1 y vuelo  —  base: The Beacon (checkout) → EWR  ·  Ambos</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" ht="32" customHeight="1">
-      <c r="A166" s="34" t="inlineStr">
-        <is>
-          <t>El día arranca con el CHECKOUT de The Beacon: hacerlo temprano y dejar las valijas en el bell desk libera el día entero. El vuelo sale 23:40, así que hay margen — pero es el domingo del fin de semana largo de Labor Day, la noche de mayor tráfico del año, y EWR va a estar cargado. Por eso todo queda cerca y se sale con 2h45 de anticipación. EL CAMBIO DEL ÚLTIMO DÍA: entra MOMA PS1 y sale el Guggenheim. Se verificó el 27/8 que la rotonda del Guggenheim está cerrada hasta el 17/9 —no se camina la rampa, que es la razón para ir— y PS1 resultó ser gratis, abierto hasta las 18 los domingos, a 1,2 km de Roosevelt Island y con «Greater New York 2026» en pie hasta el 7/9. Era el último imprescindible que quedaba afuera del viaje. El Guggenheim queda escrito como alternativa por si cambian de idea.</t>
-        </is>
-      </c>
+      <c r="E166" s="39" t="inlineStr">
+        <is>
+          <t>Desayuno SIN despertador temprano: anoche terminó ~1:30 en el Village y lo único con hora fija hoy es el PS1, que cierra a las 18:00. Dormir un poco más está permitido.</t>
+        </is>
+      </c>
+      <c r="F166" s="37" t="inlineStr"/>
+      <c r="G166" s="40" t="inlineStr"/>
+      <c r="H166" s="41" t="inlineStr"/>
+      <c r="I166" s="41" t="inlineStr"/>
     </row>
     <row r="167" ht="30" customHeight="1">
       <c r="A167" s="35" t="n"/>
-      <c r="B167" s="36" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="C167" s="37" t="inlineStr">
+      <c r="B167" s="42" t="inlineStr">
         <is>
           <t>09:45</t>
         </is>
       </c>
-      <c r="D167" s="38" t="inlineStr">
+      <c r="C167" s="43" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="D167" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E167" s="39" t="inlineStr">
-        <is>
-          <t>Desayuno SIN despertador temprano: anoche terminó ~1:30 en el Village y lo único con hora fija hoy es el PS1, que cierra a las 18:00. Dormir un poco más está permitido.</t>
-        </is>
-      </c>
-      <c r="F167" s="37" t="inlineStr"/>
+      <c r="E167" s="45" t="inlineStr">
+        <is>
+          <t>★ CHECKOUT de The Beacon y dejar las valijas en el bell desk. El checkout formal suele ser 11:00-12:00, pero hacerlo antes libera el día.</t>
+        </is>
+      </c>
+      <c r="F167" s="43" t="inlineStr">
+        <is>
+          <t>Hotel The Beacon (3-6 sep)</t>
+        </is>
+      </c>
       <c r="G167" s="40" t="inlineStr"/>
       <c r="H167" s="41" t="inlineStr"/>
       <c r="I167" s="41" t="inlineStr"/>
@@ -36767,12 +36755,12 @@
       <c r="A168" s="35" t="n"/>
       <c r="B168" s="42" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="C168" s="43" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D168" s="44" t="inlineStr">
@@ -36782,63 +36770,59 @@
       </c>
       <c r="E168" s="45" t="inlineStr">
         <is>
-          <t>★ CHECKOUT de The Beacon y dejar las valijas en el bell desk. El checkout formal suele ser 11:00-12:00, pero hacerlo antes libera el día.</t>
+          <t>★ CENTRAL PARK cruzando de oeste a este: Bethesda Terrace, el Ramble, Bow Bridge. Se entra por la 72 desde Broadway, a tres cuadras del hotel.</t>
         </is>
       </c>
       <c r="F168" s="43" t="inlineStr">
         <is>
-          <t>Hotel The Beacon (3-6 sep)</t>
-        </is>
-      </c>
-      <c r="G168" s="40" t="inlineStr"/>
+          <t>Central Park</t>
+        </is>
+      </c>
+      <c r="G168" s="40" t="inlineStr">
+        <is>
+          <t>🚶 ~20 min a pie (1.5 km) o 🚇 ~15 min · estimado</t>
+        </is>
+      </c>
       <c r="H168" s="41" t="inlineStr"/>
       <c r="I168" s="41" t="inlineStr"/>
     </row>
-    <row r="169" ht="30" customHeight="1">
+    <row r="169" ht="16" customHeight="1">
       <c r="A169" s="35" t="n"/>
-      <c r="B169" s="42" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="C169" s="43" t="inlineStr">
+      <c r="B169" s="36" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="D169" s="44" t="inlineStr">
+      <c r="C169" s="37" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D169" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E169" s="45" t="inlineStr">
-        <is>
-          <t>★ CENTRAL PARK cruzando de oeste a este: Bethesda Terrace, el Ramble, Bow Bridge. Se entra por la 72 desde Broadway, a tres cuadras del hotel.</t>
-        </is>
-      </c>
-      <c r="F169" s="43" t="inlineStr">
-        <is>
-          <t>Central Park</t>
-        </is>
-      </c>
-      <c r="G169" s="40" t="inlineStr">
-        <is>
-          <t>🚶 ~20 min a pie (1.5 km) o 🚇 ~15 min · estimado</t>
-        </is>
-      </c>
+      <c r="E169" s="39" t="inlineStr">
+        <is>
+          <t>Almuerzo en el Upper East Side, saliendo del parque por la Quinta.</t>
+        </is>
+      </c>
+      <c r="F169" s="37" t="inlineStr"/>
+      <c r="G169" s="40" t="inlineStr"/>
       <c r="H169" s="41" t="inlineStr"/>
       <c r="I169" s="41" t="inlineStr"/>
     </row>
-    <row r="170" ht="16" customHeight="1">
+    <row r="170" ht="30" customHeight="1">
       <c r="A170" s="35" t="n"/>
       <c r="B170" s="36" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="C170" s="37" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="D170" s="38" t="inlineStr">
@@ -36848,7 +36832,7 @@
       </c>
       <c r="E170" s="39" t="inlineStr">
         <is>
-          <t>Almuerzo en el Upper East Side, saliendo del parque por la Quinta.</t>
+          <t>Bajar a 59 St y 2ª Av: subte 6 desde 68 St-Hunter College (el 4/5 exprés NO para ahí), o caminando por la Quinta si el día está lindo.</t>
         </is>
       </c>
       <c r="F170" s="37" t="inlineStr"/>
@@ -36858,56 +36842,60 @@
     </row>
     <row r="171" ht="30" customHeight="1">
       <c r="A171" s="35" t="n"/>
-      <c r="B171" s="36" t="inlineStr">
-        <is>
-          <t>13:30</t>
-        </is>
-      </c>
-      <c r="C171" s="37" t="inlineStr">
+      <c r="B171" s="42" t="inlineStr">
         <is>
           <t>13:50</t>
         </is>
       </c>
-      <c r="D171" s="38" t="inlineStr">
+      <c r="C171" s="43" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="D171" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E171" s="39" t="inlineStr">
-        <is>
-          <t>Bajar a 59 St y 2ª Av: subte 6 desde 68 St-Hunter College (el 4/5 exprés NO para ahí), o caminando por la Quinta si el día está lindo.</t>
-        </is>
-      </c>
-      <c r="F171" s="37" t="inlineStr"/>
+      <c r="E171" s="45" t="inlineStr">
+        <is>
+          <t>★ ROOSEVELT ISLAND TRAMWAY ($3, OMNY) — cruza el East River a 76 metros de altura con el Queensboro Bridge al lado. Es la vista de $50 por el precio de un viaje de subte.</t>
+        </is>
+      </c>
+      <c r="F171" s="43" t="inlineStr">
+        <is>
+          <t>Roosevelt Island Tramway</t>
+        </is>
+      </c>
       <c r="G171" s="40" t="inlineStr"/>
       <c r="H171" s="41" t="inlineStr"/>
       <c r="I171" s="41" t="inlineStr"/>
     </row>
     <row r="172" ht="30" customHeight="1">
       <c r="A172" s="35" t="n"/>
-      <c r="B172" s="42" t="inlineStr">
-        <is>
-          <t>13:50</t>
-        </is>
-      </c>
-      <c r="C172" s="43" t="inlineStr">
+      <c r="B172" s="36" t="inlineStr">
         <is>
           <t>14:25</t>
         </is>
       </c>
-      <c r="D172" s="44" t="inlineStr">
+      <c r="C172" s="37" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="D172" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E172" s="45" t="inlineStr">
-        <is>
-          <t>★ ROOSEVELT ISLAND TRAMWAY ($3, OMNY) — cruza el East River a 76 metros de altura con el Queensboro Bridge al lado. Es la vista de $50 por el precio de un viaje de subte.</t>
-        </is>
-      </c>
-      <c r="F172" s="43" t="inlineStr">
-        <is>
-          <t>Roosevelt Island Tramway</t>
+      <c r="E172" s="39" t="inlineStr">
+        <is>
+          <t>FDR Four Freedoms Park — del teleférico son ~20 min a pie por el borde del río. La última obra de Louis Kahn: granito, plátanos y una sala abierta al río apuntando a Manhattan. Gratis y vacía. Se pasa por las ruinas del Smallpox Hospital.</t>
+        </is>
+      </c>
+      <c r="F172" s="37" t="inlineStr">
+        <is>
+          <t>FDR Four Freedoms Park</t>
         </is>
       </c>
       <c r="G172" s="40" t="inlineStr"/>
@@ -36918,12 +36906,12 @@
       <c r="A173" s="35" t="n"/>
       <c r="B173" s="36" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C173" s="37" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D173" s="38" t="inlineStr">
@@ -36933,14 +36921,10 @@
       </c>
       <c r="E173" s="39" t="inlineStr">
         <is>
-          <t>FDR Four Freedoms Park — del teleférico son ~20 min a pie por el borde del río. La última obra de Louis Kahn: granito, plátanos y una sala abierta al río apuntando a Manhattan. Gratis y vacía. Se pasa por las ruinas del Smallpox Hospital.</t>
-        </is>
-      </c>
-      <c r="F173" s="37" t="inlineStr">
-        <is>
-          <t>FDR Four Freedoms Park</t>
-        </is>
-      </c>
+          <t>SALIR 15:05 de Four Freedoms Park y caminar 15 min al norte por el borde del río hasta la ESTACIÓN DEL F, que está en el medio de la isla (Main St y Roosevelt Island Bridge). Hoy NO se vuelve en teleférico: se cruza a Queens por abajo.</t>
+        </is>
+      </c>
+      <c r="F173" s="37" t="inlineStr"/>
       <c r="G173" s="40" t="inlineStr"/>
       <c r="H173" s="41" t="inlineStr"/>
       <c r="I173" s="41" t="inlineStr"/>
@@ -36949,12 +36933,12 @@
       <c r="A174" s="35" t="n"/>
       <c r="B174" s="36" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="C174" s="37" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="D174" s="38" t="inlineStr">
@@ -36964,7 +36948,7 @@
       </c>
       <c r="E174" s="39" t="inlineStr">
         <is>
-          <t>SALIR 15:05 de Four Freedoms Park y caminar 15 min al norte por el borde del río hasta la ESTACIÓN DEL F, que está en el medio de la isla (Main St y Roosevelt Island Bridge). Hoy NO se vuelve en teleférico: se cruza a Queens por abajo.</t>
+          <t>Subte F, UNA parada: Roosevelt Island → 21 St-Queensbridge (~4 min). Salir y caminar 12-15 min al sur por 21st St / Jackson Ave.</t>
         </is>
       </c>
       <c r="F174" s="37" t="inlineStr"/>
@@ -36974,58 +36958,58 @@
     </row>
     <row r="175" ht="30" customHeight="1">
       <c r="A175" s="35" t="n"/>
-      <c r="B175" s="36" t="inlineStr">
-        <is>
-          <t>15:30</t>
-        </is>
-      </c>
-      <c r="C175" s="37" t="inlineStr">
+      <c r="B175" s="42" t="inlineStr">
         <is>
           <t>15:45</t>
         </is>
       </c>
-      <c r="D175" s="38" t="inlineStr">
+      <c r="C175" s="43" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="D175" s="44" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E175" s="39" t="inlineStr">
-        <is>
-          <t>Subte F, UNA parada: Roosevelt Island → 21 St-Queensbridge (~4 min). Salir y caminar 12-15 min al sur por 21st St / Jackson Ave.</t>
-        </is>
-      </c>
-      <c r="F175" s="37" t="inlineStr"/>
+      <c r="E175" s="45" t="inlineStr">
+        <is>
+          <t>★★ MOMA PS1 — el último imprescindible del viaje, y entra gratis. Escuela pública de 1892 reconvertida en el laboratorio del MoMA: lo que no se anima a mostrar en la Quinta Avenida. VERIFICADO el 27/8: ENTRADA GRATUITA para todos, abre domingos 12:00-18:00, y «Greater New York 2026» —la encuesta insignia de la casa, que se hace cada cinco años— sigue en pie hasta el 7 de septiembre, o sea que la agarran por un día. Más el Courtyard Commission de Precious Okoyomon al aire libre. Dos horas holgadas hasta las 17:45.</t>
+        </is>
+      </c>
+      <c r="F175" s="43" t="inlineStr">
+        <is>
+          <t>MoMA PS1</t>
+        </is>
+      </c>
       <c r="G175" s="40" t="inlineStr"/>
       <c r="H175" s="41" t="inlineStr"/>
       <c r="I175" s="41" t="inlineStr"/>
     </row>
     <row r="176" ht="30" customHeight="1">
       <c r="A176" s="35" t="n"/>
-      <c r="B176" s="42" t="inlineStr">
-        <is>
-          <t>15:45</t>
-        </is>
-      </c>
-      <c r="C176" s="43" t="inlineStr">
+      <c r="B176" s="36" t="inlineStr">
         <is>
           <t>17:45</t>
         </is>
       </c>
-      <c r="D176" s="44" t="inlineStr">
+      <c r="C176" s="37" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="D176" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
         </is>
       </c>
-      <c r="E176" s="45" t="inlineStr">
-        <is>
-          <t>★★ MOMA PS1 — el último imprescindible del viaje, y entra gratis. Escuela pública de 1892 reconvertida en el laboratorio del MoMA: lo que no se anima a mostrar en la Quinta Avenida. VERIFICADO el 27/8: ENTRADA GRATUITA para todos, abre domingos 12:00-18:00, y «Greater New York 2026» —la encuesta insignia de la casa, que se hace cada cinco años— sigue en pie hasta el 7 de septiembre, o sea que la agarran por un día. Más el Courtyard Commission de Precious Okoyomon al aire libre. Dos horas holgadas hasta las 17:45.</t>
-        </is>
-      </c>
-      <c r="F176" s="43" t="inlineStr">
-        <is>
-          <t>MoMA PS1</t>
-        </is>
-      </c>
+      <c r="E176" s="39" t="inlineStr">
+        <is>
+          <t>Del PS1 al hotel: subte 7 desde Court Sq hasta Times Sq y 1/2/3 hasta 72 St, o E/M hasta 53 St (~45 min). Llegan 18:30, justo para las valijas. El vuelo no se toca.</t>
+        </is>
+      </c>
+      <c r="F176" s="37" t="inlineStr"/>
       <c r="G176" s="40" t="inlineStr"/>
       <c r="H176" s="41" t="inlineStr"/>
       <c r="I176" s="41" t="inlineStr"/>
@@ -37034,12 +37018,12 @@
       <c r="A177" s="35" t="n"/>
       <c r="B177" s="36" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C177" s="37" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="D177" s="38" t="inlineStr">
@@ -37049,7 +37033,7 @@
       </c>
       <c r="E177" s="39" t="inlineStr">
         <is>
-          <t>Del PS1 al hotel: subte 7 desde Court Sq hasta Times Sq y 1/2/3 hasta 72 St, o E/M hasta 53 St (~45 min). Llegan 18:30, justo para las valijas. El vuelo no se toca.</t>
+          <t>◇ SI PREFIEREN EL GUGGENHEIM, sigue estando y este bloque se ignora: pay-what-you-wish domingos 16:00-17:30 (mínimo $1) y entrada rebajada a $16 el resto del horario. ⚠️ PERO la rotonda está CERRADA del 3/8 al 17/9 por el montaje de Taryn Simon: no se camina la rampa —que es la razón para ir— y avisan que puede haber ruido de obra. Quedan las torres 4, 5 y 7 con «Guggenheim Pop» (Lichtenstein, Warhol, Oldenburg, Cattelan) y la colección Thannhauser. Para hacerlo: en vez de cruzar a Queens, teleférico de vuelta y subte 4/5/6 de 59 St a 86 St, y hay que salir del FDR Park 15:05 para entrar 16:00 — la ventana a voluntad va hasta las 17:30 y el museo cierra ahí.</t>
         </is>
       </c>
       <c r="F177" s="37" t="inlineStr"/>
@@ -37057,16 +37041,16 @@
       <c r="H177" s="41" t="inlineStr"/>
       <c r="I177" s="41" t="inlineStr"/>
     </row>
-    <row r="178" ht="30" customHeight="1">
+    <row r="178" ht="16" customHeight="1">
       <c r="A178" s="35" t="n"/>
       <c r="B178" s="36" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:30</t>
         </is>
       </c>
       <c r="C178" s="37" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="D178" s="38" t="inlineStr">
@@ -37076,7 +37060,7 @@
       </c>
       <c r="E178" s="39" t="inlineStr">
         <is>
-          <t>◇ SI PREFIEREN EL GUGGENHEIM, sigue estando y este bloque se ignora: pay-what-you-wish domingos 16:00-17:30 (mínimo $1) y entrada rebajada a $16 el resto del horario. ⚠️ PERO la rotonda está CERRADA del 3/8 al 17/9 por el montaje de Taryn Simon: no se camina la rampa —que es la razón para ir— y avisan que puede haber ruido de obra. Quedan las torres 4, 5 y 7 con «Guggenheim Pop» (Lichtenstein, Warhol, Oldenburg, Cattelan) y la colección Thannhauser. Para hacerlo: en vez de cruzar a Queens, teleférico de vuelta y subte 4/5/6 de 59 St a 86 St, y hay que salir del FDR Park 15:05 para entrar 16:00 — la ventana a voluntad va hasta las 17:30 y el museo cierra ahí.</t>
+          <t>Retirar las valijas del bell desk. Cena tranquila cerca del hotel: es la última.</t>
         </is>
       </c>
       <c r="F178" s="37" t="inlineStr"/>
@@ -37088,12 +37072,12 @@
       <c r="A179" s="35" t="n"/>
       <c r="B179" s="36" t="inlineStr">
         <is>
-          <t>18:30</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C179" s="37" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="D179" s="38" t="inlineStr">
@@ -37103,7 +37087,7 @@
       </c>
       <c r="E179" s="39" t="inlineStr">
         <is>
-          <t>Retirar las valijas del bell desk. Cena tranquila cerca del hotel: es la última.</t>
+          <t>Salir de The Beacon. Subte 1/2/3 desde 72 St hasta 34 St-Penn Station: ~10 min, $3.</t>
         </is>
       </c>
       <c r="F179" s="37" t="inlineStr"/>
@@ -37111,16 +37095,16 @@
       <c r="H179" s="41" t="inlineStr"/>
       <c r="I179" s="41" t="inlineStr"/>
     </row>
-    <row r="180" ht="16" customHeight="1">
+    <row r="180" ht="30" customHeight="1">
       <c r="A180" s="35" t="n"/>
       <c r="B180" s="36" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C180" s="37" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="D180" s="38" t="inlineStr">
@@ -37130,7 +37114,7 @@
       </c>
       <c r="E180" s="39" t="inlineStr">
         <is>
-          <t>Salir de The Beacon. Subte 1/2/3 desde 72 St hasta 34 St-Penn Station: ~10 min, $3.</t>
+          <t>NJ Transit Penn Station → EWR, llega 20:38. $17,25 (incluye el AirTrain). VERIFICAR el horario dominical en njtransit.com unos días antes.</t>
         </is>
       </c>
       <c r="F180" s="37" t="inlineStr"/>
@@ -37138,16 +37122,16 @@
       <c r="H180" s="41" t="inlineStr"/>
       <c r="I180" s="41" t="inlineStr"/>
     </row>
-    <row r="181" ht="30" customHeight="1">
+    <row r="181" ht="16" customHeight="1">
       <c r="A181" s="35" t="n"/>
       <c r="B181" s="36" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C181" s="37" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="D181" s="38" t="inlineStr">
@@ -37157,7 +37141,7 @@
       </c>
       <c r="E181" s="39" t="inlineStr">
         <is>
-          <t>NJ Transit Penn Station → EWR, llega 20:38. $17,25 (incluye el AirTrain). VERIFICAR el horario dominical en njtransit.com unos días antes.</t>
+          <t>AirTrain hasta la terminal: 10-15 min.</t>
         </is>
       </c>
       <c r="F181" s="37" t="inlineStr"/>
@@ -37165,18 +37149,14 @@
       <c r="H181" s="41" t="inlineStr"/>
       <c r="I181" s="41" t="inlineStr"/>
     </row>
-    <row r="182" ht="16" customHeight="1">
+    <row r="182" ht="30" customHeight="1">
       <c r="A182" s="35" t="n"/>
       <c r="B182" s="36" t="inlineStr">
         <is>
-          <t>20:45</t>
-        </is>
-      </c>
-      <c r="C182" s="37" t="inlineStr">
-        <is>
           <t>20:55</t>
         </is>
       </c>
+      <c r="C182" s="37" t="inlineStr"/>
       <c r="D182" s="38" t="inlineStr">
         <is>
           <t>Ambos</t>
@@ -37184,7 +37164,7 @@
       </c>
       <c r="E182" s="39" t="inlineStr">
         <is>
-          <t>AirTrain hasta la terminal: 10-15 min.</t>
+          <t>En terminal. Faltan 2h45 para el vuelo de las 23:40 — correcto para un internacional en el domingo de Labor Day, que es la noche de más tráfico del año en EWR.</t>
         </is>
       </c>
       <c r="F182" s="37" t="inlineStr"/>
@@ -37192,31 +37172,8 @@
       <c r="H182" s="41" t="inlineStr"/>
       <c r="I182" s="41" t="inlineStr"/>
     </row>
-    <row r="183" ht="30" customHeight="1">
-      <c r="A183" s="35" t="n"/>
-      <c r="B183" s="36" t="inlineStr">
-        <is>
-          <t>20:55</t>
-        </is>
-      </c>
-      <c r="C183" s="37" t="inlineStr"/>
-      <c r="D183" s="38" t="inlineStr">
-        <is>
-          <t>Ambos</t>
-        </is>
-      </c>
-      <c r="E183" s="39" t="inlineStr">
-        <is>
-          <t>En terminal. Faltan 2h45 para el vuelo de las 23:40 — correcto para un internacional en el domingo de Labor Day, que es la noche de más tráfico del año en EWR.</t>
-        </is>
-      </c>
-      <c r="F183" s="37" t="inlineStr"/>
-      <c r="G183" s="40" t="inlineStr"/>
-      <c r="H183" s="41" t="inlineStr"/>
-      <c r="I183" s="41" t="inlineStr"/>
-    </row>
-    <row r="184" ht="32" customHeight="1">
-      <c r="A184" s="46" t="inlineStr">
+    <row r="183" ht="32" customHeight="1">
+      <c r="A183" s="46" t="inlineStr">
         <is>
           <t>ALTERNATIVA / OJO:  COLCHÓN: si algo se atrasa, el tren siguiente sale 20:55 y llega a EWR 21:16, o sea terminal ~21:35 y 2h05 antes del vuelo. Es el último que yo tomaría. // Si prefieren un último día sin moverse, salteen el teleférico y estiren Central Park hasta el Guggenheim: el parque solo da para toda la mañana y la tarde. Lo que NO conviene hoy es meter algo nuevo y grande. // LO QUE SE PIERDEN POR EL VUELO, y duele: esta noche a las 20:00 el Met proyecta gratis en Lincoln Center «El Último Sueño de Frida y Diego» —la misma Frida de la muestra del MoMA del lunes— y ustedes salen del hotel 19:40 hacia Penn Station. Está a diez cuadras del Beacon. No hay forma de que entre sin poner en riesgo el vuelo. // SI QUIEREN VOLVER AL GUGGENHEIM en vez del PS1: está escrito en el bloque de las 18:20, con los tiempos hechos. Cuesta el último imprescindible del viaje y hay que aceptar que la rampa —la razón para ir— no se camina hasta el 17/9. Tercera opción si ninguna convence: el Whitney también abre los domingos.</t>
         </is>
@@ -37224,38 +37181,38 @@
     </row>
   </sheetData>
   <mergeCells count="29">
-    <mergeCell ref="A128:I128"/>
+    <mergeCell ref="A183:I183"/>
+    <mergeCell ref="A164:I164"/>
     <mergeCell ref="A84:I84"/>
     <mergeCell ref="A66:I66"/>
-    <mergeCell ref="A105:I105"/>
-    <mergeCell ref="A163:I163"/>
+    <mergeCell ref="A145:I145"/>
     <mergeCell ref="A26:I26"/>
+    <mergeCell ref="A101:I101"/>
     <mergeCell ref="A86:I86"/>
     <mergeCell ref="A104:I104"/>
     <mergeCell ref="A47:I47"/>
     <mergeCell ref="A5:I5"/>
-    <mergeCell ref="A144:I144"/>
-    <mergeCell ref="A184:I184"/>
-    <mergeCell ref="A125:I125"/>
-    <mergeCell ref="A147:I147"/>
+    <mergeCell ref="A126:I126"/>
     <mergeCell ref="A29:I29"/>
     <mergeCell ref="A165:I165"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A68:I68"/>
     <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A102:I102"/>
     <mergeCell ref="A127:I127"/>
+    <mergeCell ref="A143:I143"/>
     <mergeCell ref="A48:I48"/>
-    <mergeCell ref="A166:I166"/>
+    <mergeCell ref="A103:I103"/>
     <mergeCell ref="A45:I45"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A146:I146"/>
+    <mergeCell ref="A124:I124"/>
     <mergeCell ref="A6:I6"/>
+    <mergeCell ref="A162:I162"/>
     <mergeCell ref="A69:I69"/>
     <mergeCell ref="A87:I87"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H5:H186" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H5:H185" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Pendiente,Reservado,Confirmado,Descartado"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>